<commit_message>
Further refine camera support
</commit_message>
<xml_diff>
--- a/bom/schlieren-bom.xlsx
+++ b/bom/schlieren-bom.xlsx
@@ -11,7 +11,7 @@
     <sheet name="BOM" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'BOM'!$A$1:$L$137</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'BOM'!$A$1:$L$139</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -837,7 +837,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L137"/>
+  <dimension ref="A1:L139"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -5080,7 +5080,7 @@
         </is>
       </c>
       <c r="C82" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="D82" t="inlineStr">
         <is>
@@ -5089,7 +5089,7 @@
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>Lens pointer adjusters</t>
+          <t>Lens pointer adjusters and yoke joints</t>
         </is>
       </c>
       <c r="F82" t="inlineStr">
@@ -5122,7 +5122,7 @@
       </c>
       <c r="L82" t="inlineStr">
         <is>
-          <t>One per adjuster, set in the pointer shoe yoke bosses. One pack of 25 in hand; 21 spare.</t>
+          <t>Four set in the yoke arms (one per adjuster) and two in the yoke column feet for the joint screws (CAM-016). One pack of 25 in hand; 19 spare.</t>
         </is>
       </c>
     </row>
@@ -5220,7 +5220,7 @@
       </c>
       <c r="L84" t="inlineStr">
         <is>
-          <t>Phone-specific rail shoe with an arm carrying the rest rod. Concept mock-up only.</t>
+          <t>Phone-specific rail shoe with an arm carrying the rest rod. Retainer and safety catch not yet designed.</t>
         </is>
       </c>
     </row>
@@ -5245,12 +5245,12 @@
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>Rail shoe with the two yokes that hold the four adjusters</t>
+          <t>Rail-shoe saddle that carries the two yokes</t>
         </is>
       </c>
       <c r="J85" t="inlineStr">
         <is>
-          <t>CAD open</t>
+          <t>CAD ready</t>
         </is>
       </c>
       <c r="K85" t="inlineStr">
@@ -5260,7 +5260,7 @@
       </c>
       <c r="L85" t="inlineStr">
         <is>
-          <t>Lens-specific. Concept mock-up only.</t>
+          <t>Lens-specific. Two locating walls and a countersunk M5 hole per yoke; two M5 side-slot clamp holes.</t>
         </is>
       </c>
     </row>
@@ -5376,7 +5376,7 @@
       </c>
       <c r="L87" t="inlineStr">
         <is>
-          <t>Working-stock assortment; rod diameters and cut lengths remain open.</t>
+          <t>Working-stock assortment. Model uses two groove rods of 3 mm diameter × 10 mm and one phone rest rod of 4 mm diameter × 20 mm; confirm the assortment has these diameters.</t>
         </is>
       </c>
     </row>
@@ -5406,7 +5406,7 @@
       </c>
       <c r="J88" t="inlineStr">
         <is>
-          <t>CAD open</t>
+          <t>CAD ready</t>
         </is>
       </c>
       <c r="K88" t="inlineStr">
@@ -5416,7 +5416,7 @@
       </c>
       <c r="L88" t="inlineStr">
         <is>
-          <t>Two identical collars for the 37 mm barrel. Concept mock-up only.</t>
+          <t>Two collars for the 37 mm barrel, identical except that the aft collar's left pad pocket seats the groove rods (CAM-010) in place of a magnet.</t>
         </is>
       </c>
     </row>
@@ -5474,7 +5474,7 @@
       </c>
       <c r="L89" t="inlineStr">
         <is>
-          <t>Shared common 100-pack. Provisional: one screw per collar.</t>
+          <t>Shared common 100-pack. One screw per collar.</t>
         </is>
       </c>
     </row>
@@ -5532,7 +5532,7 @@
       </c>
       <c r="L90" t="inlineStr">
         <is>
-          <t>Shared common 100-pack (see CAS-004). Provisional: one nut per collar.</t>
+          <t>Shared common 100-pack (see CAS-004). One nut per collar.</t>
         </is>
       </c>
     </row>
@@ -5597,60 +5597,52 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>MIR-001</t>
+          <t>CAM-015</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>Mirror cell</t>
+          <t>Imager</t>
         </is>
       </c>
       <c r="C92" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>Skyoptikst D203F1600 spherical mirror, Ø203 mm, f=1600 mm</t>
-        </is>
-      </c>
-      <c r="F92" t="inlineStr">
-        <is>
-          <t>Amazon</t>
-        </is>
-      </c>
-      <c r="G92" t="inlineStr">
-        <is>
-          <t>B0B5RR41CT</t>
-        </is>
-      </c>
-      <c r="H92" t="n">
-        <v>1</v>
-      </c>
-      <c r="I92" t="inlineStr">
-        <is>
-          <t>each</t>
+          <t>ABS printed lens pointer yokes</t>
+        </is>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>Carry the adjuster inserts and the retaining-band pegs</t>
         </is>
       </c>
       <c r="J92" t="inlineStr">
         <is>
-          <t>In hand</t>
+          <t>CAD ready</t>
         </is>
       </c>
       <c r="K92" t="inlineStr">
         <is>
-          <t>§10.5</t>
+          <t>§9.5</t>
+        </is>
+      </c>
+      <c r="L92" t="inlineStr">
+        <is>
+          <t>Printed on their side; each bolted to the pointer shoe with one countersunk M5 screw (CAM-016) into a heat-set insert (CAM-005).</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>MIR-002</t>
+          <t>CAM-016</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>Mirror cell</t>
+          <t>Imager</t>
         </is>
       </c>
       <c r="C93" t="n">
@@ -5658,26 +5650,26 @@
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>Baltic birch plywood panel 12 × 12 × 1/2 in</t>
+          <t>M5 × 0.8 × 10 mm 18-8 stainless hex-drive flat head screw, 90°</t>
         </is>
       </c>
       <c r="E93" t="inlineStr">
         <is>
-          <t>Base and adjuster plates</t>
+          <t>Yoke-to-shoe joint screws</t>
         </is>
       </c>
       <c r="F93" t="inlineStr">
         <is>
-          <t>Amazon</t>
+          <t>McMaster</t>
         </is>
       </c>
       <c r="G93" t="inlineStr">
         <is>
-          <t>B09D941GXR</t>
+          <t>92125A208</t>
         </is>
       </c>
       <c r="H93" t="n">
-        <v>4</v>
+        <v>100</v>
       </c>
       <c r="I93" t="inlineStr">
         <is>
@@ -5686,19 +5678,24 @@
       </c>
       <c r="J93" t="inlineStr">
         <is>
-          <t>In hand</t>
+          <t>To procure</t>
         </is>
       </c>
       <c r="K93" t="inlineStr">
         <is>
-          <t>§10.1</t>
+          <t>§§9.5, 9.7</t>
+        </is>
+      </c>
+      <c r="L93" t="inlineStr">
+        <is>
+          <t>10 mm head, 3 mm hex drive. Each screws up through the pointer shoe deck into a heat-set insert in the yoke foot.</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>MIR-003</t>
+          <t>MIR-001</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
@@ -5711,12 +5708,7 @@
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>Baltic birch plywood panel 12 × 12 × 3/4 in</t>
-        </is>
-      </c>
-      <c r="E94" t="inlineStr">
-        <is>
-          <t>Mirror plate</t>
+          <t>Skyoptikst D203F1600 spherical mirror, Ø203 mm, f=1600 mm</t>
         </is>
       </c>
       <c r="F94" t="inlineStr">
@@ -5726,7 +5718,7 @@
       </c>
       <c r="G94" t="inlineStr">
         <is>
-          <t>B0GL9G45GH</t>
+          <t>B0B5RR41CT</t>
         </is>
       </c>
       <c r="H94" t="n">
@@ -5744,14 +5736,14 @@
       </c>
       <c r="K94" t="inlineStr">
         <is>
-          <t>§10.1</t>
+          <t>§10.5</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>MIR-004</t>
+          <t>MIR-002</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
@@ -5760,29 +5752,34 @@
         </is>
       </c>
       <c r="C95" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>1/4-80 TPI Imperial fine adjustment screws, 2.5 in</t>
+          <t>Baltic birch plywood panel 12 × 12 × 1/2 in</t>
+        </is>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>Base and adjuster plates</t>
         </is>
       </c>
       <c r="F95" t="inlineStr">
         <is>
-          <t>Kozak</t>
+          <t>Amazon</t>
         </is>
       </c>
       <c r="G95" t="inlineStr">
         <is>
-          <t>TS250-80-2500</t>
+          <t>B09D941GXR</t>
         </is>
       </c>
       <c r="H95" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I95" t="inlineStr">
         <is>
-          <t>each</t>
+          <t>pack</t>
         </is>
       </c>
       <c r="J95" t="inlineStr">
@@ -5792,14 +5789,14 @@
       </c>
       <c r="K95" t="inlineStr">
         <is>
-          <t>§10.2</t>
+          <t>§10.1</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>MIR-005</t>
+          <t>MIR-003</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
@@ -5808,25 +5805,30 @@
         </is>
       </c>
       <c r="C96" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>Imperial Fine Adjustment Carrier Bushings</t>
+          <t>Baltic birch plywood panel 12 × 12 × 3/4 in</t>
+        </is>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>Mirror plate</t>
         </is>
       </c>
       <c r="F96" t="inlineStr">
         <is>
-          <t>Kozak</t>
+          <t>Amazon</t>
         </is>
       </c>
       <c r="G96" t="inlineStr">
         <is>
-          <t>TB250-80-625</t>
+          <t>B0GL9G45GH</t>
         </is>
       </c>
       <c r="H96" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="I96" t="inlineStr">
         <is>
@@ -5840,14 +5842,14 @@
       </c>
       <c r="K96" t="inlineStr">
         <is>
-          <t>§10.2</t>
+          <t>§10.1</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>MIR-006</t>
+          <t>MIR-004</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
@@ -5860,7 +5862,7 @@
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>Imperial Adjustment Knobs</t>
+          <t>1/4-80 TPI Imperial fine adjustment screws, 2.5 in</t>
         </is>
       </c>
       <c r="F97" t="inlineStr">
@@ -5870,7 +5872,7 @@
       </c>
       <c r="G97" t="inlineStr">
         <is>
-          <t>KB250-80</t>
+          <t>TS250-80-2500</t>
         </is>
       </c>
       <c r="H97" t="n">
@@ -5895,7 +5897,7 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>MIR-007</t>
+          <t>MIR-005</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
@@ -5908,22 +5910,17 @@
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>Leveling Washer, Two Piece, 1/4" Screw Size, Black-Oxide Steel</t>
-        </is>
-      </c>
-      <c r="E98" t="inlineStr">
-        <is>
-          <t>Spherical washers</t>
+          <t>Imperial Fine Adjustment Carrier Bushings</t>
         </is>
       </c>
       <c r="F98" t="inlineStr">
         <is>
-          <t>McMaster</t>
+          <t>Kozak</t>
         </is>
       </c>
       <c r="G98" t="inlineStr">
         <is>
-          <t>91131A028</t>
+          <t>TB250-80-625</t>
         </is>
       </c>
       <c r="H98" t="n">
@@ -5941,14 +5938,14 @@
       </c>
       <c r="K98" t="inlineStr">
         <is>
-          <t>§10.4</t>
+          <t>§10.2</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>MIR-008</t>
+          <t>MIR-006</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
@@ -5961,25 +5958,25 @@
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>Compression Springs, 0.75" Long, 0.5" OD, 0.424" ID</t>
+          <t>Imperial Adjustment Knobs</t>
         </is>
       </c>
       <c r="F99" t="inlineStr">
         <is>
-          <t>McMaster</t>
+          <t>Kozak</t>
         </is>
       </c>
       <c r="G99" t="inlineStr">
         <is>
-          <t>2022N186</t>
+          <t>KB250-80</t>
         </is>
       </c>
       <c r="H99" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="I99" t="inlineStr">
         <is>
-          <t>pack</t>
+          <t>each</t>
         </is>
       </c>
       <c r="J99" t="inlineStr">
@@ -5989,14 +5986,14 @@
       </c>
       <c r="K99" t="inlineStr">
         <is>
-          <t>§10.3</t>
+          <t>§10.2</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>MIR-009</t>
+          <t>MIR-007</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
@@ -6005,16 +6002,16 @@
         </is>
       </c>
       <c r="C100" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>Washer for 3/8" washer, 0.390" ID, 0.028" to 0.036" thick, 18-8 SS</t>
+          <t>Leveling Washer, Two Piece, 1/4" Screw Size, Black-Oxide Steel</t>
         </is>
       </c>
       <c r="E100" t="inlineStr">
         <is>
-          <t>Spring seat washers</t>
+          <t>Spherical washers</t>
         </is>
       </c>
       <c r="F100" t="inlineStr">
@@ -6024,15 +6021,15 @@
       </c>
       <c r="G100" t="inlineStr">
         <is>
-          <t>98017A199</t>
+          <t>91131A028</t>
         </is>
       </c>
       <c r="H100" t="n">
-        <v>100</v>
+        <v>3</v>
       </c>
       <c r="I100" t="inlineStr">
         <is>
-          <t>pack</t>
+          <t>each</t>
         </is>
       </c>
       <c r="J100" t="inlineStr">
@@ -6042,14 +6039,14 @@
       </c>
       <c r="K100" t="inlineStr">
         <is>
-          <t>§10.3</t>
+          <t>§10.4</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>MIR-010</t>
+          <t>MIR-008</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
@@ -6058,16 +6055,11 @@
         </is>
       </c>
       <c r="C101" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>3" Long Corner Bracket, aluminum</t>
-        </is>
-      </c>
-      <c r="E101" t="inlineStr">
-        <is>
-          <t>Adjuster plate to base plate mounting</t>
+          <t>Compression Springs, 0.75" Long, 0.5" OD, 0.424" ID</t>
         </is>
       </c>
       <c r="F101" t="inlineStr">
@@ -6077,15 +6069,15 @@
       </c>
       <c r="G101" t="inlineStr">
         <is>
-          <t>8681N11</t>
+          <t>2022N186</t>
         </is>
       </c>
       <c r="H101" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="I101" t="inlineStr">
         <is>
-          <t>each</t>
+          <t>pack</t>
         </is>
       </c>
       <c r="J101" t="inlineStr">
@@ -6095,14 +6087,14 @@
       </c>
       <c r="K101" t="inlineStr">
         <is>
-          <t>§10.7</t>
+          <t>§10.3</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>MIR-011</t>
+          <t>MIR-009</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
@@ -6110,14 +6102,17 @@
           <t>Mirror cell</t>
         </is>
       </c>
+      <c r="C102" t="n">
+        <v>6</v>
+      </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t>5/16" × 1-1/2" hex-drive flat-head screw, 316 SS</t>
+          <t>Washer for 3/8" washer, 0.390" ID, 0.028" to 0.036" thick, 18-8 SS</t>
         </is>
       </c>
       <c r="E102" t="inlineStr">
         <is>
-          <t>Existing alternate/fallback bracket screw stock</t>
+          <t>Spring seat washers</t>
         </is>
       </c>
       <c r="F102" t="inlineStr">
@@ -6127,11 +6122,11 @@
       </c>
       <c r="G102" t="inlineStr">
         <is>
-          <t>90585A587</t>
+          <t>98017A199</t>
         </is>
       </c>
       <c r="H102" t="n">
-        <v>5</v>
+        <v>100</v>
       </c>
       <c r="I102" t="inlineStr">
         <is>
@@ -6145,19 +6140,14 @@
       </c>
       <c r="K102" t="inlineStr">
         <is>
-          <t>§10.7</t>
-        </is>
-      </c>
-      <c r="L102" t="inlineStr">
-        <is>
-          <t>Previously baseline bracket screw; retained as in-hand alternate stock after corner-clearance review.</t>
+          <t>§10.3</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>MIR-012</t>
+          <t>MIR-010</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
@@ -6166,11 +6156,11 @@
         </is>
       </c>
       <c r="C103" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>5/16"-18 heavy-profile nylon-insert locknut, 18-8 SS</t>
+          <t>3" Long Corner Bracket, aluminum</t>
         </is>
       </c>
       <c r="E103" t="inlineStr">
@@ -6185,15 +6175,15 @@
       </c>
       <c r="G103" t="inlineStr">
         <is>
-          <t>90099A030</t>
+          <t>8681N11</t>
         </is>
       </c>
       <c r="H103" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="I103" t="inlineStr">
         <is>
-          <t>pack</t>
+          <t>each</t>
         </is>
       </c>
       <c r="J103" t="inlineStr">
@@ -6204,18 +6194,13 @@
       <c r="K103" t="inlineStr">
         <is>
           <t>§10.7</t>
-        </is>
-      </c>
-      <c r="L103" t="inlineStr">
-        <is>
-          <t>Six installed for the revised three-fastener-per-bracket pattern; existing stock confirmed in hand.</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>MIR-013</t>
+          <t>MIR-011</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
@@ -6223,17 +6208,14 @@
           <t>Mirror cell</t>
         </is>
       </c>
-      <c r="C104" t="n">
-        <v>6</v>
-      </c>
       <c r="D104" t="inlineStr">
         <is>
-          <t>5/16" SAE washer, 0.344" ID × 0.688" OD, 18-8 SS black oxide</t>
+          <t>5/16" × 1-1/2" hex-drive flat-head screw, 316 SS</t>
         </is>
       </c>
       <c r="E104" t="inlineStr">
         <is>
-          <t>Adjuster plate to base plate mounting</t>
+          <t>Existing alternate/fallback bracket screw stock</t>
         </is>
       </c>
       <c r="F104" t="inlineStr">
@@ -6243,11 +6225,11 @@
       </c>
       <c r="G104" t="inlineStr">
         <is>
-          <t>96659A134</t>
+          <t>90585A587</t>
         </is>
       </c>
       <c r="H104" t="n">
-        <v>25</v>
+        <v>5</v>
       </c>
       <c r="I104" t="inlineStr">
         <is>
@@ -6266,14 +6248,14 @@
       </c>
       <c r="L104" t="inlineStr">
         <is>
-          <t>Six installed for the revised three-fastener-per-bracket pattern.</t>
+          <t>Previously baseline bracket screw; retained as in-hand alternate stock after corner-clearance review.</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>MIR-015</t>
+          <t>MIR-012</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
@@ -6282,16 +6264,16 @@
         </is>
       </c>
       <c r="C105" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>1/4"-20 × 1-1/2" flat-head screws</t>
+          <t>5/16"-18 heavy-profile nylon-insert locknut, 18-8 SS</t>
         </is>
       </c>
       <c r="E105" t="inlineStr">
         <is>
-          <t>Existing spare stock; former C2564 tripod-interface hardware</t>
+          <t>Adjuster plate to base plate mounting</t>
         </is>
       </c>
       <c r="F105" t="inlineStr">
@@ -6301,15 +6283,15 @@
       </c>
       <c r="G105" t="inlineStr">
         <is>
-          <t>94518A525</t>
+          <t>90099A030</t>
         </is>
       </c>
       <c r="H105" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="I105" t="inlineStr">
         <is>
-          <t>each</t>
+          <t>pack</t>
         </is>
       </c>
       <c r="J105" t="inlineStr">
@@ -6317,16 +6299,21 @@
           <t>In hand</t>
         </is>
       </c>
+      <c r="K105" t="inlineStr">
+        <is>
+          <t>§10.7</t>
+        </is>
+      </c>
       <c r="L105" t="inlineStr">
         <is>
-          <t>No longer allocated to the active tripod interface after transition to the CAMVATE 577/501/504 quick-release system; retain as in-hand spare hardware.</t>
+          <t>Six installed for the revised three-fastener-per-bracket pattern; existing stock confirmed in hand.</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>MIR-017</t>
+          <t>MIR-013</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
@@ -6335,16 +6322,16 @@
         </is>
       </c>
       <c r="C106" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>1/4"-20 flex-top locknuts</t>
+          <t>5/16" SAE washer, 0.344" ID × 0.688" OD, 18-8 SS black oxide</t>
         </is>
       </c>
       <c r="E106" t="inlineStr">
         <is>
-          <t>Existing spare stock; former C2564 tripod-interface hardware</t>
+          <t>Adjuster plate to base plate mounting</t>
         </is>
       </c>
       <c r="F106" t="inlineStr">
@@ -6354,11 +6341,11 @@
       </c>
       <c r="G106" t="inlineStr">
         <is>
-          <t>91839A123</t>
+          <t>96659A134</t>
         </is>
       </c>
       <c r="H106" t="n">
-        <v>5</v>
+        <v>25</v>
       </c>
       <c r="I106" t="inlineStr">
         <is>
@@ -6370,16 +6357,21 @@
           <t>In hand</t>
         </is>
       </c>
+      <c r="K106" t="inlineStr">
+        <is>
+          <t>§10.7</t>
+        </is>
+      </c>
       <c r="L106" t="inlineStr">
         <is>
-          <t>No longer allocated to the active tripod interface after transition to the CAMVATE 577/501/504 quick-release system; retain as in-hand spare hardware.</t>
+          <t>Six installed for the revised three-fastener-per-bracket pattern.</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>MIR-018</t>
+          <t>MIR-015</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
@@ -6392,7 +6384,7 @@
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t>1/4" thin washers</t>
+          <t>1/4"-20 × 1-1/2" flat-head screws</t>
         </is>
       </c>
       <c r="E107" t="inlineStr">
@@ -6407,15 +6399,15 @@
       </c>
       <c r="G107" t="inlineStr">
         <is>
-          <t>98019A255</t>
+          <t>94518A525</t>
         </is>
       </c>
       <c r="H107" t="n">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="I107" t="inlineStr">
         <is>
-          <t>pack</t>
+          <t>each</t>
         </is>
       </c>
       <c r="J107" t="inlineStr">
@@ -6432,7 +6424,7 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>MIR-023</t>
+          <t>MIR-017</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
@@ -6445,12 +6437,12 @@
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>M4 × 0.7 × 16 mm 90° flat-head hex-drive screw, 18-8 stainless</t>
+          <t>1/4"-20 flex-top locknuts</t>
         </is>
       </c>
       <c r="E108" t="inlineStr">
         <is>
-          <t>Provisional quick-release plate mounting screw; short-length option</t>
+          <t>Existing spare stock; former C2564 tripod-interface hardware</t>
         </is>
       </c>
       <c r="F108" t="inlineStr">
@@ -6460,11 +6452,11 @@
       </c>
       <c r="G108" t="inlineStr">
         <is>
-          <t>92125A194</t>
+          <t>91839A123</t>
         </is>
       </c>
       <c r="H108" t="n">
-        <v>100</v>
+        <v>5</v>
       </c>
       <c r="I108" t="inlineStr">
         <is>
@@ -6476,21 +6468,16 @@
           <t>In hand</t>
         </is>
       </c>
-      <c r="K108" t="inlineStr">
-        <is>
-          <t>§10.9</t>
-        </is>
-      </c>
       <c r="L108" t="inlineStr">
         <is>
-          <t>Order one pack. Four screws are the provisional installed quantity if this length matches the measured CAMVATE plate thickness; otherwise use MIR-024.</t>
+          <t>No longer allocated to the active tripod interface after transition to the CAMVATE 577/501/504 quick-release system; retain as in-hand spare hardware.</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>MIR-024</t>
+          <t>MIR-018</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
@@ -6503,12 +6490,12 @@
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t>M4 × 0.7 × 18 mm 90° flat-head hex-drive screw, 18-8 stainless</t>
+          <t>1/4" thin washers</t>
         </is>
       </c>
       <c r="E109" t="inlineStr">
         <is>
-          <t>Provisional quick-release plate mounting screw; long-length option</t>
+          <t>Existing spare stock; former C2564 tripod-interface hardware</t>
         </is>
       </c>
       <c r="F109" t="inlineStr">
@@ -6518,11 +6505,11 @@
       </c>
       <c r="G109" t="inlineStr">
         <is>
-          <t>92125A196</t>
+          <t>98019A255</t>
         </is>
       </c>
       <c r="H109" t="n">
-        <v>100</v>
+        <v>10</v>
       </c>
       <c r="I109" t="inlineStr">
         <is>
@@ -6534,21 +6521,16 @@
           <t>In hand</t>
         </is>
       </c>
-      <c r="K109" t="inlineStr">
-        <is>
-          <t>§10.9</t>
-        </is>
-      </c>
       <c r="L109" t="inlineStr">
         <is>
-          <t>Order one pack. Four screws are the provisional installed quantity if this length matches the measured CAMVATE plate thickness; otherwise use MIR-023.</t>
+          <t>No longer allocated to the active tripod interface after transition to the CAMVATE 577/501/504 quick-release system; retain as in-hand spare hardware.</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>MIR-025</t>
+          <t>MIR-023</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
@@ -6557,34 +6539,34 @@
         </is>
       </c>
       <c r="C110" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D110" t="inlineStr">
         <is>
-          <t>CAMVATE Manfrotto-Type Quick Release Assembly with Sliding Plate Camera Mount</t>
+          <t>M4 × 0.7 × 16 mm 90° flat-head hex-drive screw, 18-8 stainless</t>
         </is>
       </c>
       <c r="E110" t="inlineStr">
         <is>
-          <t>Mirror-cell quick-release / tripod interface</t>
+          <t>Provisional quick-release plate mounting screw; short-length option</t>
         </is>
       </c>
       <c r="F110" t="inlineStr">
         <is>
-          <t>Amazon</t>
+          <t>McMaster</t>
         </is>
       </c>
       <c r="G110" t="inlineStr">
         <is>
-          <t>B0B2WBC921</t>
+          <t>92125A194</t>
         </is>
       </c>
       <c r="H110" t="n">
-        <v>1</v>
+        <v>100</v>
       </c>
       <c r="I110" t="inlineStr">
         <is>
-          <t>each</t>
+          <t>pack</t>
         </is>
       </c>
       <c r="J110" t="inlineStr">
@@ -6599,14 +6581,14 @@
       </c>
       <c r="L110" t="inlineStr">
         <is>
-          <t>Complete 577/501/504-compatible quick-release assembly with removable sliding plate and receiver. Exact removable-plate hole pattern and final M4 screw length to be verified on arrival.</t>
+          <t>Order one pack. Four screws are the provisional installed quantity if this length matches the measured CAMVATE plate thickness; otherwise use MIR-024.</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>MIR-019</t>
+          <t>MIR-024</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
@@ -6615,16 +6597,16 @@
         </is>
       </c>
       <c r="C111" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>DOWSIL 737 clear silicone, 3 fl. oz.</t>
+          <t>M4 × 0.7 × 18 mm 90° flat-head hex-drive screw, 18-8 stainless</t>
         </is>
       </c>
       <c r="E111" t="inlineStr">
         <is>
-          <t>Mirror mounting</t>
+          <t>Provisional quick-release plate mounting screw; long-length option</t>
         </is>
       </c>
       <c r="F111" t="inlineStr">
@@ -6634,15 +6616,15 @@
       </c>
       <c r="G111" t="inlineStr">
         <is>
-          <t>7587A25</t>
+          <t>92125A196</t>
         </is>
       </c>
       <c r="H111" t="n">
-        <v>1</v>
+        <v>100</v>
       </c>
       <c r="I111" t="inlineStr">
         <is>
-          <t>each</t>
+          <t>pack</t>
         </is>
       </c>
       <c r="J111" t="inlineStr">
@@ -6652,14 +6634,19 @@
       </c>
       <c r="K111" t="inlineStr">
         <is>
-          <t>§10.5</t>
+          <t>§10.9</t>
+        </is>
+      </c>
+      <c r="L111" t="inlineStr">
+        <is>
+          <t>Order one pack. Four screws are the provisional installed quantity if this length matches the measured CAMVATE plate thickness; otherwise use MIR-023.</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>MIR-020</t>
+          <t>MIR-025</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
@@ -6672,22 +6659,22 @@
       </c>
       <c r="D112" t="inlineStr">
         <is>
-          <t>Adhesive backed F1 felt</t>
+          <t>CAMVATE Manfrotto-Type Quick Release Assembly with Sliding Plate Camera Mount</t>
         </is>
       </c>
       <c r="E112" t="inlineStr">
         <is>
-          <t>Safety retainer padding</t>
+          <t>Mirror-cell quick-release / tripod interface</t>
         </is>
       </c>
       <c r="F112" t="inlineStr">
         <is>
-          <t>McMaster</t>
+          <t>Amazon</t>
         </is>
       </c>
       <c r="G112" t="inlineStr">
         <is>
-          <t>8334K15</t>
+          <t>B0B2WBC921</t>
         </is>
       </c>
       <c r="H112" t="n">
@@ -6695,7 +6682,7 @@
       </c>
       <c r="I112" t="inlineStr">
         <is>
-          <t>sheet</t>
+          <t>each</t>
         </is>
       </c>
       <c r="J112" t="inlineStr">
@@ -6705,14 +6692,19 @@
       </c>
       <c r="K112" t="inlineStr">
         <is>
-          <t>§10.8</t>
+          <t>§10.9</t>
+        </is>
+      </c>
+      <c r="L112" t="inlineStr">
+        <is>
+          <t>Complete 577/501/504-compatible quick-release assembly with removable sliding plate and receiver. Exact removable-plate hole pattern and final M4 screw length to be verified on arrival.</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>MIR-021</t>
+          <t>MIR-019</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
@@ -6721,28 +6713,51 @@
         </is>
       </c>
       <c r="C113" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D113" t="inlineStr">
         <is>
-          <t>ABS printed front safety retainers</t>
+          <t>DOWSIL 737 clear silicone, 3 fl. oz.</t>
+        </is>
+      </c>
+      <c r="E113" t="inlineStr">
+        <is>
+          <t>Mirror mounting</t>
+        </is>
+      </c>
+      <c r="F113" t="inlineStr">
+        <is>
+          <t>McMaster</t>
+        </is>
+      </c>
+      <c r="G113" t="inlineStr">
+        <is>
+          <t>7587A25</t>
+        </is>
+      </c>
+      <c r="H113" t="n">
+        <v>1</v>
+      </c>
+      <c r="I113" t="inlineStr">
+        <is>
+          <t>each</t>
         </is>
       </c>
       <c r="J113" t="inlineStr">
         <is>
-          <t>CAD open</t>
+          <t>In hand</t>
         </is>
       </c>
       <c r="K113" t="inlineStr">
         <is>
-          <t>§10.8</t>
+          <t>§10.5</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>MIR-022</t>
+          <t>MIR-020</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
@@ -6751,16 +6766,16 @@
         </is>
       </c>
       <c r="C114" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="D114" t="inlineStr">
         <is>
-          <t>5/16"-18 × 1-3/8" hex-drive flat-head screw, 316 SS</t>
+          <t>Adhesive backed F1 felt</t>
         </is>
       </c>
       <c r="E114" t="inlineStr">
         <is>
-          <t>Primary structural-bracket screws</t>
+          <t>Safety retainer padding</t>
         </is>
       </c>
       <c r="F114" t="inlineStr">
@@ -6770,15 +6785,15 @@
       </c>
       <c r="G114" t="inlineStr">
         <is>
-          <t>90585A997</t>
+          <t>8334K15</t>
         </is>
       </c>
       <c r="H114" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="I114" t="inlineStr">
         <is>
-          <t>pack</t>
+          <t>sheet</t>
         </is>
       </c>
       <c r="J114" t="inlineStr">
@@ -6788,80 +6803,62 @@
       </c>
       <c r="K114" t="inlineStr">
         <is>
-          <t>§10.7</t>
-        </is>
-      </c>
-      <c r="L114" t="inlineStr">
-        <is>
-          <t>Use six installed: two through the vertical plate and one through the base plate per bracket. Two 5-packs required; four spare.</t>
+          <t>§10.8</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>SHP-001</t>
+          <t>MIR-021</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>Shop supplies</t>
+          <t>Mirror cell</t>
         </is>
       </c>
       <c r="C115" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t>Loctite 271 threadlocker, .34 fl. oz.</t>
-        </is>
-      </c>
-      <c r="F115" t="inlineStr">
-        <is>
-          <t>McMaster</t>
-        </is>
-      </c>
-      <c r="G115" t="inlineStr">
-        <is>
-          <t>91458A160</t>
-        </is>
-      </c>
-      <c r="H115" t="n">
-        <v>1</v>
-      </c>
-      <c r="I115" t="inlineStr">
-        <is>
-          <t>each</t>
+          <t>ABS printed front safety retainers</t>
         </is>
       </c>
       <c r="J115" t="inlineStr">
         <is>
-          <t>In hand</t>
+          <t>CAD open</t>
         </is>
       </c>
       <c r="K115" t="inlineStr">
         <is>
-          <t>§9.5</t>
+          <t>§10.8</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>SHP-002</t>
+          <t>MIR-022</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>Shop supplies</t>
+          <t>Mirror cell</t>
         </is>
       </c>
       <c r="C116" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="D116" t="inlineStr">
         <is>
-          <t>Heat-set installation tip</t>
+          <t>5/16"-18 × 1-3/8" hex-drive flat-head screw, 316 SS</t>
+        </is>
+      </c>
+      <c r="E116" t="inlineStr">
+        <is>
+          <t>Primary structural-bracket screws</t>
         </is>
       </c>
       <c r="F116" t="inlineStr">
@@ -6871,15 +6868,15 @@
       </c>
       <c r="G116" t="inlineStr">
         <is>
-          <t>92160A327</t>
+          <t>90585A997</t>
         </is>
       </c>
       <c r="H116" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="I116" t="inlineStr">
         <is>
-          <t>each</t>
+          <t>pack</t>
         </is>
       </c>
       <c r="J116" t="inlineStr">
@@ -6889,14 +6886,19 @@
       </c>
       <c r="K116" t="inlineStr">
         <is>
-          <t>§9.5</t>
+          <t>§10.7</t>
+        </is>
+      </c>
+      <c r="L116" t="inlineStr">
+        <is>
+          <t>Use six installed: two through the vertical plate and one through the base plate per bracket. Two 5-packs required; four spare.</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>SHP-003</t>
+          <t>SHP-001</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
@@ -6909,17 +6911,17 @@
       </c>
       <c r="D117" t="inlineStr">
         <is>
-          <t>Optical spanner wrench</t>
+          <t>Loctite 271 threadlocker, .34 fl. oz.</t>
         </is>
       </c>
       <c r="F117" t="inlineStr">
         <is>
-          <t>Amazon</t>
+          <t>McMaster</t>
         </is>
       </c>
       <c r="G117" t="inlineStr">
         <is>
-          <t>B0CKSL364Q</t>
+          <t>91458A160</t>
         </is>
       </c>
       <c r="H117" t="n">
@@ -6933,13 +6935,18 @@
       <c r="J117" t="inlineStr">
         <is>
           <t>In hand</t>
+        </is>
+      </c>
+      <c r="K117" t="inlineStr">
+        <is>
+          <t>§9.5</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>SHP-004</t>
+          <t>SHP-002</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
@@ -6952,22 +6959,17 @@
       </c>
       <c r="D118" t="inlineStr">
         <is>
-          <t>Metric feeler gauge set</t>
-        </is>
-      </c>
-      <c r="E118" t="inlineStr">
-        <is>
-          <t>Source-slit blade spacing</t>
+          <t>Heat-set installation tip</t>
         </is>
       </c>
       <c r="F118" t="inlineStr">
         <is>
-          <t>Amazon</t>
+          <t>McMaster</t>
         </is>
       </c>
       <c r="G118" t="inlineStr">
         <is>
-          <t>B07XPD9L1C</t>
+          <t>92160A327</t>
         </is>
       </c>
       <c r="H118" t="n">
@@ -6985,14 +6987,14 @@
       </c>
       <c r="K118" t="inlineStr">
         <is>
-          <t>§7.4</t>
+          <t>§9.5</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>SHP-005</t>
+          <t>SHP-003</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
@@ -7005,22 +7007,17 @@
       </c>
       <c r="D119" t="inlineStr">
         <is>
-          <t>M2 tap</t>
-        </is>
-      </c>
-      <c r="E119" t="inlineStr">
-        <is>
-          <t>LED board mounting into SM1CP2M cap</t>
+          <t>Optical spanner wrench</t>
         </is>
       </c>
       <c r="F119" t="inlineStr">
         <is>
-          <t>McMaster</t>
+          <t>Amazon</t>
         </is>
       </c>
       <c r="G119" t="inlineStr">
         <is>
-          <t>8305A78</t>
+          <t>B0CKSL364Q</t>
         </is>
       </c>
       <c r="H119" t="n">
@@ -7034,18 +7031,13 @@
       <c r="J119" t="inlineStr">
         <is>
           <t>In hand</t>
-        </is>
-      </c>
-      <c r="K119" t="inlineStr">
-        <is>
-          <t>§6.4</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>SHP-006</t>
+          <t>SHP-004</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
@@ -7058,22 +7050,22 @@
       </c>
       <c r="D120" t="inlineStr">
         <is>
-          <t>M2 tap drill, 1.6mm</t>
+          <t>Metric feeler gauge set</t>
         </is>
       </c>
       <c r="E120" t="inlineStr">
         <is>
-          <t>LED mounting</t>
+          <t>Source-slit blade spacing</t>
         </is>
       </c>
       <c r="F120" t="inlineStr">
         <is>
-          <t>McMaster</t>
+          <t>Amazon</t>
         </is>
       </c>
       <c r="G120" t="inlineStr">
         <is>
-          <t>2979N13</t>
+          <t>B07XPD9L1C</t>
         </is>
       </c>
       <c r="H120" t="n">
@@ -7091,14 +7083,14 @@
       </c>
       <c r="K120" t="inlineStr">
         <is>
-          <t>§6.4</t>
+          <t>§7.4</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>SHP-007</t>
+          <t>SHP-005</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
@@ -7106,14 +7098,35 @@
           <t>Shop supplies</t>
         </is>
       </c>
+      <c r="C121" t="n">
+        <v>1</v>
+      </c>
       <c r="D121" t="inlineStr">
         <is>
-          <t>18 AWG wire</t>
+          <t>M2 tap</t>
         </is>
       </c>
       <c r="E121" t="inlineStr">
         <is>
-          <t>LED wiring</t>
+          <t>LED board mounting into SM1CP2M cap</t>
+        </is>
+      </c>
+      <c r="F121" t="inlineStr">
+        <is>
+          <t>McMaster</t>
+        </is>
+      </c>
+      <c r="G121" t="inlineStr">
+        <is>
+          <t>8305A78</t>
+        </is>
+      </c>
+      <c r="H121" t="n">
+        <v>1</v>
+      </c>
+      <c r="I121" t="inlineStr">
+        <is>
+          <t>each</t>
         </is>
       </c>
       <c r="J121" t="inlineStr">
@@ -7123,14 +7136,14 @@
       </c>
       <c r="K121" t="inlineStr">
         <is>
-          <t>§6.5</t>
+          <t>§6.4</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>SHP-008</t>
+          <t>SHP-006</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
@@ -7138,26 +7151,52 @@
           <t>Shop supplies</t>
         </is>
       </c>
+      <c r="C122" t="n">
+        <v>1</v>
+      </c>
       <c r="D122" t="inlineStr">
         <is>
-          <t>Heat-shrink tubing</t>
+          <t>M2 tap drill, 1.6mm</t>
         </is>
       </c>
       <c r="E122" t="inlineStr">
         <is>
-          <t>LED wiring</t>
+          <t>LED mounting</t>
+        </is>
+      </c>
+      <c r="F122" t="inlineStr">
+        <is>
+          <t>McMaster</t>
+        </is>
+      </c>
+      <c r="G122" t="inlineStr">
+        <is>
+          <t>2979N13</t>
+        </is>
+      </c>
+      <c r="H122" t="n">
+        <v>1</v>
+      </c>
+      <c r="I122" t="inlineStr">
+        <is>
+          <t>each</t>
         </is>
       </c>
       <c r="J122" t="inlineStr">
         <is>
           <t>In hand</t>
+        </is>
+      </c>
+      <c r="K122" t="inlineStr">
+        <is>
+          <t>§6.4</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>SHP-009</t>
+          <t>SHP-007</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
@@ -7167,24 +7206,29 @@
       </c>
       <c r="D123" t="inlineStr">
         <is>
-          <t>USB-C chargers/cables</t>
+          <t>18 AWG wire</t>
         </is>
       </c>
       <c r="E123" t="inlineStr">
         <is>
-          <t>DP100 power</t>
+          <t>LED wiring</t>
         </is>
       </c>
       <c r="J123" t="inlineStr">
         <is>
           <t>In hand</t>
+        </is>
+      </c>
+      <c r="K123" t="inlineStr">
+        <is>
+          <t>§6.5</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>SHP-010</t>
+          <t>SHP-008</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
@@ -7194,29 +7238,24 @@
       </c>
       <c r="D124" t="inlineStr">
         <is>
-          <t>Thermal compound</t>
+          <t>Heat-shrink tubing</t>
         </is>
       </c>
       <c r="E124" t="inlineStr">
         <is>
-          <t>LED heatsink interfaces</t>
+          <t>LED wiring</t>
         </is>
       </c>
       <c r="J124" t="inlineStr">
         <is>
           <t>In hand</t>
-        </is>
-      </c>
-      <c r="K124" t="inlineStr">
-        <is>
-          <t>§6.4</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>SHP-011</t>
+          <t>SHP-009</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
@@ -7224,57 +7263,26 @@
           <t>Shop supplies</t>
         </is>
       </c>
-      <c r="C125" t="n">
-        <v>1</v>
-      </c>
       <c r="D125" t="inlineStr">
         <is>
-          <t>Loctite 4061 cyanoacrylate adhesive, 0.7 fl. oz., low viscosity (~20 cP)</t>
+          <t>USB-C chargers/cables</t>
         </is>
       </c>
       <c r="E125" t="inlineStr">
         <is>
-          <t>Plywood fiber conditioning and localized tack bonds</t>
-        </is>
-      </c>
-      <c r="F125" t="inlineStr">
-        <is>
-          <t>McMaster</t>
-        </is>
-      </c>
-      <c r="G125" t="inlineStr">
-        <is>
-          <t>1818A45</t>
-        </is>
-      </c>
-      <c r="H125" t="n">
-        <v>1</v>
-      </c>
-      <c r="I125" t="inlineStr">
-        <is>
-          <t>each</t>
+          <t>DP100 power</t>
         </is>
       </c>
       <c r="J125" t="inlineStr">
         <is>
           <t>In hand</t>
-        </is>
-      </c>
-      <c r="K125" t="inlineStr">
-        <is>
-          <t>§§6.2, 7, 8.4, 10.4</t>
-        </is>
-      </c>
-      <c r="L125" t="inlineStr">
-        <is>
-          <t>Use sparingly: wick into Baltic-birch fibers for spherical-washer sockets; use needle-sized localized drops for ABS/metal calibration tacks and captive screw retention. No accelerator required.</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>SHP-012</t>
+          <t>SHP-010</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
@@ -7282,35 +7290,14 @@
           <t>Shop supplies</t>
         </is>
       </c>
-      <c r="C126" t="n">
-        <v>1</v>
-      </c>
       <c r="D126" t="inlineStr">
         <is>
-          <t>UHMW Sheet 1/8" x 12" x 12"</t>
+          <t>Thermal compound</t>
         </is>
       </c>
       <c r="E126" t="inlineStr">
         <is>
-          <t>Mirror mount releasing assembly surface</t>
-        </is>
-      </c>
-      <c r="F126" t="inlineStr">
-        <is>
-          <t>US Plastics</t>
-        </is>
-      </c>
-      <c r="G126" t="inlineStr">
-        <is>
-          <t>46489</t>
-        </is>
-      </c>
-      <c r="H126" t="n">
-        <v>1</v>
-      </c>
-      <c r="I126" t="inlineStr">
-        <is>
-          <t>each</t>
+          <t>LED heatsink interfaces</t>
         </is>
       </c>
       <c r="J126" t="inlineStr">
@@ -7320,14 +7307,14 @@
       </c>
       <c r="K126" t="inlineStr">
         <is>
-          <t>§10.6</t>
+          <t>§6.4</t>
         </is>
       </c>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>SHP-013</t>
+          <t>SHP-011</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
@@ -7335,26 +7322,57 @@
           <t>Shop supplies</t>
         </is>
       </c>
+      <c r="C127" t="n">
+        <v>1</v>
+      </c>
       <c r="D127" t="inlineStr">
         <is>
-          <t>Soldering tools / supplies</t>
+          <t>Loctite 4061 cyanoacrylate adhesive, 0.7 fl. oz., low viscosity (~20 cP)</t>
         </is>
       </c>
       <c r="E127" t="inlineStr">
         <is>
-          <t>LED wiring</t>
+          <t>Plywood fiber conditioning and localized tack bonds</t>
+        </is>
+      </c>
+      <c r="F127" t="inlineStr">
+        <is>
+          <t>McMaster</t>
+        </is>
+      </c>
+      <c r="G127" t="inlineStr">
+        <is>
+          <t>1818A45</t>
+        </is>
+      </c>
+      <c r="H127" t="n">
+        <v>1</v>
+      </c>
+      <c r="I127" t="inlineStr">
+        <is>
+          <t>each</t>
         </is>
       </c>
       <c r="J127" t="inlineStr">
         <is>
           <t>In hand</t>
+        </is>
+      </c>
+      <c r="K127" t="inlineStr">
+        <is>
+          <t>§§6.2, 7, 8.4, 10.4</t>
+        </is>
+      </c>
+      <c r="L127" t="inlineStr">
+        <is>
+          <t>Use sparingly: wick into Baltic-birch fibers for spherical-washer sockets; use needle-sized localized drops for ABS/metal calibration tacks and captive screw retention. No accelerator required.</t>
         </is>
       </c>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>SHP-014</t>
+          <t>SHP-012</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
@@ -7367,22 +7385,22 @@
       </c>
       <c r="D128" t="inlineStr">
         <is>
-          <t>West System G/Flex 650 Epoxy Adhesive, 2 x 4 oz</t>
+          <t>UHMW Sheet 1/8" x 12" x 12"</t>
         </is>
       </c>
       <c r="E128" t="inlineStr">
         <is>
-          <t>Mirror cell adjuster sleeves, spring seat washer tack</t>
+          <t>Mirror mount releasing assembly surface</t>
         </is>
       </c>
       <c r="F128" t="inlineStr">
         <is>
-          <t>Amazon</t>
+          <t>US Plastics</t>
         </is>
       </c>
       <c r="G128" t="inlineStr">
         <is>
-          <t>B002IZFPQE</t>
+          <t>46489</t>
         </is>
       </c>
       <c r="H128" t="n">
@@ -7400,14 +7418,14 @@
       </c>
       <c r="K128" t="inlineStr">
         <is>
-          <t>§10.2</t>
+          <t>§10.6</t>
         </is>
       </c>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>SHP-015</t>
+          <t>SHP-013</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
@@ -7415,57 +7433,26 @@
           <t>Shop supplies</t>
         </is>
       </c>
-      <c r="C129" t="n">
-        <v>1</v>
-      </c>
       <c r="D129" t="inlineStr">
         <is>
-          <t>Silicone grease, clear, NLGI 1</t>
+          <t>Soldering tools / supplies</t>
         </is>
       </c>
       <c r="E129" t="inlineStr">
         <is>
-          <t>ABS carriage sliding-interface lubricant</t>
-        </is>
-      </c>
-      <c r="F129" t="inlineStr">
-        <is>
-          <t>McMaster</t>
-        </is>
-      </c>
-      <c r="G129" t="inlineStr">
-        <is>
-          <t>1418K51</t>
-        </is>
-      </c>
-      <c r="H129" t="n">
-        <v>1</v>
-      </c>
-      <c r="I129" t="inlineStr">
-        <is>
-          <t>each</t>
+          <t>LED wiring</t>
         </is>
       </c>
       <c r="J129" t="inlineStr">
         <is>
           <t>In hand</t>
-        </is>
-      </c>
-      <c r="K129" t="inlineStr">
-        <is>
-          <t>§8.4</t>
-        </is>
-      </c>
-      <c r="L129" t="inlineStr">
-        <is>
-          <t>Use only a trace film on dressed ABS-on-ABS sliding interfaces.</t>
         </is>
       </c>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>SHP-016</t>
+          <t>SHP-014</t>
         </is>
       </c>
       <c r="B130" t="inlineStr">
@@ -7478,17 +7465,22 @@
       </c>
       <c r="D130" t="inlineStr">
         <is>
-          <t>White lithium grease, NLGI #2</t>
+          <t>West System G/Flex 650 Epoxy Adhesive, 2 x 4 oz</t>
         </is>
       </c>
       <c r="E130" t="inlineStr">
         <is>
-          <t>Light grease for mirror-cell spherical washer interfaces</t>
+          <t>Mirror cell adjuster sleeves, spring seat washer tack</t>
         </is>
       </c>
       <c r="F130" t="inlineStr">
         <is>
-          <t>Lucas Oil Products</t>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="G130" t="inlineStr">
+        <is>
+          <t>B002IZFPQE</t>
         </is>
       </c>
       <c r="H130" t="n">
@@ -7506,19 +7498,14 @@
       </c>
       <c r="K130" t="inlineStr">
         <is>
-          <t>§10.4</t>
-        </is>
-      </c>
-      <c r="L130" t="inlineStr">
-        <is>
-          <t>Existing shop stock inspected 2026-09-16 and appears usable.</t>
+          <t>§10.2</t>
         </is>
       </c>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>SHP-017</t>
+          <t>SHP-015</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
@@ -7531,12 +7518,12 @@
       </c>
       <c r="D131" t="inlineStr">
         <is>
-          <t>1/2" Forstner bit, standard-point smooth-finish</t>
+          <t>Silicone grease, clear, NLGI 1</t>
         </is>
       </c>
       <c r="E131" t="inlineStr">
         <is>
-          <t>Spherical-washer counterbores</t>
+          <t>ABS carriage sliding-interface lubricant</t>
         </is>
       </c>
       <c r="F131" t="inlineStr">
@@ -7546,7 +7533,7 @@
       </c>
       <c r="G131" t="inlineStr">
         <is>
-          <t>2890A56</t>
+          <t>1418K51</t>
         </is>
       </c>
       <c r="H131" t="n">
@@ -7564,19 +7551,19 @@
       </c>
       <c r="K131" t="inlineStr">
         <is>
-          <t>§10.4</t>
+          <t>§8.4</t>
         </is>
       </c>
       <c r="L131" t="inlineStr">
         <is>
-          <t>Use in drill press for shallow close-fit spherical-washer sockets; test in scrap Baltic birch before cutting final plate.</t>
+          <t>Use only a trace film on dressed ABS-on-ABS sliding interfaces.</t>
         </is>
       </c>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>SHP-018</t>
+          <t>SHP-016</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
@@ -7589,22 +7576,17 @@
       </c>
       <c r="D132" t="inlineStr">
         <is>
-          <t>5/8" Forstner bit, standard-point smooth-finish</t>
+          <t>White lithium grease, NLGI #2</t>
         </is>
       </c>
       <c r="E132" t="inlineStr">
         <is>
-          <t>Spring-seat washer counterbores</t>
+          <t>Light grease for mirror-cell spherical washer interfaces</t>
         </is>
       </c>
       <c r="F132" t="inlineStr">
         <is>
-          <t>McMaster</t>
-        </is>
-      </c>
-      <c r="G132" t="inlineStr">
-        <is>
-          <t>2890A58</t>
+          <t>Lucas Oil Products</t>
         </is>
       </c>
       <c r="H132" t="n">
@@ -7622,19 +7604,19 @@
       </c>
       <c r="K132" t="inlineStr">
         <is>
-          <t>§10.3</t>
+          <t>§10.4</t>
         </is>
       </c>
       <c r="L132" t="inlineStr">
         <is>
-          <t>Use in drill press for shallow spring-seat-washer registration counterbores; test depth/fit in scrap first.</t>
+          <t>Existing shop stock inspected 2026-09-16 and appears usable.</t>
         </is>
       </c>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>SHP-019</t>
+          <t>SHP-017</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
@@ -7647,12 +7629,12 @@
       </c>
       <c r="D133" t="inlineStr">
         <is>
-          <t>M4 × 0.7 high-speed-steel plug-chamfer hex-bit tap</t>
+          <t>1/2" Forstner bit, standard-point smooth-finish</t>
         </is>
       </c>
       <c r="E133" t="inlineStr">
         <is>
-          <t>Tap CAMVATE quick-release plate mounting holes</t>
+          <t>Spherical-washer counterbores</t>
         </is>
       </c>
       <c r="F133" t="inlineStr">
@@ -7662,7 +7644,7 @@
       </c>
       <c r="G133" t="inlineStr">
         <is>
-          <t>1021N23</t>
+          <t>2890A56</t>
         </is>
       </c>
       <c r="H133" t="n">
@@ -7680,19 +7662,19 @@
       </c>
       <c r="K133" t="inlineStr">
         <is>
-          <t>§10.9</t>
+          <t>§10.4</t>
         </is>
       </c>
       <c r="L133" t="inlineStr">
         <is>
-          <t>Use with 3.3 mm tap drill; exact hole locations await measurement of the delivered plate.</t>
+          <t>Use in drill press for shallow close-fit spherical-washer sockets; test in scrap Baltic birch before cutting final plate.</t>
         </is>
       </c>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>SHP-020</t>
+          <t>SHP-018</t>
         </is>
       </c>
       <c r="B134" t="inlineStr">
@@ -7705,12 +7687,12 @@
       </c>
       <c r="D134" t="inlineStr">
         <is>
-          <t>3.3 mm black-oxide HSS jobber-length drill bit</t>
+          <t>5/8" Forstner bit, standard-point smooth-finish</t>
         </is>
       </c>
       <c r="E134" t="inlineStr">
         <is>
-          <t>M4 × 0.7 tap drill for CAMVATE quick-release plate</t>
+          <t>Spring-seat washer counterbores</t>
         </is>
       </c>
       <c r="F134" t="inlineStr">
@@ -7720,7 +7702,7 @@
       </c>
       <c r="G134" t="inlineStr">
         <is>
-          <t>2958A64</t>
+          <t>2890A58</t>
         </is>
       </c>
       <c r="H134" t="n">
@@ -7738,19 +7720,19 @@
       </c>
       <c r="K134" t="inlineStr">
         <is>
-          <t>§10.9</t>
+          <t>§10.3</t>
         </is>
       </c>
       <c r="L134" t="inlineStr">
         <is>
-          <t>Standard 3.3 mm tap-drill size for M4 × 0.7.</t>
+          <t>Use in drill press for shallow spring-seat-washer registration counterbores; test depth/fit in scrap first.</t>
         </is>
       </c>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>SHP-021</t>
+          <t>SHP-019</t>
         </is>
       </c>
       <c r="B135" t="inlineStr">
@@ -7763,12 +7745,12 @@
       </c>
       <c r="D135" t="inlineStr">
         <is>
-          <t>Loctite 243 medium-strength removable threadlocker, 0.34 fl. oz.</t>
+          <t>M4 × 0.7 high-speed-steel plug-chamfer hex-bit tap</t>
         </is>
       </c>
       <c r="E135" t="inlineStr">
         <is>
-          <t>Removable thread retention for quick-release plate mounting screws</t>
+          <t>Tap CAMVATE quick-release plate mounting holes</t>
         </is>
       </c>
       <c r="F135" t="inlineStr">
@@ -7778,7 +7760,7 @@
       </c>
       <c r="G135" t="inlineStr">
         <is>
-          <t>91458A115</t>
+          <t>1021N23</t>
         </is>
       </c>
       <c r="H135" t="n">
@@ -7801,14 +7783,14 @@
       </c>
       <c r="L135" t="inlineStr">
         <is>
-          <t>Apply only after fit and screw length are validated; preferred over high-strength Loctite 271 for this serviceable joint.</t>
+          <t>Use with 3.3 mm tap drill; exact hole locations await measurement of the delivered plate.</t>
         </is>
       </c>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>SHP-022</t>
+          <t>SHP-020</t>
         </is>
       </c>
       <c r="B136" t="inlineStr">
@@ -7821,22 +7803,22 @@
       </c>
       <c r="D136" t="inlineStr">
         <is>
-          <t>Rosco Photofoil matte black aluminum wrap, 12"x10'</t>
+          <t>3.3 mm black-oxide HSS jobber-length drill bit</t>
         </is>
       </c>
       <c r="E136" t="inlineStr">
         <is>
-          <t>Opaque masking / thin-sheet cutoff experiments</t>
+          <t>M4 × 0.7 tap drill for CAMVATE quick-release plate</t>
         </is>
       </c>
       <c r="F136" t="inlineStr">
         <is>
-          <t>Fullcompass</t>
+          <t>McMaster</t>
         </is>
       </c>
       <c r="G136" t="inlineStr">
         <is>
-          <t>01001-1210</t>
+          <t>2958A64</t>
         </is>
       </c>
       <c r="H136" t="n">
@@ -7844,7 +7826,7 @@
       </c>
       <c r="I136" t="inlineStr">
         <is>
-          <t>pack</t>
+          <t>each</t>
         </is>
       </c>
       <c r="J136" t="inlineStr">
@@ -7854,58 +7836,174 @@
       </c>
       <c r="K136" t="inlineStr">
         <is>
-          <t>§§8, 8.7</t>
+          <t>§10.9</t>
         </is>
       </c>
       <c r="L136" t="inlineStr">
         <is>
-          <t>Retained as general shop stock for opaque masking and thin-sheet cutoff experiments.</t>
+          <t>Standard 3.3 mm tap-drill size for M4 × 0.7.</t>
         </is>
       </c>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
+          <t>SHP-021</t>
+        </is>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>Shop supplies</t>
+        </is>
+      </c>
+      <c r="C137" t="n">
+        <v>1</v>
+      </c>
+      <c r="D137" t="inlineStr">
+        <is>
+          <t>Loctite 243 medium-strength removable threadlocker, 0.34 fl. oz.</t>
+        </is>
+      </c>
+      <c r="E137" t="inlineStr">
+        <is>
+          <t>Removable thread retention for quick-release plate mounting screws</t>
+        </is>
+      </c>
+      <c r="F137" t="inlineStr">
+        <is>
+          <t>McMaster</t>
+        </is>
+      </c>
+      <c r="G137" t="inlineStr">
+        <is>
+          <t>91458A115</t>
+        </is>
+      </c>
+      <c r="H137" t="n">
+        <v>1</v>
+      </c>
+      <c r="I137" t="inlineStr">
+        <is>
+          <t>each</t>
+        </is>
+      </c>
+      <c r="J137" t="inlineStr">
+        <is>
+          <t>In hand</t>
+        </is>
+      </c>
+      <c r="K137" t="inlineStr">
+        <is>
+          <t>§10.9</t>
+        </is>
+      </c>
+      <c r="L137" t="inlineStr">
+        <is>
+          <t>Apply only after fit and screw length are validated; preferred over high-strength Loctite 271 for this serviceable joint.</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>SHP-022</t>
+        </is>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>Shop supplies</t>
+        </is>
+      </c>
+      <c r="C138" t="n">
+        <v>1</v>
+      </c>
+      <c r="D138" t="inlineStr">
+        <is>
+          <t>Rosco Photofoil matte black aluminum wrap, 12"x10'</t>
+        </is>
+      </c>
+      <c r="E138" t="inlineStr">
+        <is>
+          <t>Opaque masking / thin-sheet cutoff experiments</t>
+        </is>
+      </c>
+      <c r="F138" t="inlineStr">
+        <is>
+          <t>Fullcompass</t>
+        </is>
+      </c>
+      <c r="G138" t="inlineStr">
+        <is>
+          <t>01001-1210</t>
+        </is>
+      </c>
+      <c r="H138" t="n">
+        <v>1</v>
+      </c>
+      <c r="I138" t="inlineStr">
+        <is>
+          <t>pack</t>
+        </is>
+      </c>
+      <c r="J138" t="inlineStr">
+        <is>
+          <t>In hand</t>
+        </is>
+      </c>
+      <c r="K138" t="inlineStr">
+        <is>
+          <t>§§8, 8.7</t>
+        </is>
+      </c>
+      <c r="L138" t="inlineStr">
+        <is>
+          <t>Retained as general shop stock for opaque masking and thin-sheet cutoff experiments.</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
           <t>SHP-023</t>
         </is>
       </c>
-      <c r="B137" t="inlineStr">
+      <c r="B139" t="inlineStr">
         <is>
           <t>Shop supplies</t>
         </is>
       </c>
-      <c r="C137" t="n">
-        <v>1</v>
-      </c>
-      <c r="D137" t="inlineStr">
+      <c r="C139" t="n">
+        <v>1</v>
+      </c>
+      <c r="D139" t="inlineStr">
         <is>
           <t>M3 × 0.5 tap and 2.5 mm tap drill</t>
         </is>
       </c>
-      <c r="E137" t="inlineStr">
+      <c r="E139" t="inlineStr">
         <is>
           <t>Tap SM1CP2M rear for heatsink screws</t>
         </is>
       </c>
-      <c r="J137" t="inlineStr">
+      <c r="J139" t="inlineStr">
         <is>
           <t>Specified</t>
         </is>
       </c>
-      <c r="K137" t="inlineStr">
+      <c r="K139" t="inlineStr">
         <is>
           <t>§6.2</t>
         </is>
       </c>
-      <c r="L137" t="inlineStr">
+      <c r="L139" t="inlineStr">
         <is>
           <t>Confirm whether already in shop stock before purchasing; vendor and SKU not yet chosen.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L137"/>
-  <conditionalFormatting sqref="J2:J137">
+  <autoFilter ref="A1:L139"/>
+  <conditionalFormatting sqref="J2:J139">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"In hand"</formula>
     </cfRule>

</xml_diff>

<commit_message>
add light source drill/tap plan
</commit_message>
<xml_diff>
--- a/bom/schlieren-bom.xlsx
+++ b/bom/schlieren-bom.xlsx
@@ -11,7 +11,7 @@
     <sheet name="BOM" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'BOM'!$A$1:$L$139</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'BOM'!$A$1:$L$141</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -837,7 +837,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L139"/>
+  <dimension ref="A1:L141"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -2991,6 +2991,9 @@
           <t>Light source</t>
         </is>
       </c>
+      <c r="C42" t="n">
+        <v>6</v>
+      </c>
       <c r="D42" t="inlineStr">
         <is>
           <t>M3 × 6 mm socket head screw</t>
@@ -3013,12 +3016,12 @@
       </c>
       <c r="K42" t="inlineStr">
         <is>
-          <t>§6.2</t>
+          <t>§§6.2, 6.4</t>
         </is>
       </c>
       <c r="L42" t="inlineStr">
         <is>
-          <t>Provisional length (3 mm base + ~2.5 mm thread into cap). Quantity per module (2–3) and SKU to be confirmed; check existing M3 stock.</t>
+          <t>Three per module. Provisional length (3 mm base + ~3 mm thread into the through-tapped cap; shorter than the cap thickness). SKU to be confirmed; check existing M3 stock.</t>
         </is>
       </c>
     </row>
@@ -7139,6 +7142,11 @@
           <t>§6.4</t>
         </is>
       </c>
+      <c r="L121" t="inlineStr">
+        <is>
+          <t>Plug chamfer; sufficient for the through M2 holes.</t>
+        </is>
+      </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
@@ -7808,7 +7816,7 @@
       </c>
       <c r="E136" t="inlineStr">
         <is>
-          <t>M4 × 0.7 tap drill for CAMVATE quick-release plate</t>
+          <t>M4 × 0.7 tap drill for CAMVATE quick-release plate; M3 heatsink clearance holes</t>
         </is>
       </c>
       <c r="F136" t="inlineStr">
@@ -7836,12 +7844,12 @@
       </c>
       <c r="K136" t="inlineStr">
         <is>
-          <t>§10.9</t>
+          <t>§§6.4, 10.9</t>
         </is>
       </c>
       <c r="L136" t="inlineStr">
         <is>
-          <t>Standard 3.3 mm tap-drill size for M4 × 0.7.</t>
+          <t>Standard 3.3 mm tap-drill size for M4 × 0.7. Also drills the Ø3.3 M3 clearance holes in the heatsink base (§6.4).</t>
         </is>
       </c>
     </row>
@@ -7977,33 +7985,167 @@
       </c>
       <c r="D139" t="inlineStr">
         <is>
-          <t>M3 × 0.5 tap and 2.5 mm tap drill</t>
+          <t>M3 × 0.5 high-speed-steel plug-chamfer tap, 5/8" thread length</t>
         </is>
       </c>
       <c r="E139" t="inlineStr">
         <is>
-          <t>Tap SM1CP2M rear for heatsink screws</t>
+          <t>Tap through M3 heatsink-screw holes in SM1CP2M cap</t>
+        </is>
+      </c>
+      <c r="F139" t="inlineStr">
+        <is>
+          <t>McMaster</t>
+        </is>
+      </c>
+      <c r="G139" t="inlineStr">
+        <is>
+          <t>8305A32</t>
+        </is>
+      </c>
+      <c r="H139" t="n">
+        <v>1</v>
+      </c>
+      <c r="I139" t="inlineStr">
+        <is>
+          <t>each</t>
         </is>
       </c>
       <c r="J139" t="inlineStr">
         <is>
-          <t>Specified</t>
+          <t>To procure</t>
         </is>
       </c>
       <c r="K139" t="inlineStr">
         <is>
-          <t>§6.2</t>
+          <t>§6.4</t>
         </is>
       </c>
       <c r="L139" t="inlineStr">
         <is>
-          <t>Confirm whether already in shop stock before purchasing; vendor and SKU not yet chosen.</t>
+          <t>All holes are through holes, so a plug chamfer is enough; no bottoming tap needed. Use with the 2.5 mm tap drill (SHP-025). Confirm no M3 tap already in shop stock.</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>SHP-025</t>
+        </is>
+      </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>Shop supplies</t>
+        </is>
+      </c>
+      <c r="C140" t="n">
+        <v>1</v>
+      </c>
+      <c r="D140" t="inlineStr">
+        <is>
+          <t>2.5 mm TiN-coated HSS short-length drill bit, 43 mm overall</t>
+        </is>
+      </c>
+      <c r="E140" t="inlineStr">
+        <is>
+          <t>M3 tap drill for through holes in SM1CP2M cap</t>
+        </is>
+      </c>
+      <c r="F140" t="inlineStr">
+        <is>
+          <t>McMaster</t>
+        </is>
+      </c>
+      <c r="G140" t="inlineStr">
+        <is>
+          <t>2979N15</t>
+        </is>
+      </c>
+      <c r="H140" t="n">
+        <v>1</v>
+      </c>
+      <c r="I140" t="inlineStr">
+        <is>
+          <t>each</t>
+        </is>
+      </c>
+      <c r="J140" t="inlineStr">
+        <is>
+          <t>To procure</t>
+        </is>
+      </c>
+      <c r="K140" t="inlineStr">
+        <is>
+          <t>§6.4</t>
+        </is>
+      </c>
+      <c r="L140" t="inlineStr">
+        <is>
+          <t>Short-length stub drill for rigid drilling in the thin cap; same series as the 1.6 mm drill SHP-006.</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>SHP-026</t>
+        </is>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>Shop supplies</t>
+        </is>
+      </c>
+      <c r="C141" t="n">
+        <v>1</v>
+      </c>
+      <c r="D141" t="inlineStr">
+        <is>
+          <t>2.0 mm uncoated HSS short-length drill bit, 38 mm overall</t>
+        </is>
+      </c>
+      <c r="E141" t="inlineStr">
+        <is>
+          <t>Lead holes through SM1CP2M cap and heatsink base</t>
+        </is>
+      </c>
+      <c r="F141" t="inlineStr">
+        <is>
+          <t>McMaster</t>
+        </is>
+      </c>
+      <c r="G141" t="inlineStr">
+        <is>
+          <t>2979N14</t>
+        </is>
+      </c>
+      <c r="H141" t="n">
+        <v>1</v>
+      </c>
+      <c r="I141" t="inlineStr">
+        <is>
+          <t>each</t>
+        </is>
+      </c>
+      <c r="J141" t="inlineStr">
+        <is>
+          <t>To procure</t>
+        </is>
+      </c>
+      <c r="K141" t="inlineStr">
+        <is>
+          <t>§6.4</t>
+        </is>
+      </c>
+      <c r="L141" t="inlineStr">
+        <is>
+          <t>Same series as the 1.6 mm drill SHP-006.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L139"/>
-  <conditionalFormatting sqref="J2:J139">
+  <autoFilter ref="A1:L141"/>
+  <conditionalFormatting sqref="J2:J141">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"In hand"</formula>
     </cfRule>

</xml_diff>

<commit_message>
Add mirror cell model
</commit_message>
<xml_diff>
--- a/bom/schlieren-bom.xlsx
+++ b/bom/schlieren-bom.xlsx
@@ -11,7 +11,7 @@
     <sheet name="BOM" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'BOM'!$A$1:$L$141</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'BOM'!$A$1:$L$142</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -837,7 +837,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L141"/>
+  <dimension ref="A1:L142"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -6267,7 +6267,7 @@
         </is>
       </c>
       <c r="C105" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="D105" t="inlineStr">
         <is>
@@ -6309,7 +6309,7 @@
       </c>
       <c r="L105" t="inlineStr">
         <is>
-          <t>Six installed for the revised three-fastener-per-bracket pattern; existing stock confirmed in hand.</t>
+          <t>Eight installed, four per bracket; existing stock was confirmed in hand for six, so confirm two more.</t>
         </is>
       </c>
     </row>
@@ -6325,7 +6325,7 @@
         </is>
       </c>
       <c r="C106" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="D106" t="inlineStr">
         <is>
@@ -6367,7 +6367,7 @@
       </c>
       <c r="L106" t="inlineStr">
         <is>
-          <t>Six installed for the revised three-fastener-per-bracket pattern.</t>
+          <t>Eight installed, one under each bracket locknut.</t>
         </is>
       </c>
     </row>
@@ -6851,9 +6851,6 @@
           <t>Mirror cell</t>
         </is>
       </c>
-      <c r="C116" t="n">
-        <v>6</v>
-      </c>
       <c r="D116" t="inlineStr">
         <is>
           <t>5/16"-18 × 1-3/8" hex-drive flat-head screw, 316 SS</t>
@@ -6861,7 +6858,7 @@
       </c>
       <c r="E116" t="inlineStr">
         <is>
-          <t>Primary structural-bracket screws</t>
+          <t>Existing alternate bracket screw stock</t>
         </is>
       </c>
       <c r="F116" t="inlineStr">
@@ -6894,27 +6891,32 @@
       </c>
       <c r="L116" t="inlineStr">
         <is>
-          <t>Use six installed: two through the vertical plate and one through the base plate per bracket. Two 5-packs required; four spare.</t>
+          <t>Former baseline bracket screw; retained as in-hand alternate stock after the change to button-head screws (MIR-026).</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>SHP-001</t>
+          <t>MIR-026</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>Shop supplies</t>
+          <t>Mirror cell</t>
         </is>
       </c>
       <c r="C117" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="D117" t="inlineStr">
         <is>
-          <t>Loctite 271 threadlocker, .34 fl. oz.</t>
+          <t>5/16"-18 × 1-3/8" 316 stainless button-head hex-drive screw</t>
+        </is>
+      </c>
+      <c r="E117" t="inlineStr">
+        <is>
+          <t>Bracket screws, heads on the bracket</t>
         </is>
       </c>
       <c r="F117" t="inlineStr">
@@ -6924,32 +6926,37 @@
       </c>
       <c r="G117" t="inlineStr">
         <is>
-          <t>91458A160</t>
+          <t>98164A527</t>
         </is>
       </c>
       <c r="H117" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="I117" t="inlineStr">
         <is>
-          <t>each</t>
+          <t>pack</t>
         </is>
       </c>
       <c r="J117" t="inlineStr">
         <is>
-          <t>In hand</t>
+          <t>To procure</t>
         </is>
       </c>
       <c r="K117" t="inlineStr">
         <is>
-          <t>§9.5</t>
+          <t>§10.7</t>
+        </is>
+      </c>
+      <c r="L117" t="inlineStr">
+        <is>
+          <t>Four per bracket, two through the plate and two through the base; eight installed, so order two 5-packs (two spare). 3/16 in hex drive; head Ø0.547 in × 0.166 in. Pushed through from the bracket side, with MIR-013 washers and MIR-012 locknuts behind the plywood. Thread projects about 0.12 in past the locknut.</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>SHP-002</t>
+          <t>SHP-001</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
@@ -6962,7 +6969,7 @@
       </c>
       <c r="D118" t="inlineStr">
         <is>
-          <t>Heat-set installation tip</t>
+          <t>Loctite 271 threadlocker, .34 fl. oz.</t>
         </is>
       </c>
       <c r="F118" t="inlineStr">
@@ -6972,7 +6979,7 @@
       </c>
       <c r="G118" t="inlineStr">
         <is>
-          <t>92160A327</t>
+          <t>91458A160</t>
         </is>
       </c>
       <c r="H118" t="n">
@@ -6997,7 +7004,7 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>SHP-003</t>
+          <t>SHP-002</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
@@ -7010,17 +7017,17 @@
       </c>
       <c r="D119" t="inlineStr">
         <is>
-          <t>Optical spanner wrench</t>
+          <t>Heat-set installation tip</t>
         </is>
       </c>
       <c r="F119" t="inlineStr">
         <is>
-          <t>Amazon</t>
+          <t>McMaster</t>
         </is>
       </c>
       <c r="G119" t="inlineStr">
         <is>
-          <t>B0CKSL364Q</t>
+          <t>92160A327</t>
         </is>
       </c>
       <c r="H119" t="n">
@@ -7034,13 +7041,18 @@
       <c r="J119" t="inlineStr">
         <is>
           <t>In hand</t>
+        </is>
+      </c>
+      <c r="K119" t="inlineStr">
+        <is>
+          <t>§9.5</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>SHP-004</t>
+          <t>SHP-003</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
@@ -7053,12 +7065,7 @@
       </c>
       <c r="D120" t="inlineStr">
         <is>
-          <t>Metric feeler gauge set</t>
-        </is>
-      </c>
-      <c r="E120" t="inlineStr">
-        <is>
-          <t>Source-slit blade spacing</t>
+          <t>Optical spanner wrench</t>
         </is>
       </c>
       <c r="F120" t="inlineStr">
@@ -7068,7 +7075,7 @@
       </c>
       <c r="G120" t="inlineStr">
         <is>
-          <t>B07XPD9L1C</t>
+          <t>B0CKSL364Q</t>
         </is>
       </c>
       <c r="H120" t="n">
@@ -7082,18 +7089,13 @@
       <c r="J120" t="inlineStr">
         <is>
           <t>In hand</t>
-        </is>
-      </c>
-      <c r="K120" t="inlineStr">
-        <is>
-          <t>§7.4</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>SHP-005</t>
+          <t>SHP-004</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
@@ -7106,22 +7108,22 @@
       </c>
       <c r="D121" t="inlineStr">
         <is>
-          <t>M2 tap</t>
+          <t>Metric feeler gauge set</t>
         </is>
       </c>
       <c r="E121" t="inlineStr">
         <is>
-          <t>LED board mounting into SM1CP2M cap</t>
+          <t>Source-slit blade spacing</t>
         </is>
       </c>
       <c r="F121" t="inlineStr">
         <is>
-          <t>McMaster</t>
+          <t>Amazon</t>
         </is>
       </c>
       <c r="G121" t="inlineStr">
         <is>
-          <t>8305A78</t>
+          <t>B07XPD9L1C</t>
         </is>
       </c>
       <c r="H121" t="n">
@@ -7139,19 +7141,14 @@
       </c>
       <c r="K121" t="inlineStr">
         <is>
-          <t>§6.4</t>
-        </is>
-      </c>
-      <c r="L121" t="inlineStr">
-        <is>
-          <t>Plug chamfer; sufficient for the through M2 holes.</t>
+          <t>§7.4</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>SHP-006</t>
+          <t>SHP-005</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
@@ -7164,12 +7161,12 @@
       </c>
       <c r="D122" t="inlineStr">
         <is>
-          <t>M2 tap drill, 1.6mm</t>
+          <t>M2 tap</t>
         </is>
       </c>
       <c r="E122" t="inlineStr">
         <is>
-          <t>LED mounting</t>
+          <t>LED board mounting into SM1CP2M cap</t>
         </is>
       </c>
       <c r="F122" t="inlineStr">
@@ -7179,7 +7176,7 @@
       </c>
       <c r="G122" t="inlineStr">
         <is>
-          <t>2979N13</t>
+          <t>8305A78</t>
         </is>
       </c>
       <c r="H122" t="n">
@@ -7198,13 +7195,18 @@
       <c r="K122" t="inlineStr">
         <is>
           <t>§6.4</t>
+        </is>
+      </c>
+      <c r="L122" t="inlineStr">
+        <is>
+          <t>Plug chamfer; sufficient for the through M2 holes.</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>SHP-007</t>
+          <t>SHP-006</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
@@ -7212,14 +7214,35 @@
           <t>Shop supplies</t>
         </is>
       </c>
+      <c r="C123" t="n">
+        <v>1</v>
+      </c>
       <c r="D123" t="inlineStr">
         <is>
-          <t>18 AWG wire</t>
+          <t>M2 tap drill, 1.6mm</t>
         </is>
       </c>
       <c r="E123" t="inlineStr">
         <is>
-          <t>LED wiring</t>
+          <t>LED mounting</t>
+        </is>
+      </c>
+      <c r="F123" t="inlineStr">
+        <is>
+          <t>McMaster</t>
+        </is>
+      </c>
+      <c r="G123" t="inlineStr">
+        <is>
+          <t>2979N13</t>
+        </is>
+      </c>
+      <c r="H123" t="n">
+        <v>1</v>
+      </c>
+      <c r="I123" t="inlineStr">
+        <is>
+          <t>each</t>
         </is>
       </c>
       <c r="J123" t="inlineStr">
@@ -7229,14 +7252,14 @@
       </c>
       <c r="K123" t="inlineStr">
         <is>
-          <t>§6.5</t>
+          <t>§6.4</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>SHP-008</t>
+          <t>SHP-007</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
@@ -7246,7 +7269,7 @@
       </c>
       <c r="D124" t="inlineStr">
         <is>
-          <t>Heat-shrink tubing</t>
+          <t>18 AWG wire</t>
         </is>
       </c>
       <c r="E124" t="inlineStr">
@@ -7257,13 +7280,18 @@
       <c r="J124" t="inlineStr">
         <is>
           <t>In hand</t>
+        </is>
+      </c>
+      <c r="K124" t="inlineStr">
+        <is>
+          <t>§6.5</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>SHP-009</t>
+          <t>SHP-008</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
@@ -7273,12 +7301,12 @@
       </c>
       <c r="D125" t="inlineStr">
         <is>
-          <t>USB-C chargers/cables</t>
+          <t>Heat-shrink tubing</t>
         </is>
       </c>
       <c r="E125" t="inlineStr">
         <is>
-          <t>DP100 power</t>
+          <t>LED wiring</t>
         </is>
       </c>
       <c r="J125" t="inlineStr">
@@ -7290,7 +7318,7 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>SHP-010</t>
+          <t>SHP-009</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
@@ -7300,29 +7328,24 @@
       </c>
       <c r="D126" t="inlineStr">
         <is>
-          <t>Thermal compound</t>
+          <t>USB-C chargers/cables</t>
         </is>
       </c>
       <c r="E126" t="inlineStr">
         <is>
-          <t>LED heatsink interfaces</t>
+          <t>DP100 power</t>
         </is>
       </c>
       <c r="J126" t="inlineStr">
         <is>
           <t>In hand</t>
-        </is>
-      </c>
-      <c r="K126" t="inlineStr">
-        <is>
-          <t>§6.4</t>
         </is>
       </c>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>SHP-011</t>
+          <t>SHP-010</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
@@ -7330,35 +7353,14 @@
           <t>Shop supplies</t>
         </is>
       </c>
-      <c r="C127" t="n">
-        <v>1</v>
-      </c>
       <c r="D127" t="inlineStr">
         <is>
-          <t>Loctite 4061 cyanoacrylate adhesive, 0.7 fl. oz., low viscosity (~20 cP)</t>
+          <t>Thermal compound</t>
         </is>
       </c>
       <c r="E127" t="inlineStr">
         <is>
-          <t>Plywood fiber conditioning and localized tack bonds</t>
-        </is>
-      </c>
-      <c r="F127" t="inlineStr">
-        <is>
-          <t>McMaster</t>
-        </is>
-      </c>
-      <c r="G127" t="inlineStr">
-        <is>
-          <t>1818A45</t>
-        </is>
-      </c>
-      <c r="H127" t="n">
-        <v>1</v>
-      </c>
-      <c r="I127" t="inlineStr">
-        <is>
-          <t>each</t>
+          <t>LED heatsink interfaces</t>
         </is>
       </c>
       <c r="J127" t="inlineStr">
@@ -7368,19 +7370,14 @@
       </c>
       <c r="K127" t="inlineStr">
         <is>
-          <t>§§6.2, 7, 8.4, 10.4</t>
-        </is>
-      </c>
-      <c r="L127" t="inlineStr">
-        <is>
-          <t>Use sparingly: wick into Baltic-birch fibers for spherical-washer sockets; use needle-sized localized drops for ABS/metal calibration tacks and captive screw retention. No accelerator required.</t>
+          <t>§6.4</t>
         </is>
       </c>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>SHP-012</t>
+          <t>SHP-011</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
@@ -7393,22 +7390,22 @@
       </c>
       <c r="D128" t="inlineStr">
         <is>
-          <t>UHMW Sheet 1/8" x 12" x 12"</t>
+          <t>Loctite 4061 cyanoacrylate adhesive, 0.7 fl. oz., low viscosity (~20 cP)</t>
         </is>
       </c>
       <c r="E128" t="inlineStr">
         <is>
-          <t>Mirror mount releasing assembly surface</t>
+          <t>Plywood fiber conditioning and localized tack bonds</t>
         </is>
       </c>
       <c r="F128" t="inlineStr">
         <is>
-          <t>US Plastics</t>
+          <t>McMaster</t>
         </is>
       </c>
       <c r="G128" t="inlineStr">
         <is>
-          <t>46489</t>
+          <t>1818A45</t>
         </is>
       </c>
       <c r="H128" t="n">
@@ -7426,14 +7423,19 @@
       </c>
       <c r="K128" t="inlineStr">
         <is>
-          <t>§10.6</t>
+          <t>§§6.2, 7, 8.4, 10.4</t>
+        </is>
+      </c>
+      <c r="L128" t="inlineStr">
+        <is>
+          <t>Use sparingly: wick into Baltic-birch fibers for spherical-washer sockets; use needle-sized localized drops for ABS/metal calibration tacks and captive screw retention. No accelerator required.</t>
         </is>
       </c>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>SHP-013</t>
+          <t>SHP-012</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
@@ -7441,26 +7443,52 @@
           <t>Shop supplies</t>
         </is>
       </c>
+      <c r="C129" t="n">
+        <v>1</v>
+      </c>
       <c r="D129" t="inlineStr">
         <is>
-          <t>Soldering tools / supplies</t>
+          <t>UHMW Sheet 1/8" x 12" x 12"</t>
         </is>
       </c>
       <c r="E129" t="inlineStr">
         <is>
-          <t>LED wiring</t>
+          <t>Mirror mount releasing assembly surface</t>
+        </is>
+      </c>
+      <c r="F129" t="inlineStr">
+        <is>
+          <t>US Plastics</t>
+        </is>
+      </c>
+      <c r="G129" t="inlineStr">
+        <is>
+          <t>46489</t>
+        </is>
+      </c>
+      <c r="H129" t="n">
+        <v>1</v>
+      </c>
+      <c r="I129" t="inlineStr">
+        <is>
+          <t>each</t>
         </is>
       </c>
       <c r="J129" t="inlineStr">
         <is>
           <t>In hand</t>
+        </is>
+      </c>
+      <c r="K129" t="inlineStr">
+        <is>
+          <t>§10.6</t>
         </is>
       </c>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>SHP-014</t>
+          <t>SHP-013</t>
         </is>
       </c>
       <c r="B130" t="inlineStr">
@@ -7468,52 +7496,26 @@
           <t>Shop supplies</t>
         </is>
       </c>
-      <c r="C130" t="n">
-        <v>1</v>
-      </c>
       <c r="D130" t="inlineStr">
         <is>
-          <t>West System G/Flex 650 Epoxy Adhesive, 2 x 4 oz</t>
+          <t>Soldering tools / supplies</t>
         </is>
       </c>
       <c r="E130" t="inlineStr">
         <is>
-          <t>Mirror cell adjuster sleeves, spring seat washer tack</t>
-        </is>
-      </c>
-      <c r="F130" t="inlineStr">
-        <is>
-          <t>Amazon</t>
-        </is>
-      </c>
-      <c r="G130" t="inlineStr">
-        <is>
-          <t>B002IZFPQE</t>
-        </is>
-      </c>
-      <c r="H130" t="n">
-        <v>1</v>
-      </c>
-      <c r="I130" t="inlineStr">
-        <is>
-          <t>each</t>
+          <t>LED wiring</t>
         </is>
       </c>
       <c r="J130" t="inlineStr">
         <is>
           <t>In hand</t>
-        </is>
-      </c>
-      <c r="K130" t="inlineStr">
-        <is>
-          <t>§10.2</t>
         </is>
       </c>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>SHP-015</t>
+          <t>SHP-014</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
@@ -7526,22 +7528,22 @@
       </c>
       <c r="D131" t="inlineStr">
         <is>
-          <t>Silicone grease, clear, NLGI 1</t>
+          <t>West System G/Flex 650 Epoxy Adhesive, 2 x 4 oz</t>
         </is>
       </c>
       <c r="E131" t="inlineStr">
         <is>
-          <t>ABS carriage sliding-interface lubricant</t>
+          <t>Mirror cell adjuster sleeves, spring seat washer tack</t>
         </is>
       </c>
       <c r="F131" t="inlineStr">
         <is>
-          <t>McMaster</t>
+          <t>Amazon</t>
         </is>
       </c>
       <c r="G131" t="inlineStr">
         <is>
-          <t>1418K51</t>
+          <t>B002IZFPQE</t>
         </is>
       </c>
       <c r="H131" t="n">
@@ -7559,19 +7561,14 @@
       </c>
       <c r="K131" t="inlineStr">
         <is>
-          <t>§8.4</t>
-        </is>
-      </c>
-      <c r="L131" t="inlineStr">
-        <is>
-          <t>Use only a trace film on dressed ABS-on-ABS sliding interfaces.</t>
+          <t>§10.2</t>
         </is>
       </c>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>SHP-016</t>
+          <t>SHP-015</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
@@ -7584,17 +7581,22 @@
       </c>
       <c r="D132" t="inlineStr">
         <is>
-          <t>White lithium grease, NLGI #2</t>
+          <t>Silicone grease, clear, NLGI 1</t>
         </is>
       </c>
       <c r="E132" t="inlineStr">
         <is>
-          <t>Light grease for mirror-cell spherical washer interfaces</t>
+          <t>ABS carriage sliding-interface lubricant</t>
         </is>
       </c>
       <c r="F132" t="inlineStr">
         <is>
-          <t>Lucas Oil Products</t>
+          <t>McMaster</t>
+        </is>
+      </c>
+      <c r="G132" t="inlineStr">
+        <is>
+          <t>1418K51</t>
         </is>
       </c>
       <c r="H132" t="n">
@@ -7612,19 +7614,19 @@
       </c>
       <c r="K132" t="inlineStr">
         <is>
-          <t>§10.4</t>
+          <t>§8.4</t>
         </is>
       </c>
       <c r="L132" t="inlineStr">
         <is>
-          <t>Existing shop stock inspected 2026-09-16 and appears usable.</t>
+          <t>Use only a trace film on dressed ABS-on-ABS sliding interfaces.</t>
         </is>
       </c>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>SHP-017</t>
+          <t>SHP-016</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
@@ -7637,22 +7639,17 @@
       </c>
       <c r="D133" t="inlineStr">
         <is>
-          <t>1/2" Forstner bit, standard-point smooth-finish</t>
+          <t>White lithium grease, NLGI #2</t>
         </is>
       </c>
       <c r="E133" t="inlineStr">
         <is>
-          <t>Spherical-washer counterbores</t>
+          <t>Light grease for mirror-cell spherical washer interfaces</t>
         </is>
       </c>
       <c r="F133" t="inlineStr">
         <is>
-          <t>McMaster</t>
-        </is>
-      </c>
-      <c r="G133" t="inlineStr">
-        <is>
-          <t>2890A56</t>
+          <t>Lucas Oil Products</t>
         </is>
       </c>
       <c r="H133" t="n">
@@ -7675,14 +7672,14 @@
       </c>
       <c r="L133" t="inlineStr">
         <is>
-          <t>Use in drill press for shallow close-fit spherical-washer sockets; test in scrap Baltic birch before cutting final plate.</t>
+          <t>Existing shop stock inspected 2026-09-16 and appears usable.</t>
         </is>
       </c>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>SHP-018</t>
+          <t>SHP-017</t>
         </is>
       </c>
       <c r="B134" t="inlineStr">
@@ -7695,12 +7692,12 @@
       </c>
       <c r="D134" t="inlineStr">
         <is>
-          <t>5/8" Forstner bit, standard-point smooth-finish</t>
+          <t>1/2" Forstner bit, standard-point smooth-finish</t>
         </is>
       </c>
       <c r="E134" t="inlineStr">
         <is>
-          <t>Spring-seat washer counterbores</t>
+          <t>Spherical-washer counterbores</t>
         </is>
       </c>
       <c r="F134" t="inlineStr">
@@ -7710,7 +7707,7 @@
       </c>
       <c r="G134" t="inlineStr">
         <is>
-          <t>2890A58</t>
+          <t>2890A56</t>
         </is>
       </c>
       <c r="H134" t="n">
@@ -7728,19 +7725,19 @@
       </c>
       <c r="K134" t="inlineStr">
         <is>
-          <t>§10.3</t>
+          <t>§10.4</t>
         </is>
       </c>
       <c r="L134" t="inlineStr">
         <is>
-          <t>Use in drill press for shallow spring-seat-washer registration counterbores; test depth/fit in scrap first.</t>
+          <t>Use in drill press for shallow close-fit spherical-washer sockets; test in scrap Baltic birch before cutting final plate.</t>
         </is>
       </c>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>SHP-019</t>
+          <t>SHP-018</t>
         </is>
       </c>
       <c r="B135" t="inlineStr">
@@ -7753,12 +7750,12 @@
       </c>
       <c r="D135" t="inlineStr">
         <is>
-          <t>M4 × 0.7 high-speed-steel plug-chamfer hex-bit tap</t>
+          <t>5/8" Forstner bit, standard-point smooth-finish</t>
         </is>
       </c>
       <c r="E135" t="inlineStr">
         <is>
-          <t>Tap CAMVATE quick-release plate mounting holes</t>
+          <t>Spring-seat washer counterbores</t>
         </is>
       </c>
       <c r="F135" t="inlineStr">
@@ -7768,7 +7765,7 @@
       </c>
       <c r="G135" t="inlineStr">
         <is>
-          <t>1021N23</t>
+          <t>2890A58</t>
         </is>
       </c>
       <c r="H135" t="n">
@@ -7786,19 +7783,19 @@
       </c>
       <c r="K135" t="inlineStr">
         <is>
-          <t>§10.9</t>
+          <t>§10.3</t>
         </is>
       </c>
       <c r="L135" t="inlineStr">
         <is>
-          <t>Use with 3.3 mm tap drill; exact hole locations await measurement of the delivered plate.</t>
+          <t>Use in drill press for shallow spring-seat-washer registration counterbores; test depth/fit in scrap first.</t>
         </is>
       </c>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>SHP-020</t>
+          <t>SHP-019</t>
         </is>
       </c>
       <c r="B136" t="inlineStr">
@@ -7811,12 +7808,12 @@
       </c>
       <c r="D136" t="inlineStr">
         <is>
-          <t>3.3 mm black-oxide HSS jobber-length drill bit</t>
+          <t>M4 × 0.7 high-speed-steel plug-chamfer hex-bit tap</t>
         </is>
       </c>
       <c r="E136" t="inlineStr">
         <is>
-          <t>M4 × 0.7 tap drill for CAMVATE quick-release plate; M3 heatsink clearance holes</t>
+          <t>Tap CAMVATE quick-release plate mounting holes</t>
         </is>
       </c>
       <c r="F136" t="inlineStr">
@@ -7826,7 +7823,7 @@
       </c>
       <c r="G136" t="inlineStr">
         <is>
-          <t>2958A64</t>
+          <t>1021N23</t>
         </is>
       </c>
       <c r="H136" t="n">
@@ -7844,19 +7841,19 @@
       </c>
       <c r="K136" t="inlineStr">
         <is>
-          <t>§§6.4, 10.9</t>
+          <t>§10.9</t>
         </is>
       </c>
       <c r="L136" t="inlineStr">
         <is>
-          <t>Standard 3.3 mm tap-drill size for M4 × 0.7. Also drills the Ø3.3 M3 clearance holes in the heatsink base (§6.4).</t>
+          <t>Use with 3.3 mm tap drill; exact hole locations await measurement of the delivered plate.</t>
         </is>
       </c>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>SHP-021</t>
+          <t>SHP-020</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
@@ -7869,12 +7866,12 @@
       </c>
       <c r="D137" t="inlineStr">
         <is>
-          <t>Loctite 243 medium-strength removable threadlocker, 0.34 fl. oz.</t>
+          <t>3.3 mm black-oxide HSS jobber-length drill bit</t>
         </is>
       </c>
       <c r="E137" t="inlineStr">
         <is>
-          <t>Removable thread retention for quick-release plate mounting screws</t>
+          <t>M4 × 0.7 tap drill for CAMVATE quick-release plate; M3 heatsink clearance holes</t>
         </is>
       </c>
       <c r="F137" t="inlineStr">
@@ -7884,7 +7881,7 @@
       </c>
       <c r="G137" t="inlineStr">
         <is>
-          <t>91458A115</t>
+          <t>2958A64</t>
         </is>
       </c>
       <c r="H137" t="n">
@@ -7902,19 +7899,19 @@
       </c>
       <c r="K137" t="inlineStr">
         <is>
-          <t>§10.9</t>
+          <t>§§6.4, 10.9</t>
         </is>
       </c>
       <c r="L137" t="inlineStr">
         <is>
-          <t>Apply only after fit and screw length are validated; preferred over high-strength Loctite 271 for this serviceable joint.</t>
+          <t>Standard 3.3 mm tap-drill size for M4 × 0.7. Also drills the Ø3.3 M3 clearance holes in the heatsink base (§6.4).</t>
         </is>
       </c>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>SHP-022</t>
+          <t>SHP-021</t>
         </is>
       </c>
       <c r="B138" t="inlineStr">
@@ -7927,22 +7924,22 @@
       </c>
       <c r="D138" t="inlineStr">
         <is>
-          <t>Rosco Photofoil matte black aluminum wrap, 12"x10'</t>
+          <t>Loctite 243 medium-strength removable threadlocker, 0.34 fl. oz.</t>
         </is>
       </c>
       <c r="E138" t="inlineStr">
         <is>
-          <t>Opaque masking / thin-sheet cutoff experiments</t>
+          <t>Removable thread retention for quick-release plate mounting screws</t>
         </is>
       </c>
       <c r="F138" t="inlineStr">
         <is>
-          <t>Fullcompass</t>
+          <t>McMaster</t>
         </is>
       </c>
       <c r="G138" t="inlineStr">
         <is>
-          <t>01001-1210</t>
+          <t>91458A115</t>
         </is>
       </c>
       <c r="H138" t="n">
@@ -7950,7 +7947,7 @@
       </c>
       <c r="I138" t="inlineStr">
         <is>
-          <t>pack</t>
+          <t>each</t>
         </is>
       </c>
       <c r="J138" t="inlineStr">
@@ -7960,19 +7957,19 @@
       </c>
       <c r="K138" t="inlineStr">
         <is>
-          <t>§§8, 8.7</t>
+          <t>§10.9</t>
         </is>
       </c>
       <c r="L138" t="inlineStr">
         <is>
-          <t>Retained as general shop stock for opaque masking and thin-sheet cutoff experiments.</t>
+          <t>Apply only after fit and screw length are validated; preferred over high-strength Loctite 271 for this serviceable joint.</t>
         </is>
       </c>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>SHP-023</t>
+          <t>SHP-022</t>
         </is>
       </c>
       <c r="B139" t="inlineStr">
@@ -7985,22 +7982,22 @@
       </c>
       <c r="D139" t="inlineStr">
         <is>
-          <t>M3 × 0.5 high-speed-steel plug-chamfer tap, 5/8" thread length</t>
+          <t>Rosco Photofoil matte black aluminum wrap, 12"x10'</t>
         </is>
       </c>
       <c r="E139" t="inlineStr">
         <is>
-          <t>Tap through M3 heatsink-screw holes in SM1CP2M cap</t>
+          <t>Opaque masking / thin-sheet cutoff experiments</t>
         </is>
       </c>
       <c r="F139" t="inlineStr">
         <is>
-          <t>McMaster</t>
+          <t>Fullcompass</t>
         </is>
       </c>
       <c r="G139" t="inlineStr">
         <is>
-          <t>8305A32</t>
+          <t>01001-1210</t>
         </is>
       </c>
       <c r="H139" t="n">
@@ -8008,29 +8005,29 @@
       </c>
       <c r="I139" t="inlineStr">
         <is>
-          <t>each</t>
+          <t>pack</t>
         </is>
       </c>
       <c r="J139" t="inlineStr">
         <is>
-          <t>To procure</t>
+          <t>In hand</t>
         </is>
       </c>
       <c r="K139" t="inlineStr">
         <is>
-          <t>§6.4</t>
+          <t>§§8, 8.7</t>
         </is>
       </c>
       <c r="L139" t="inlineStr">
         <is>
-          <t>All holes are through holes, so a plug chamfer is enough; no bottoming tap needed. Use with the 2.5 mm tap drill (SHP-025). Confirm no M3 tap already in shop stock.</t>
+          <t>Retained as general shop stock for opaque masking and thin-sheet cutoff experiments.</t>
         </is>
       </c>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>SHP-025</t>
+          <t>SHP-023</t>
         </is>
       </c>
       <c r="B140" t="inlineStr">
@@ -8043,12 +8040,12 @@
       </c>
       <c r="D140" t="inlineStr">
         <is>
-          <t>2.5 mm TiN-coated HSS short-length drill bit, 43 mm overall</t>
+          <t>M3 × 0.5 high-speed-steel plug-chamfer tap, 5/8" thread length</t>
         </is>
       </c>
       <c r="E140" t="inlineStr">
         <is>
-          <t>M3 tap drill for through holes in SM1CP2M cap</t>
+          <t>Tap through M3 heatsink-screw holes in SM1CP2M cap</t>
         </is>
       </c>
       <c r="F140" t="inlineStr">
@@ -8058,7 +8055,7 @@
       </c>
       <c r="G140" t="inlineStr">
         <is>
-          <t>2979N15</t>
+          <t>8305A32</t>
         </is>
       </c>
       <c r="H140" t="n">
@@ -8081,71 +8078,129 @@
       </c>
       <c r="L140" t="inlineStr">
         <is>
-          <t>Short-length stub drill for rigid drilling in the thin cap; same series as the 1.6 mm drill SHP-006.</t>
+          <t>All holes are through holes, so a plug chamfer is enough; no bottoming tap needed. Use with the 2.5 mm tap drill (SHP-025). Confirm no M3 tap already in shop stock.</t>
         </is>
       </c>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
+          <t>SHP-025</t>
+        </is>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>Shop supplies</t>
+        </is>
+      </c>
+      <c r="C141" t="n">
+        <v>1</v>
+      </c>
+      <c r="D141" t="inlineStr">
+        <is>
+          <t>2.5 mm TiN-coated HSS short-length drill bit, 43 mm overall</t>
+        </is>
+      </c>
+      <c r="E141" t="inlineStr">
+        <is>
+          <t>M3 tap drill for through holes in SM1CP2M cap</t>
+        </is>
+      </c>
+      <c r="F141" t="inlineStr">
+        <is>
+          <t>McMaster</t>
+        </is>
+      </c>
+      <c r="G141" t="inlineStr">
+        <is>
+          <t>2979N15</t>
+        </is>
+      </c>
+      <c r="H141" t="n">
+        <v>1</v>
+      </c>
+      <c r="I141" t="inlineStr">
+        <is>
+          <t>each</t>
+        </is>
+      </c>
+      <c r="J141" t="inlineStr">
+        <is>
+          <t>To procure</t>
+        </is>
+      </c>
+      <c r="K141" t="inlineStr">
+        <is>
+          <t>§6.4</t>
+        </is>
+      </c>
+      <c r="L141" t="inlineStr">
+        <is>
+          <t>Short-length stub drill for rigid drilling in the thin cap; same series as the 1.6 mm drill SHP-006.</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
           <t>SHP-026</t>
         </is>
       </c>
-      <c r="B141" t="inlineStr">
+      <c r="B142" t="inlineStr">
         <is>
           <t>Shop supplies</t>
         </is>
       </c>
-      <c r="C141" t="n">
-        <v>1</v>
-      </c>
-      <c r="D141" t="inlineStr">
+      <c r="C142" t="n">
+        <v>1</v>
+      </c>
+      <c r="D142" t="inlineStr">
         <is>
           <t>2.0 mm uncoated HSS short-length drill bit, 38 mm overall</t>
         </is>
       </c>
-      <c r="E141" t="inlineStr">
+      <c r="E142" t="inlineStr">
         <is>
           <t>Lead holes through SM1CP2M cap and heatsink base</t>
         </is>
       </c>
-      <c r="F141" t="inlineStr">
+      <c r="F142" t="inlineStr">
         <is>
           <t>McMaster</t>
         </is>
       </c>
-      <c r="G141" t="inlineStr">
+      <c r="G142" t="inlineStr">
         <is>
           <t>2979N14</t>
         </is>
       </c>
-      <c r="H141" t="n">
-        <v>1</v>
-      </c>
-      <c r="I141" t="inlineStr">
+      <c r="H142" t="n">
+        <v>1</v>
+      </c>
+      <c r="I142" t="inlineStr">
         <is>
           <t>each</t>
         </is>
       </c>
-      <c r="J141" t="inlineStr">
+      <c r="J142" t="inlineStr">
         <is>
           <t>To procure</t>
         </is>
       </c>
-      <c r="K141" t="inlineStr">
+      <c r="K142" t="inlineStr">
         <is>
           <t>§6.4</t>
         </is>
       </c>
-      <c r="L141" t="inlineStr">
+      <c r="L142" t="inlineStr">
         <is>
           <t>Same series as the 1.6 mm drill SHP-006.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L141"/>
-  <conditionalFormatting sqref="J2:J141">
+  <autoFilter ref="A1:L142"/>
+  <conditionalFormatting sqref="J2:J142">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"In hand"</formula>
     </cfRule>

</xml_diff>

<commit_message>
BOM xslx conversion enhancements
</commit_message>
<xml_diff>
--- a/bom/schlieren-bom.xlsx
+++ b/bom/schlieren-bom.xlsx
@@ -8217,6 +8217,11 @@
       <formula>"CAD open"</formula>
     </cfRule>
   </conditionalFormatting>
+  <dataValidations count="1">
+    <dataValidation sqref="J2:J142" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
+      <formula1>"In hand,On order,To procure,Specified,CAD ready,CAD open"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Sub dowel pins for cut stainless rods
</commit_message>
<xml_diff>
--- a/bom/schlieren-bom.xlsx
+++ b/bom/schlieren-bom.xlsx
@@ -11,7 +11,7 @@
     <sheet name="BOM" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'BOM'!$A$1:$L$142</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'BOM'!$A$1:$L$143</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -837,7 +837,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L142"/>
+  <dimension ref="A1:L143"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -5337,30 +5337,30 @@
         </is>
       </c>
       <c r="C87" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>Stainless steel round rod assortment, 100 mm length</t>
+          <t>Ø3 × 10 mm 18-8 stainless dowel pin, ISO 2338 m6</t>
         </is>
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>Groove rods at the fourth lens-pointer screw; phone rest rod</t>
+          <t>Groove rods at the fourth lens-pointer screw</t>
         </is>
       </c>
       <c r="F87" t="inlineStr">
         <is>
-          <t>Amazon</t>
+          <t>McMaster</t>
         </is>
       </c>
       <c r="G87" t="inlineStr">
         <is>
-          <t>B08N4TSNPW</t>
+          <t>91585A351</t>
         </is>
       </c>
       <c r="H87" t="n">
-        <v>1</v>
+        <v>50</v>
       </c>
       <c r="I87" t="inlineStr">
         <is>
@@ -5369,7 +5369,7 @@
       </c>
       <c r="J87" t="inlineStr">
         <is>
-          <t>In hand</t>
+          <t>To procure</t>
         </is>
       </c>
       <c r="K87" t="inlineStr">
@@ -5379,7 +5379,7 @@
       </c>
       <c r="L87" t="inlineStr">
         <is>
-          <t>Working-stock assortment. Model uses two groove rods of 3 mm diameter × 10 mm and one phone rest rod of 4 mm diameter × 20 mm; confirm the assortment has these diameters.</t>
+          <t>Chamfered ends. Two installed, lying across the rail in the aft collar pad pocket; one pack of 50.</t>
         </is>
       </c>
     </row>
@@ -5698,12 +5698,12 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>MIR-001</t>
+          <t>CAM-017</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>Mirror cell</t>
+          <t>Imager</t>
         </is>
       </c>
       <c r="C94" t="n">
@@ -5711,42 +5711,52 @@
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>Skyoptikst D203F1600 spherical mirror, Ø203 mm, f=1600 mm</t>
+          <t>Ø4 × 20 mm 18-8 stainless dowel pin, ISO 2338 m6</t>
+        </is>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>Phone rest rod</t>
         </is>
       </c>
       <c r="F94" t="inlineStr">
         <is>
-          <t>Amazon</t>
+          <t>McMaster</t>
         </is>
       </c>
       <c r="G94" t="inlineStr">
         <is>
-          <t>B0B5RR41CT</t>
+          <t>91585A457</t>
         </is>
       </c>
       <c r="H94" t="n">
-        <v>1</v>
+        <v>25</v>
       </c>
       <c r="I94" t="inlineStr">
         <is>
-          <t>each</t>
+          <t>pack</t>
         </is>
       </c>
       <c r="J94" t="inlineStr">
         <is>
-          <t>In hand</t>
+          <t>To procure</t>
         </is>
       </c>
       <c r="K94" t="inlineStr">
         <is>
-          <t>§10.5</t>
+          <t>§9.6</t>
+        </is>
+      </c>
+      <c r="L94" t="inlineStr">
+        <is>
+          <t>Chamfered ends. Lies along the rail in the half-round seat of the phone rest arm (CAM-007); one pack of 25.</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>MIR-002</t>
+          <t>MIR-001</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
@@ -5755,16 +5765,11 @@
         </is>
       </c>
       <c r="C95" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>Baltic birch plywood panel 12 × 12 × 1/2 in</t>
-        </is>
-      </c>
-      <c r="E95" t="inlineStr">
-        <is>
-          <t>Base and adjuster plates</t>
+          <t>Skyoptikst D203F1600 spherical mirror, Ø203 mm, f=1600 mm</t>
         </is>
       </c>
       <c r="F95" t="inlineStr">
@@ -5774,15 +5779,15 @@
       </c>
       <c r="G95" t="inlineStr">
         <is>
-          <t>B09D941GXR</t>
+          <t>B0B5RR41CT</t>
         </is>
       </c>
       <c r="H95" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="I95" t="inlineStr">
         <is>
-          <t>pack</t>
+          <t>each</t>
         </is>
       </c>
       <c r="J95" t="inlineStr">
@@ -5792,14 +5797,14 @@
       </c>
       <c r="K95" t="inlineStr">
         <is>
-          <t>§10.1</t>
+          <t>§10.5</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>MIR-003</t>
+          <t>MIR-002</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
@@ -5808,16 +5813,16 @@
         </is>
       </c>
       <c r="C96" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>Baltic birch plywood panel 12 × 12 × 3/4 in</t>
+          <t>Baltic birch plywood panel 12 × 12 × 1/2 in</t>
         </is>
       </c>
       <c r="E96" t="inlineStr">
         <is>
-          <t>Mirror plate</t>
+          <t>Base and adjuster plates</t>
         </is>
       </c>
       <c r="F96" t="inlineStr">
@@ -5827,15 +5832,15 @@
       </c>
       <c r="G96" t="inlineStr">
         <is>
-          <t>B0GL9G45GH</t>
+          <t>B09D941GXR</t>
         </is>
       </c>
       <c r="H96" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="I96" t="inlineStr">
         <is>
-          <t>each</t>
+          <t>pack</t>
         </is>
       </c>
       <c r="J96" t="inlineStr">
@@ -5852,7 +5857,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>MIR-004</t>
+          <t>MIR-003</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
@@ -5861,25 +5866,30 @@
         </is>
       </c>
       <c r="C97" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>1/4-80 TPI Imperial fine adjustment screws, 2.5 in</t>
+          <t>Baltic birch plywood panel 12 × 12 × 3/4 in</t>
+        </is>
+      </c>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>Mirror plate</t>
         </is>
       </c>
       <c r="F97" t="inlineStr">
         <is>
-          <t>Kozak</t>
+          <t>Amazon</t>
         </is>
       </c>
       <c r="G97" t="inlineStr">
         <is>
-          <t>TS250-80-2500</t>
+          <t>B0GL9G45GH</t>
         </is>
       </c>
       <c r="H97" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="I97" t="inlineStr">
         <is>
@@ -5893,14 +5903,14 @@
       </c>
       <c r="K97" t="inlineStr">
         <is>
-          <t>§10.2</t>
+          <t>§10.1</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>MIR-005</t>
+          <t>MIR-004</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
@@ -5913,7 +5923,7 @@
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>Imperial Fine Adjustment Carrier Bushings</t>
+          <t>1/4-80 TPI Imperial fine adjustment screws, 2.5 in</t>
         </is>
       </c>
       <c r="F98" t="inlineStr">
@@ -5923,7 +5933,7 @@
       </c>
       <c r="G98" t="inlineStr">
         <is>
-          <t>TB250-80-625</t>
+          <t>TS250-80-2500</t>
         </is>
       </c>
       <c r="H98" t="n">
@@ -5948,7 +5958,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>MIR-006</t>
+          <t>MIR-005</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
@@ -5961,7 +5971,7 @@
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>Imperial Adjustment Knobs</t>
+          <t>Imperial Fine Adjustment Carrier Bushings</t>
         </is>
       </c>
       <c r="F99" t="inlineStr">
@@ -5971,7 +5981,7 @@
       </c>
       <c r="G99" t="inlineStr">
         <is>
-          <t>KB250-80</t>
+          <t>TB250-80-625</t>
         </is>
       </c>
       <c r="H99" t="n">
@@ -5996,7 +6006,7 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>MIR-007</t>
+          <t>MIR-006</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
@@ -6009,22 +6019,17 @@
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>Leveling Washer, Two Piece, 1/4" Screw Size, Black-Oxide Steel</t>
-        </is>
-      </c>
-      <c r="E100" t="inlineStr">
-        <is>
-          <t>Spherical washers</t>
+          <t>Imperial Adjustment Knobs</t>
         </is>
       </c>
       <c r="F100" t="inlineStr">
         <is>
-          <t>McMaster</t>
+          <t>Kozak</t>
         </is>
       </c>
       <c r="G100" t="inlineStr">
         <is>
-          <t>91131A028</t>
+          <t>KB250-80</t>
         </is>
       </c>
       <c r="H100" t="n">
@@ -6042,14 +6047,14 @@
       </c>
       <c r="K100" t="inlineStr">
         <is>
-          <t>§10.4</t>
+          <t>§10.2</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>MIR-008</t>
+          <t>MIR-007</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
@@ -6062,7 +6067,12 @@
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>Compression Springs, 0.75" Long, 0.5" OD, 0.424" ID</t>
+          <t>Leveling Washer, Two Piece, 1/4" Screw Size, Black-Oxide Steel</t>
+        </is>
+      </c>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>Spherical washers</t>
         </is>
       </c>
       <c r="F101" t="inlineStr">
@@ -6072,15 +6082,15 @@
       </c>
       <c r="G101" t="inlineStr">
         <is>
-          <t>2022N186</t>
+          <t>91131A028</t>
         </is>
       </c>
       <c r="H101" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="I101" t="inlineStr">
         <is>
-          <t>pack</t>
+          <t>each</t>
         </is>
       </c>
       <c r="J101" t="inlineStr">
@@ -6090,14 +6100,14 @@
       </c>
       <c r="K101" t="inlineStr">
         <is>
-          <t>§10.3</t>
+          <t>§10.4</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>MIR-009</t>
+          <t>MIR-008</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
@@ -6106,16 +6116,11 @@
         </is>
       </c>
       <c r="C102" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t>Washer for 3/8" washer, 0.390" ID, 0.028" to 0.036" thick, 18-8 SS</t>
-        </is>
-      </c>
-      <c r="E102" t="inlineStr">
-        <is>
-          <t>Spring seat washers</t>
+          <t>Compression Springs, 0.75" Long, 0.5" OD, 0.424" ID</t>
         </is>
       </c>
       <c r="F102" t="inlineStr">
@@ -6125,11 +6130,11 @@
       </c>
       <c r="G102" t="inlineStr">
         <is>
-          <t>98017A199</t>
+          <t>2022N186</t>
         </is>
       </c>
       <c r="H102" t="n">
-        <v>100</v>
+        <v>5</v>
       </c>
       <c r="I102" t="inlineStr">
         <is>
@@ -6150,7 +6155,7 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>MIR-010</t>
+          <t>MIR-009</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
@@ -6159,16 +6164,16 @@
         </is>
       </c>
       <c r="C103" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>3" Long Corner Bracket, aluminum</t>
+          <t>Washer for 3/8" washer, 0.390" ID, 0.028" to 0.036" thick, 18-8 SS</t>
         </is>
       </c>
       <c r="E103" t="inlineStr">
         <is>
-          <t>Adjuster plate to base plate mounting</t>
+          <t>Spring seat washers</t>
         </is>
       </c>
       <c r="F103" t="inlineStr">
@@ -6178,15 +6183,15 @@
       </c>
       <c r="G103" t="inlineStr">
         <is>
-          <t>8681N11</t>
+          <t>98017A199</t>
         </is>
       </c>
       <c r="H103" t="n">
-        <v>2</v>
+        <v>100</v>
       </c>
       <c r="I103" t="inlineStr">
         <is>
-          <t>each</t>
+          <t>pack</t>
         </is>
       </c>
       <c r="J103" t="inlineStr">
@@ -6196,14 +6201,14 @@
       </c>
       <c r="K103" t="inlineStr">
         <is>
-          <t>§10.7</t>
+          <t>§10.3</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>MIR-011</t>
+          <t>MIR-010</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
@@ -6211,14 +6216,17 @@
           <t>Mirror cell</t>
         </is>
       </c>
+      <c r="C104" t="n">
+        <v>2</v>
+      </c>
       <c r="D104" t="inlineStr">
         <is>
-          <t>5/16" × 1-1/2" hex-drive flat-head screw, 316 SS</t>
+          <t>3" Long Corner Bracket, aluminum</t>
         </is>
       </c>
       <c r="E104" t="inlineStr">
         <is>
-          <t>Existing alternate/fallback bracket screw stock</t>
+          <t>Adjuster plate to base plate mounting</t>
         </is>
       </c>
       <c r="F104" t="inlineStr">
@@ -6228,15 +6236,15 @@
       </c>
       <c r="G104" t="inlineStr">
         <is>
-          <t>90585A587</t>
+          <t>8681N11</t>
         </is>
       </c>
       <c r="H104" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="I104" t="inlineStr">
         <is>
-          <t>pack</t>
+          <t>each</t>
         </is>
       </c>
       <c r="J104" t="inlineStr">
@@ -6247,18 +6255,13 @@
       <c r="K104" t="inlineStr">
         <is>
           <t>§10.7</t>
-        </is>
-      </c>
-      <c r="L104" t="inlineStr">
-        <is>
-          <t>Previously baseline bracket screw; retained as in-hand alternate stock after corner-clearance review.</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>MIR-012</t>
+          <t>MIR-011</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
@@ -6266,17 +6269,14 @@
           <t>Mirror cell</t>
         </is>
       </c>
-      <c r="C105" t="n">
-        <v>8</v>
-      </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>5/16"-18 heavy-profile nylon-insert locknut, 18-8 SS</t>
+          <t>5/16" × 1-1/2" hex-drive flat-head screw, 316 SS</t>
         </is>
       </c>
       <c r="E105" t="inlineStr">
         <is>
-          <t>Adjuster plate to base plate mounting</t>
+          <t>Existing alternate/fallback bracket screw stock</t>
         </is>
       </c>
       <c r="F105" t="inlineStr">
@@ -6286,7 +6286,7 @@
       </c>
       <c r="G105" t="inlineStr">
         <is>
-          <t>90099A030</t>
+          <t>90585A587</t>
         </is>
       </c>
       <c r="H105" t="n">
@@ -6309,14 +6309,14 @@
       </c>
       <c r="L105" t="inlineStr">
         <is>
-          <t>Eight installed, four per bracket; existing stock was confirmed in hand for six, so confirm two more.</t>
+          <t>Previously baseline bracket screw; retained as in-hand alternate stock after corner-clearance review.</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>MIR-013</t>
+          <t>MIR-012</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
@@ -6329,7 +6329,7 @@
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>5/16" SAE washer, 0.344" ID × 0.688" OD, 18-8 SS black oxide</t>
+          <t>5/16"-18 heavy-profile nylon-insert locknut, 18-8 SS</t>
         </is>
       </c>
       <c r="E106" t="inlineStr">
@@ -6344,11 +6344,11 @@
       </c>
       <c r="G106" t="inlineStr">
         <is>
-          <t>96659A134</t>
+          <t>90099A030</t>
         </is>
       </c>
       <c r="H106" t="n">
-        <v>25</v>
+        <v>5</v>
       </c>
       <c r="I106" t="inlineStr">
         <is>
@@ -6367,14 +6367,14 @@
       </c>
       <c r="L106" t="inlineStr">
         <is>
-          <t>Eight installed, one under each bracket locknut.</t>
+          <t>Eight installed, four per bracket; existing stock was confirmed in hand for six, so confirm two more.</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>MIR-015</t>
+          <t>MIR-013</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
@@ -6383,16 +6383,16 @@
         </is>
       </c>
       <c r="C107" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t>1/4"-20 × 1-1/2" flat-head screws</t>
+          <t>5/16" SAE washer, 0.344" ID × 0.688" OD, 18-8 SS black oxide</t>
         </is>
       </c>
       <c r="E107" t="inlineStr">
         <is>
-          <t>Existing spare stock; former C2564 tripod-interface hardware</t>
+          <t>Adjuster plate to base plate mounting</t>
         </is>
       </c>
       <c r="F107" t="inlineStr">
@@ -6402,15 +6402,15 @@
       </c>
       <c r="G107" t="inlineStr">
         <is>
-          <t>94518A525</t>
+          <t>96659A134</t>
         </is>
       </c>
       <c r="H107" t="n">
-        <v>4</v>
+        <v>25</v>
       </c>
       <c r="I107" t="inlineStr">
         <is>
-          <t>each</t>
+          <t>pack</t>
         </is>
       </c>
       <c r="J107" t="inlineStr">
@@ -6418,16 +6418,21 @@
           <t>In hand</t>
         </is>
       </c>
+      <c r="K107" t="inlineStr">
+        <is>
+          <t>§10.7</t>
+        </is>
+      </c>
       <c r="L107" t="inlineStr">
         <is>
-          <t>No longer allocated to the active tripod interface after transition to the CAMVATE 577/501/504 quick-release system; retain as in-hand spare hardware.</t>
+          <t>Eight installed, one under each bracket locknut.</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>MIR-017</t>
+          <t>MIR-015</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
@@ -6440,7 +6445,7 @@
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>1/4"-20 flex-top locknuts</t>
+          <t>1/4"-20 × 1-1/2" flat-head screws</t>
         </is>
       </c>
       <c r="E108" t="inlineStr">
@@ -6455,15 +6460,15 @@
       </c>
       <c r="G108" t="inlineStr">
         <is>
-          <t>91839A123</t>
+          <t>94518A525</t>
         </is>
       </c>
       <c r="H108" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="I108" t="inlineStr">
         <is>
-          <t>pack</t>
+          <t>each</t>
         </is>
       </c>
       <c r="J108" t="inlineStr">
@@ -6480,7 +6485,7 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>MIR-018</t>
+          <t>MIR-017</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
@@ -6493,7 +6498,7 @@
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t>1/4" thin washers</t>
+          <t>1/4"-20 flex-top locknuts</t>
         </is>
       </c>
       <c r="E109" t="inlineStr">
@@ -6508,11 +6513,11 @@
       </c>
       <c r="G109" t="inlineStr">
         <is>
-          <t>98019A255</t>
+          <t>91839A123</t>
         </is>
       </c>
       <c r="H109" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="I109" t="inlineStr">
         <is>
@@ -6533,7 +6538,7 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>MIR-023</t>
+          <t>MIR-018</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
@@ -6546,12 +6551,12 @@
       </c>
       <c r="D110" t="inlineStr">
         <is>
-          <t>M4 × 0.7 × 16 mm 90° flat-head hex-drive screw, 18-8 stainless</t>
+          <t>1/4" thin washers</t>
         </is>
       </c>
       <c r="E110" t="inlineStr">
         <is>
-          <t>Provisional quick-release plate mounting screw; short-length option</t>
+          <t>Existing spare stock; former C2564 tripod-interface hardware</t>
         </is>
       </c>
       <c r="F110" t="inlineStr">
@@ -6561,11 +6566,11 @@
       </c>
       <c r="G110" t="inlineStr">
         <is>
-          <t>92125A194</t>
+          <t>98019A255</t>
         </is>
       </c>
       <c r="H110" t="n">
-        <v>100</v>
+        <v>10</v>
       </c>
       <c r="I110" t="inlineStr">
         <is>
@@ -6577,21 +6582,16 @@
           <t>In hand</t>
         </is>
       </c>
-      <c r="K110" t="inlineStr">
-        <is>
-          <t>§10.9</t>
-        </is>
-      </c>
       <c r="L110" t="inlineStr">
         <is>
-          <t>Order one pack. Four screws are the provisional installed quantity if this length matches the measured CAMVATE plate thickness; otherwise use MIR-024.</t>
+          <t>No longer allocated to the active tripod interface after transition to the CAMVATE 577/501/504 quick-release system; retain as in-hand spare hardware.</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>MIR-024</t>
+          <t>MIR-023</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
@@ -6604,12 +6604,12 @@
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>M4 × 0.7 × 18 mm 90° flat-head hex-drive screw, 18-8 stainless</t>
+          <t>M4 × 0.7 × 16 mm 90° flat-head hex-drive screw, 18-8 stainless</t>
         </is>
       </c>
       <c r="E111" t="inlineStr">
         <is>
-          <t>Provisional quick-release plate mounting screw; long-length option</t>
+          <t>Provisional quick-release plate mounting screw; short-length option</t>
         </is>
       </c>
       <c r="F111" t="inlineStr">
@@ -6619,7 +6619,7 @@
       </c>
       <c r="G111" t="inlineStr">
         <is>
-          <t>92125A196</t>
+          <t>92125A194</t>
         </is>
       </c>
       <c r="H111" t="n">
@@ -6642,14 +6642,14 @@
       </c>
       <c r="L111" t="inlineStr">
         <is>
-          <t>Order one pack. Four screws are the provisional installed quantity if this length matches the measured CAMVATE plate thickness; otherwise use MIR-023.</t>
+          <t>Order one pack. Four screws are the provisional installed quantity if this length matches the measured CAMVATE plate thickness; otherwise use MIR-024.</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>MIR-025</t>
+          <t>MIR-024</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
@@ -6658,34 +6658,34 @@
         </is>
       </c>
       <c r="C112" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D112" t="inlineStr">
         <is>
-          <t>CAMVATE Manfrotto-Type Quick Release Assembly with Sliding Plate Camera Mount</t>
+          <t>M4 × 0.7 × 18 mm 90° flat-head hex-drive screw, 18-8 stainless</t>
         </is>
       </c>
       <c r="E112" t="inlineStr">
         <is>
-          <t>Mirror-cell quick-release / tripod interface</t>
+          <t>Provisional quick-release plate mounting screw; long-length option</t>
         </is>
       </c>
       <c r="F112" t="inlineStr">
         <is>
-          <t>Amazon</t>
+          <t>McMaster</t>
         </is>
       </c>
       <c r="G112" t="inlineStr">
         <is>
-          <t>B0B2WBC921</t>
+          <t>92125A196</t>
         </is>
       </c>
       <c r="H112" t="n">
-        <v>1</v>
+        <v>100</v>
       </c>
       <c r="I112" t="inlineStr">
         <is>
-          <t>each</t>
+          <t>pack</t>
         </is>
       </c>
       <c r="J112" t="inlineStr">
@@ -6700,14 +6700,14 @@
       </c>
       <c r="L112" t="inlineStr">
         <is>
-          <t>Complete 577/501/504-compatible quick-release assembly with removable sliding plate and receiver. Exact removable-plate hole pattern and final M4 screw length to be verified on arrival.</t>
+          <t>Order one pack. Four screws are the provisional installed quantity if this length matches the measured CAMVATE plate thickness; otherwise use MIR-023.</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>MIR-019</t>
+          <t>MIR-025</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
@@ -6720,22 +6720,22 @@
       </c>
       <c r="D113" t="inlineStr">
         <is>
-          <t>DOWSIL 737 clear silicone, 3 fl. oz.</t>
+          <t>CAMVATE Manfrotto-Type Quick Release Assembly with Sliding Plate Camera Mount</t>
         </is>
       </c>
       <c r="E113" t="inlineStr">
         <is>
-          <t>Mirror mounting</t>
+          <t>Mirror-cell quick-release / tripod interface</t>
         </is>
       </c>
       <c r="F113" t="inlineStr">
         <is>
-          <t>McMaster</t>
+          <t>Amazon</t>
         </is>
       </c>
       <c r="G113" t="inlineStr">
         <is>
-          <t>7587A25</t>
+          <t>B0B2WBC921</t>
         </is>
       </c>
       <c r="H113" t="n">
@@ -6753,14 +6753,19 @@
       </c>
       <c r="K113" t="inlineStr">
         <is>
-          <t>§10.5</t>
+          <t>§10.9</t>
+        </is>
+      </c>
+      <c r="L113" t="inlineStr">
+        <is>
+          <t>Complete 577/501/504-compatible quick-release assembly with removable sliding plate and receiver. Exact removable-plate hole pattern and final M4 screw length to be verified on arrival.</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>MIR-020</t>
+          <t>MIR-019</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
@@ -6773,12 +6778,12 @@
       </c>
       <c r="D114" t="inlineStr">
         <is>
-          <t>Adhesive backed F1 felt</t>
+          <t>DOWSIL 737 clear silicone, 3 fl. oz.</t>
         </is>
       </c>
       <c r="E114" t="inlineStr">
         <is>
-          <t>Safety retainer padding</t>
+          <t>Mirror mounting</t>
         </is>
       </c>
       <c r="F114" t="inlineStr">
@@ -6788,7 +6793,7 @@
       </c>
       <c r="G114" t="inlineStr">
         <is>
-          <t>8334K15</t>
+          <t>7587A25</t>
         </is>
       </c>
       <c r="H114" t="n">
@@ -6796,7 +6801,7 @@
       </c>
       <c r="I114" t="inlineStr">
         <is>
-          <t>sheet</t>
+          <t>each</t>
         </is>
       </c>
       <c r="J114" t="inlineStr">
@@ -6806,14 +6811,14 @@
       </c>
       <c r="K114" t="inlineStr">
         <is>
-          <t>§10.8</t>
+          <t>§10.5</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>MIR-021</t>
+          <t>MIR-020</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
@@ -6822,16 +6827,39 @@
         </is>
       </c>
       <c r="C115" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t>ABS printed front safety retainers</t>
+          <t>Adhesive backed F1 felt</t>
+        </is>
+      </c>
+      <c r="E115" t="inlineStr">
+        <is>
+          <t>Safety retainer padding</t>
+        </is>
+      </c>
+      <c r="F115" t="inlineStr">
+        <is>
+          <t>McMaster</t>
+        </is>
+      </c>
+      <c r="G115" t="inlineStr">
+        <is>
+          <t>8334K15</t>
+        </is>
+      </c>
+      <c r="H115" t="n">
+        <v>1</v>
+      </c>
+      <c r="I115" t="inlineStr">
+        <is>
+          <t>sheet</t>
         </is>
       </c>
       <c r="J115" t="inlineStr">
         <is>
-          <t>CAD open</t>
+          <t>In hand</t>
         </is>
       </c>
       <c r="K115" t="inlineStr">
@@ -6843,7 +6871,7 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>MIR-022</t>
+          <t>MIR-021</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
@@ -6851,54 +6879,29 @@
           <t>Mirror cell</t>
         </is>
       </c>
+      <c r="C116" t="n">
+        <v>3</v>
+      </c>
       <c r="D116" t="inlineStr">
         <is>
-          <t>5/16"-18 × 1-3/8" hex-drive flat-head screw, 316 SS</t>
-        </is>
-      </c>
-      <c r="E116" t="inlineStr">
-        <is>
-          <t>Existing alternate bracket screw stock</t>
-        </is>
-      </c>
-      <c r="F116" t="inlineStr">
-        <is>
-          <t>McMaster</t>
-        </is>
-      </c>
-      <c r="G116" t="inlineStr">
-        <is>
-          <t>90585A997</t>
-        </is>
-      </c>
-      <c r="H116" t="n">
-        <v>5</v>
-      </c>
-      <c r="I116" t="inlineStr">
-        <is>
-          <t>pack</t>
+          <t>ABS printed front safety retainers</t>
         </is>
       </c>
       <c r="J116" t="inlineStr">
         <is>
-          <t>In hand</t>
+          <t>CAD open</t>
         </is>
       </c>
       <c r="K116" t="inlineStr">
         <is>
-          <t>§10.7</t>
-        </is>
-      </c>
-      <c r="L116" t="inlineStr">
-        <is>
-          <t>Former baseline bracket screw; retained as in-hand alternate stock after the change to button-head screws (MIR-026).</t>
+          <t>§10.8</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>MIR-026</t>
+          <t>MIR-022</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
@@ -6906,17 +6909,14 @@
           <t>Mirror cell</t>
         </is>
       </c>
-      <c r="C117" t="n">
-        <v>8</v>
-      </c>
       <c r="D117" t="inlineStr">
         <is>
-          <t>5/16"-18 × 1-3/8" 316 stainless button-head hex-drive screw</t>
+          <t>5/16"-18 × 1-3/8" hex-drive flat-head screw, 316 SS</t>
         </is>
       </c>
       <c r="E117" t="inlineStr">
         <is>
-          <t>Bracket screws, heads on the bracket</t>
+          <t>Existing alternate bracket screw stock</t>
         </is>
       </c>
       <c r="F117" t="inlineStr">
@@ -6926,7 +6926,7 @@
       </c>
       <c r="G117" t="inlineStr">
         <is>
-          <t>98164A527</t>
+          <t>90585A997</t>
         </is>
       </c>
       <c r="H117" t="n">
@@ -6939,7 +6939,7 @@
       </c>
       <c r="J117" t="inlineStr">
         <is>
-          <t>To procure</t>
+          <t>In hand</t>
         </is>
       </c>
       <c r="K117" t="inlineStr">
@@ -6949,27 +6949,32 @@
       </c>
       <c r="L117" t="inlineStr">
         <is>
-          <t>Four per bracket, two through the plate and two through the base; eight installed, so order two 5-packs (two spare). 3/16 in hex drive; head Ø0.547 in × 0.166 in. Pushed through from the bracket side, with MIR-013 washers and MIR-012 locknuts behind the plywood. Thread projects about 0.12 in past the locknut.</t>
+          <t>Former baseline bracket screw; retained as in-hand alternate stock after the change to button-head screws (MIR-026).</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>SHP-001</t>
+          <t>MIR-026</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>Shop supplies</t>
+          <t>Mirror cell</t>
         </is>
       </c>
       <c r="C118" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="D118" t="inlineStr">
         <is>
-          <t>Loctite 271 threadlocker, .34 fl. oz.</t>
+          <t>5/16"-18 × 1-3/8" 316 stainless button-head hex-drive screw</t>
+        </is>
+      </c>
+      <c r="E118" t="inlineStr">
+        <is>
+          <t>Bracket screws, heads on the bracket</t>
         </is>
       </c>
       <c r="F118" t="inlineStr">
@@ -6979,32 +6984,37 @@
       </c>
       <c r="G118" t="inlineStr">
         <is>
-          <t>91458A160</t>
+          <t>98164A527</t>
         </is>
       </c>
       <c r="H118" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="I118" t="inlineStr">
         <is>
-          <t>each</t>
+          <t>pack</t>
         </is>
       </c>
       <c r="J118" t="inlineStr">
         <is>
-          <t>In hand</t>
+          <t>To procure</t>
         </is>
       </c>
       <c r="K118" t="inlineStr">
         <is>
-          <t>§9.5</t>
+          <t>§10.7</t>
+        </is>
+      </c>
+      <c r="L118" t="inlineStr">
+        <is>
+          <t>Four per bracket, two through the plate and two through the base; eight installed, so order two 5-packs (two spare). 3/16 in hex drive; head Ø0.547 in × 0.166 in. Pushed through from the bracket side, with MIR-013 washers and MIR-012 locknuts behind the plywood. Thread projects about 0.12 in past the locknut.</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>SHP-002</t>
+          <t>SHP-001</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
@@ -7017,7 +7027,7 @@
       </c>
       <c r="D119" t="inlineStr">
         <is>
-          <t>Heat-set installation tip</t>
+          <t>Loctite 271 threadlocker, .34 fl. oz.</t>
         </is>
       </c>
       <c r="F119" t="inlineStr">
@@ -7027,7 +7037,7 @@
       </c>
       <c r="G119" t="inlineStr">
         <is>
-          <t>92160A327</t>
+          <t>91458A160</t>
         </is>
       </c>
       <c r="H119" t="n">
@@ -7052,7 +7062,7 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>SHP-003</t>
+          <t>SHP-002</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
@@ -7065,17 +7075,17 @@
       </c>
       <c r="D120" t="inlineStr">
         <is>
-          <t>Optical spanner wrench</t>
+          <t>Heat-set installation tip</t>
         </is>
       </c>
       <c r="F120" t="inlineStr">
         <is>
-          <t>Amazon</t>
+          <t>McMaster</t>
         </is>
       </c>
       <c r="G120" t="inlineStr">
         <is>
-          <t>B0CKSL364Q</t>
+          <t>92160A327</t>
         </is>
       </c>
       <c r="H120" t="n">
@@ -7089,13 +7099,18 @@
       <c r="J120" t="inlineStr">
         <is>
           <t>In hand</t>
+        </is>
+      </c>
+      <c r="K120" t="inlineStr">
+        <is>
+          <t>§9.5</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>SHP-004</t>
+          <t>SHP-003</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
@@ -7108,12 +7123,7 @@
       </c>
       <c r="D121" t="inlineStr">
         <is>
-          <t>Metric feeler gauge set</t>
-        </is>
-      </c>
-      <c r="E121" t="inlineStr">
-        <is>
-          <t>Source-slit blade spacing</t>
+          <t>Optical spanner wrench</t>
         </is>
       </c>
       <c r="F121" t="inlineStr">
@@ -7123,7 +7133,7 @@
       </c>
       <c r="G121" t="inlineStr">
         <is>
-          <t>B07XPD9L1C</t>
+          <t>B0CKSL364Q</t>
         </is>
       </c>
       <c r="H121" t="n">
@@ -7137,18 +7147,13 @@
       <c r="J121" t="inlineStr">
         <is>
           <t>In hand</t>
-        </is>
-      </c>
-      <c r="K121" t="inlineStr">
-        <is>
-          <t>§7.4</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>SHP-005</t>
+          <t>SHP-004</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
@@ -7161,22 +7166,22 @@
       </c>
       <c r="D122" t="inlineStr">
         <is>
-          <t>M2 tap</t>
+          <t>Metric feeler gauge set</t>
         </is>
       </c>
       <c r="E122" t="inlineStr">
         <is>
-          <t>LED board mounting into SM1CP2M cap</t>
+          <t>Source-slit blade spacing</t>
         </is>
       </c>
       <c r="F122" t="inlineStr">
         <is>
-          <t>McMaster</t>
+          <t>Amazon</t>
         </is>
       </c>
       <c r="G122" t="inlineStr">
         <is>
-          <t>8305A78</t>
+          <t>B07XPD9L1C</t>
         </is>
       </c>
       <c r="H122" t="n">
@@ -7194,19 +7199,14 @@
       </c>
       <c r="K122" t="inlineStr">
         <is>
-          <t>§6.4</t>
-        </is>
-      </c>
-      <c r="L122" t="inlineStr">
-        <is>
-          <t>Plug chamfer; sufficient for the through M2 holes.</t>
+          <t>§7.4</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>SHP-006</t>
+          <t>SHP-005</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
@@ -7219,12 +7219,12 @@
       </c>
       <c r="D123" t="inlineStr">
         <is>
-          <t>M2 tap drill, 1.6mm</t>
+          <t>M2 tap</t>
         </is>
       </c>
       <c r="E123" t="inlineStr">
         <is>
-          <t>LED mounting</t>
+          <t>LED board mounting into SM1CP2M cap</t>
         </is>
       </c>
       <c r="F123" t="inlineStr">
@@ -7234,7 +7234,7 @@
       </c>
       <c r="G123" t="inlineStr">
         <is>
-          <t>2979N13</t>
+          <t>8305A78</t>
         </is>
       </c>
       <c r="H123" t="n">
@@ -7253,13 +7253,18 @@
       <c r="K123" t="inlineStr">
         <is>
           <t>§6.4</t>
+        </is>
+      </c>
+      <c r="L123" t="inlineStr">
+        <is>
+          <t>Plug chamfer; sufficient for the through M2 holes.</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>SHP-007</t>
+          <t>SHP-006</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
@@ -7267,14 +7272,35 @@
           <t>Shop supplies</t>
         </is>
       </c>
+      <c r="C124" t="n">
+        <v>1</v>
+      </c>
       <c r="D124" t="inlineStr">
         <is>
-          <t>18 AWG wire</t>
+          <t>M2 tap drill, 1.6mm</t>
         </is>
       </c>
       <c r="E124" t="inlineStr">
         <is>
-          <t>LED wiring</t>
+          <t>LED mounting</t>
+        </is>
+      </c>
+      <c r="F124" t="inlineStr">
+        <is>
+          <t>McMaster</t>
+        </is>
+      </c>
+      <c r="G124" t="inlineStr">
+        <is>
+          <t>2979N13</t>
+        </is>
+      </c>
+      <c r="H124" t="n">
+        <v>1</v>
+      </c>
+      <c r="I124" t="inlineStr">
+        <is>
+          <t>each</t>
         </is>
       </c>
       <c r="J124" t="inlineStr">
@@ -7284,14 +7310,14 @@
       </c>
       <c r="K124" t="inlineStr">
         <is>
-          <t>§6.5</t>
+          <t>§6.4</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>SHP-008</t>
+          <t>SHP-007</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
@@ -7301,7 +7327,7 @@
       </c>
       <c r="D125" t="inlineStr">
         <is>
-          <t>Heat-shrink tubing</t>
+          <t>18 AWG wire</t>
         </is>
       </c>
       <c r="E125" t="inlineStr">
@@ -7312,13 +7338,18 @@
       <c r="J125" t="inlineStr">
         <is>
           <t>In hand</t>
+        </is>
+      </c>
+      <c r="K125" t="inlineStr">
+        <is>
+          <t>§6.5</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>SHP-009</t>
+          <t>SHP-008</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
@@ -7328,12 +7359,12 @@
       </c>
       <c r="D126" t="inlineStr">
         <is>
-          <t>USB-C chargers/cables</t>
+          <t>Heat-shrink tubing</t>
         </is>
       </c>
       <c r="E126" t="inlineStr">
         <is>
-          <t>DP100 power</t>
+          <t>LED wiring</t>
         </is>
       </c>
       <c r="J126" t="inlineStr">
@@ -7345,7 +7376,7 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>SHP-010</t>
+          <t>SHP-009</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
@@ -7355,29 +7386,24 @@
       </c>
       <c r="D127" t="inlineStr">
         <is>
-          <t>Thermal compound</t>
+          <t>USB-C chargers/cables</t>
         </is>
       </c>
       <c r="E127" t="inlineStr">
         <is>
-          <t>LED heatsink interfaces</t>
+          <t>DP100 power</t>
         </is>
       </c>
       <c r="J127" t="inlineStr">
         <is>
           <t>In hand</t>
-        </is>
-      </c>
-      <c r="K127" t="inlineStr">
-        <is>
-          <t>§6.4</t>
         </is>
       </c>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>SHP-011</t>
+          <t>SHP-010</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
@@ -7385,35 +7411,14 @@
           <t>Shop supplies</t>
         </is>
       </c>
-      <c r="C128" t="n">
-        <v>1</v>
-      </c>
       <c r="D128" t="inlineStr">
         <is>
-          <t>Loctite 4061 cyanoacrylate adhesive, 0.7 fl. oz., low viscosity (~20 cP)</t>
+          <t>Thermal compound</t>
         </is>
       </c>
       <c r="E128" t="inlineStr">
         <is>
-          <t>Plywood fiber conditioning and localized tack bonds</t>
-        </is>
-      </c>
-      <c r="F128" t="inlineStr">
-        <is>
-          <t>McMaster</t>
-        </is>
-      </c>
-      <c r="G128" t="inlineStr">
-        <is>
-          <t>1818A45</t>
-        </is>
-      </c>
-      <c r="H128" t="n">
-        <v>1</v>
-      </c>
-      <c r="I128" t="inlineStr">
-        <is>
-          <t>each</t>
+          <t>LED heatsink interfaces</t>
         </is>
       </c>
       <c r="J128" t="inlineStr">
@@ -7423,19 +7428,14 @@
       </c>
       <c r="K128" t="inlineStr">
         <is>
-          <t>§§6.2, 7, 8.4, 10.4</t>
-        </is>
-      </c>
-      <c r="L128" t="inlineStr">
-        <is>
-          <t>Use sparingly: wick into Baltic-birch fibers for spherical-washer sockets; use needle-sized localized drops for ABS/metal calibration tacks and captive screw retention. No accelerator required.</t>
+          <t>§6.4</t>
         </is>
       </c>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>SHP-012</t>
+          <t>SHP-011</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
@@ -7448,22 +7448,22 @@
       </c>
       <c r="D129" t="inlineStr">
         <is>
-          <t>UHMW Sheet 1/8" x 12" x 12"</t>
+          <t>Loctite 4061 cyanoacrylate adhesive, 0.7 fl. oz., low viscosity (~20 cP)</t>
         </is>
       </c>
       <c r="E129" t="inlineStr">
         <is>
-          <t>Mirror mount releasing assembly surface</t>
+          <t>Plywood fiber conditioning and localized tack bonds</t>
         </is>
       </c>
       <c r="F129" t="inlineStr">
         <is>
-          <t>US Plastics</t>
+          <t>McMaster</t>
         </is>
       </c>
       <c r="G129" t="inlineStr">
         <is>
-          <t>46489</t>
+          <t>1818A45</t>
         </is>
       </c>
       <c r="H129" t="n">
@@ -7481,14 +7481,19 @@
       </c>
       <c r="K129" t="inlineStr">
         <is>
-          <t>§10.6</t>
+          <t>§§6.2, 7, 8.4, 10.4</t>
+        </is>
+      </c>
+      <c r="L129" t="inlineStr">
+        <is>
+          <t>Use sparingly: wick into Baltic-birch fibers for spherical-washer sockets; use needle-sized localized drops for ABS/metal calibration tacks and captive screw retention. No accelerator required.</t>
         </is>
       </c>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>SHP-013</t>
+          <t>SHP-012</t>
         </is>
       </c>
       <c r="B130" t="inlineStr">
@@ -7496,26 +7501,52 @@
           <t>Shop supplies</t>
         </is>
       </c>
+      <c r="C130" t="n">
+        <v>1</v>
+      </c>
       <c r="D130" t="inlineStr">
         <is>
-          <t>Soldering tools / supplies</t>
+          <t>UHMW Sheet 1/8" x 12" x 12"</t>
         </is>
       </c>
       <c r="E130" t="inlineStr">
         <is>
-          <t>LED wiring</t>
+          <t>Mirror mount releasing assembly surface</t>
+        </is>
+      </c>
+      <c r="F130" t="inlineStr">
+        <is>
+          <t>US Plastics</t>
+        </is>
+      </c>
+      <c r="G130" t="inlineStr">
+        <is>
+          <t>46489</t>
+        </is>
+      </c>
+      <c r="H130" t="n">
+        <v>1</v>
+      </c>
+      <c r="I130" t="inlineStr">
+        <is>
+          <t>each</t>
         </is>
       </c>
       <c r="J130" t="inlineStr">
         <is>
           <t>In hand</t>
+        </is>
+      </c>
+      <c r="K130" t="inlineStr">
+        <is>
+          <t>§10.6</t>
         </is>
       </c>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>SHP-014</t>
+          <t>SHP-013</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
@@ -7523,52 +7554,26 @@
           <t>Shop supplies</t>
         </is>
       </c>
-      <c r="C131" t="n">
-        <v>1</v>
-      </c>
       <c r="D131" t="inlineStr">
         <is>
-          <t>West System G/Flex 650 Epoxy Adhesive, 2 x 4 oz</t>
+          <t>Soldering tools / supplies</t>
         </is>
       </c>
       <c r="E131" t="inlineStr">
         <is>
-          <t>Mirror cell adjuster sleeves, spring seat washer tack</t>
-        </is>
-      </c>
-      <c r="F131" t="inlineStr">
-        <is>
-          <t>Amazon</t>
-        </is>
-      </c>
-      <c r="G131" t="inlineStr">
-        <is>
-          <t>B002IZFPQE</t>
-        </is>
-      </c>
-      <c r="H131" t="n">
-        <v>1</v>
-      </c>
-      <c r="I131" t="inlineStr">
-        <is>
-          <t>each</t>
+          <t>LED wiring</t>
         </is>
       </c>
       <c r="J131" t="inlineStr">
         <is>
           <t>In hand</t>
-        </is>
-      </c>
-      <c r="K131" t="inlineStr">
-        <is>
-          <t>§10.2</t>
         </is>
       </c>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>SHP-015</t>
+          <t>SHP-014</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
@@ -7581,22 +7586,22 @@
       </c>
       <c r="D132" t="inlineStr">
         <is>
-          <t>Silicone grease, clear, NLGI 1</t>
+          <t>West System G/Flex 650 Epoxy Adhesive, 2 x 4 oz</t>
         </is>
       </c>
       <c r="E132" t="inlineStr">
         <is>
-          <t>ABS carriage sliding-interface lubricant</t>
+          <t>Mirror cell adjuster sleeves, spring seat washer tack</t>
         </is>
       </c>
       <c r="F132" t="inlineStr">
         <is>
-          <t>McMaster</t>
+          <t>Amazon</t>
         </is>
       </c>
       <c r="G132" t="inlineStr">
         <is>
-          <t>1418K51</t>
+          <t>B002IZFPQE</t>
         </is>
       </c>
       <c r="H132" t="n">
@@ -7614,19 +7619,14 @@
       </c>
       <c r="K132" t="inlineStr">
         <is>
-          <t>§8.4</t>
-        </is>
-      </c>
-      <c r="L132" t="inlineStr">
-        <is>
-          <t>Use only a trace film on dressed ABS-on-ABS sliding interfaces.</t>
+          <t>§10.2</t>
         </is>
       </c>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>SHP-016</t>
+          <t>SHP-015</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
@@ -7639,17 +7639,22 @@
       </c>
       <c r="D133" t="inlineStr">
         <is>
-          <t>White lithium grease, NLGI #2</t>
+          <t>Silicone grease, clear, NLGI 1</t>
         </is>
       </c>
       <c r="E133" t="inlineStr">
         <is>
-          <t>Light grease for mirror-cell spherical washer interfaces</t>
+          <t>ABS carriage sliding-interface lubricant</t>
         </is>
       </c>
       <c r="F133" t="inlineStr">
         <is>
-          <t>Lucas Oil Products</t>
+          <t>McMaster</t>
+        </is>
+      </c>
+      <c r="G133" t="inlineStr">
+        <is>
+          <t>1418K51</t>
         </is>
       </c>
       <c r="H133" t="n">
@@ -7667,19 +7672,19 @@
       </c>
       <c r="K133" t="inlineStr">
         <is>
-          <t>§10.4</t>
+          <t>§8.4</t>
         </is>
       </c>
       <c r="L133" t="inlineStr">
         <is>
-          <t>Existing shop stock inspected 2026-09-16 and appears usable.</t>
+          <t>Use only a trace film on dressed ABS-on-ABS sliding interfaces.</t>
         </is>
       </c>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>SHP-017</t>
+          <t>SHP-016</t>
         </is>
       </c>
       <c r="B134" t="inlineStr">
@@ -7692,22 +7697,17 @@
       </c>
       <c r="D134" t="inlineStr">
         <is>
-          <t>1/2" Forstner bit, standard-point smooth-finish</t>
+          <t>White lithium grease, NLGI #2</t>
         </is>
       </c>
       <c r="E134" t="inlineStr">
         <is>
-          <t>Spherical-washer counterbores</t>
+          <t>Light grease for mirror-cell spherical washer interfaces</t>
         </is>
       </c>
       <c r="F134" t="inlineStr">
         <is>
-          <t>McMaster</t>
-        </is>
-      </c>
-      <c r="G134" t="inlineStr">
-        <is>
-          <t>2890A56</t>
+          <t>Lucas Oil Products</t>
         </is>
       </c>
       <c r="H134" t="n">
@@ -7730,14 +7730,14 @@
       </c>
       <c r="L134" t="inlineStr">
         <is>
-          <t>Use in drill press for shallow close-fit spherical-washer sockets; test in scrap Baltic birch before cutting final plate.</t>
+          <t>Existing shop stock inspected 2026-09-16 and appears usable.</t>
         </is>
       </c>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>SHP-018</t>
+          <t>SHP-017</t>
         </is>
       </c>
       <c r="B135" t="inlineStr">
@@ -7750,12 +7750,12 @@
       </c>
       <c r="D135" t="inlineStr">
         <is>
-          <t>5/8" Forstner bit, standard-point smooth-finish</t>
+          <t>1/2" Forstner bit, standard-point smooth-finish</t>
         </is>
       </c>
       <c r="E135" t="inlineStr">
         <is>
-          <t>Spring-seat washer counterbores</t>
+          <t>Spherical-washer counterbores</t>
         </is>
       </c>
       <c r="F135" t="inlineStr">
@@ -7765,7 +7765,7 @@
       </c>
       <c r="G135" t="inlineStr">
         <is>
-          <t>2890A58</t>
+          <t>2890A56</t>
         </is>
       </c>
       <c r="H135" t="n">
@@ -7783,19 +7783,19 @@
       </c>
       <c r="K135" t="inlineStr">
         <is>
-          <t>§10.3</t>
+          <t>§10.4</t>
         </is>
       </c>
       <c r="L135" t="inlineStr">
         <is>
-          <t>Use in drill press for shallow spring-seat-washer registration counterbores; test depth/fit in scrap first.</t>
+          <t>Use in drill press for shallow close-fit spherical-washer sockets; test in scrap Baltic birch before cutting final plate.</t>
         </is>
       </c>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>SHP-019</t>
+          <t>SHP-018</t>
         </is>
       </c>
       <c r="B136" t="inlineStr">
@@ -7808,12 +7808,12 @@
       </c>
       <c r="D136" t="inlineStr">
         <is>
-          <t>M4 × 0.7 high-speed-steel plug-chamfer hex-bit tap</t>
+          <t>5/8" Forstner bit, standard-point smooth-finish</t>
         </is>
       </c>
       <c r="E136" t="inlineStr">
         <is>
-          <t>Tap CAMVATE quick-release plate mounting holes</t>
+          <t>Spring-seat washer counterbores</t>
         </is>
       </c>
       <c r="F136" t="inlineStr">
@@ -7823,7 +7823,7 @@
       </c>
       <c r="G136" t="inlineStr">
         <is>
-          <t>1021N23</t>
+          <t>2890A58</t>
         </is>
       </c>
       <c r="H136" t="n">
@@ -7841,19 +7841,19 @@
       </c>
       <c r="K136" t="inlineStr">
         <is>
-          <t>§10.9</t>
+          <t>§10.3</t>
         </is>
       </c>
       <c r="L136" t="inlineStr">
         <is>
-          <t>Use with 3.3 mm tap drill; exact hole locations await measurement of the delivered plate.</t>
+          <t>Use in drill press for shallow spring-seat-washer registration counterbores; test depth/fit in scrap first.</t>
         </is>
       </c>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>SHP-020</t>
+          <t>SHP-019</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
@@ -7866,12 +7866,12 @@
       </c>
       <c r="D137" t="inlineStr">
         <is>
-          <t>3.3 mm black-oxide HSS jobber-length drill bit</t>
+          <t>M4 × 0.7 high-speed-steel plug-chamfer hex-bit tap</t>
         </is>
       </c>
       <c r="E137" t="inlineStr">
         <is>
-          <t>M4 × 0.7 tap drill for CAMVATE quick-release plate; M3 heatsink clearance holes</t>
+          <t>Tap CAMVATE quick-release plate mounting holes</t>
         </is>
       </c>
       <c r="F137" t="inlineStr">
@@ -7881,7 +7881,7 @@
       </c>
       <c r="G137" t="inlineStr">
         <is>
-          <t>2958A64</t>
+          <t>1021N23</t>
         </is>
       </c>
       <c r="H137" t="n">
@@ -7899,19 +7899,19 @@
       </c>
       <c r="K137" t="inlineStr">
         <is>
-          <t>§§6.4, 10.9</t>
+          <t>§10.9</t>
         </is>
       </c>
       <c r="L137" t="inlineStr">
         <is>
-          <t>Standard 3.3 mm tap-drill size for M4 × 0.7. Also drills the Ø3.3 M3 clearance holes in the heatsink base (§6.4).</t>
+          <t>Use with 3.3 mm tap drill; exact hole locations await measurement of the delivered plate.</t>
         </is>
       </c>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>SHP-021</t>
+          <t>SHP-020</t>
         </is>
       </c>
       <c r="B138" t="inlineStr">
@@ -7924,12 +7924,12 @@
       </c>
       <c r="D138" t="inlineStr">
         <is>
-          <t>Loctite 243 medium-strength removable threadlocker, 0.34 fl. oz.</t>
+          <t>3.3 mm black-oxide HSS jobber-length drill bit</t>
         </is>
       </c>
       <c r="E138" t="inlineStr">
         <is>
-          <t>Removable thread retention for quick-release plate mounting screws</t>
+          <t>M4 × 0.7 tap drill for CAMVATE quick-release plate; M3 heatsink clearance holes</t>
         </is>
       </c>
       <c r="F138" t="inlineStr">
@@ -7939,7 +7939,7 @@
       </c>
       <c r="G138" t="inlineStr">
         <is>
-          <t>91458A115</t>
+          <t>2958A64</t>
         </is>
       </c>
       <c r="H138" t="n">
@@ -7957,19 +7957,19 @@
       </c>
       <c r="K138" t="inlineStr">
         <is>
-          <t>§10.9</t>
+          <t>§§6.4, 10.9</t>
         </is>
       </c>
       <c r="L138" t="inlineStr">
         <is>
-          <t>Apply only after fit and screw length are validated; preferred over high-strength Loctite 271 for this serviceable joint.</t>
+          <t>Standard 3.3 mm tap-drill size for M4 × 0.7. Also drills the Ø3.3 M3 clearance holes in the heatsink base (§6.4).</t>
         </is>
       </c>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>SHP-022</t>
+          <t>SHP-021</t>
         </is>
       </c>
       <c r="B139" t="inlineStr">
@@ -7982,22 +7982,22 @@
       </c>
       <c r="D139" t="inlineStr">
         <is>
-          <t>Rosco Photofoil matte black aluminum wrap, 12"x10'</t>
+          <t>Loctite 243 medium-strength removable threadlocker, 0.34 fl. oz.</t>
         </is>
       </c>
       <c r="E139" t="inlineStr">
         <is>
-          <t>Opaque masking / thin-sheet cutoff experiments</t>
+          <t>Removable thread retention for quick-release plate mounting screws</t>
         </is>
       </c>
       <c r="F139" t="inlineStr">
         <is>
-          <t>Fullcompass</t>
+          <t>McMaster</t>
         </is>
       </c>
       <c r="G139" t="inlineStr">
         <is>
-          <t>01001-1210</t>
+          <t>91458A115</t>
         </is>
       </c>
       <c r="H139" t="n">
@@ -8005,7 +8005,7 @@
       </c>
       <c r="I139" t="inlineStr">
         <is>
-          <t>pack</t>
+          <t>each</t>
         </is>
       </c>
       <c r="J139" t="inlineStr">
@@ -8015,19 +8015,19 @@
       </c>
       <c r="K139" t="inlineStr">
         <is>
-          <t>§§8, 8.7</t>
+          <t>§10.9</t>
         </is>
       </c>
       <c r="L139" t="inlineStr">
         <is>
-          <t>Retained as general shop stock for opaque masking and thin-sheet cutoff experiments.</t>
+          <t>Apply only after fit and screw length are validated; preferred over high-strength Loctite 271 for this serviceable joint.</t>
         </is>
       </c>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>SHP-023</t>
+          <t>SHP-022</t>
         </is>
       </c>
       <c r="B140" t="inlineStr">
@@ -8040,22 +8040,22 @@
       </c>
       <c r="D140" t="inlineStr">
         <is>
-          <t>M3 × 0.5 high-speed-steel plug-chamfer tap, 5/8" thread length</t>
+          <t>Rosco Photofoil matte black aluminum wrap, 12"x10'</t>
         </is>
       </c>
       <c r="E140" t="inlineStr">
         <is>
-          <t>Tap through M3 heatsink-screw holes in SM1CP2M cap</t>
+          <t>Opaque masking / thin-sheet cutoff experiments</t>
         </is>
       </c>
       <c r="F140" t="inlineStr">
         <is>
-          <t>McMaster</t>
+          <t>Fullcompass</t>
         </is>
       </c>
       <c r="G140" t="inlineStr">
         <is>
-          <t>8305A32</t>
+          <t>01001-1210</t>
         </is>
       </c>
       <c r="H140" t="n">
@@ -8063,29 +8063,29 @@
       </c>
       <c r="I140" t="inlineStr">
         <is>
-          <t>each</t>
+          <t>pack</t>
         </is>
       </c>
       <c r="J140" t="inlineStr">
         <is>
-          <t>To procure</t>
+          <t>In hand</t>
         </is>
       </c>
       <c r="K140" t="inlineStr">
         <is>
-          <t>§6.4</t>
+          <t>§§8, 8.7</t>
         </is>
       </c>
       <c r="L140" t="inlineStr">
         <is>
-          <t>All holes are through holes, so a plug chamfer is enough; no bottoming tap needed. Use with the 2.5 mm tap drill (SHP-025). Confirm no M3 tap already in shop stock.</t>
+          <t>Retained as general shop stock for opaque masking and thin-sheet cutoff experiments.</t>
         </is>
       </c>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>SHP-025</t>
+          <t>SHP-023</t>
         </is>
       </c>
       <c r="B141" t="inlineStr">
@@ -8098,12 +8098,12 @@
       </c>
       <c r="D141" t="inlineStr">
         <is>
-          <t>2.5 mm TiN-coated HSS short-length drill bit, 43 mm overall</t>
+          <t>M3 × 0.5 high-speed-steel plug-chamfer tap, 5/8" thread length</t>
         </is>
       </c>
       <c r="E141" t="inlineStr">
         <is>
-          <t>M3 tap drill for through holes in SM1CP2M cap</t>
+          <t>Tap through M3 heatsink-screw holes in SM1CP2M cap</t>
         </is>
       </c>
       <c r="F141" t="inlineStr">
@@ -8113,7 +8113,7 @@
       </c>
       <c r="G141" t="inlineStr">
         <is>
-          <t>2979N15</t>
+          <t>8305A32</t>
         </is>
       </c>
       <c r="H141" t="n">
@@ -8136,71 +8136,129 @@
       </c>
       <c r="L141" t="inlineStr">
         <is>
-          <t>Short-length stub drill for rigid drilling in the thin cap; same series as the 1.6 mm drill SHP-006.</t>
+          <t>All holes are through holes, so a plug chamfer is enough; no bottoming tap needed. Use with the 2.5 mm tap drill (SHP-025). Confirm no M3 tap already in shop stock.</t>
         </is>
       </c>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
+          <t>SHP-025</t>
+        </is>
+      </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>Shop supplies</t>
+        </is>
+      </c>
+      <c r="C142" t="n">
+        <v>1</v>
+      </c>
+      <c r="D142" t="inlineStr">
+        <is>
+          <t>2.5 mm TiN-coated HSS short-length drill bit, 43 mm overall</t>
+        </is>
+      </c>
+      <c r="E142" t="inlineStr">
+        <is>
+          <t>M3 tap drill for through holes in SM1CP2M cap</t>
+        </is>
+      </c>
+      <c r="F142" t="inlineStr">
+        <is>
+          <t>McMaster</t>
+        </is>
+      </c>
+      <c r="G142" t="inlineStr">
+        <is>
+          <t>2979N15</t>
+        </is>
+      </c>
+      <c r="H142" t="n">
+        <v>1</v>
+      </c>
+      <c r="I142" t="inlineStr">
+        <is>
+          <t>each</t>
+        </is>
+      </c>
+      <c r="J142" t="inlineStr">
+        <is>
+          <t>To procure</t>
+        </is>
+      </c>
+      <c r="K142" t="inlineStr">
+        <is>
+          <t>§6.4</t>
+        </is>
+      </c>
+      <c r="L142" t="inlineStr">
+        <is>
+          <t>Short-length stub drill for rigid drilling in the thin cap; same series as the 1.6 mm drill SHP-006.</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
           <t>SHP-026</t>
         </is>
       </c>
-      <c r="B142" t="inlineStr">
+      <c r="B143" t="inlineStr">
         <is>
           <t>Shop supplies</t>
         </is>
       </c>
-      <c r="C142" t="n">
-        <v>1</v>
-      </c>
-      <c r="D142" t="inlineStr">
+      <c r="C143" t="n">
+        <v>1</v>
+      </c>
+      <c r="D143" t="inlineStr">
         <is>
           <t>2.0 mm uncoated HSS short-length drill bit, 38 mm overall</t>
         </is>
       </c>
-      <c r="E142" t="inlineStr">
+      <c r="E143" t="inlineStr">
         <is>
           <t>Lead holes through SM1CP2M cap and heatsink base</t>
         </is>
       </c>
-      <c r="F142" t="inlineStr">
+      <c r="F143" t="inlineStr">
         <is>
           <t>McMaster</t>
         </is>
       </c>
-      <c r="G142" t="inlineStr">
+      <c r="G143" t="inlineStr">
         <is>
           <t>2979N14</t>
         </is>
       </c>
-      <c r="H142" t="n">
-        <v>1</v>
-      </c>
-      <c r="I142" t="inlineStr">
+      <c r="H143" t="n">
+        <v>1</v>
+      </c>
+      <c r="I143" t="inlineStr">
         <is>
           <t>each</t>
         </is>
       </c>
-      <c r="J142" t="inlineStr">
+      <c r="J143" t="inlineStr">
         <is>
           <t>To procure</t>
         </is>
       </c>
-      <c r="K142" t="inlineStr">
+      <c r="K143" t="inlineStr">
         <is>
           <t>§6.4</t>
         </is>
       </c>
-      <c r="L142" t="inlineStr">
+      <c r="L143" t="inlineStr">
         <is>
           <t>Same series as the 1.6 mm drill SHP-006.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L142"/>
-  <conditionalFormatting sqref="J2:J142">
+  <autoFilter ref="A1:L143"/>
+  <conditionalFormatting sqref="J2:J143">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"In hand"</formula>
     </cfRule>
@@ -8218,7 +8276,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="J2:J142" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
+    <dataValidation sqref="J2:J143" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
       <formula1>"In hand,On order,To procure,Specified,CAD ready,CAD open"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
model and doc updates, recent procurements
</commit_message>
<xml_diff>
--- a/bom/schlieren-bom.xlsx
+++ b/bom/schlieren-bom.xlsx
@@ -2039,7 +2039,7 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>ABS printed post shoes</t>
+          <t>PLA printed post shoes</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
@@ -2911,7 +2911,7 @@
       </c>
       <c r="J40" t="inlineStr">
         <is>
-          <t>To procure</t>
+          <t>On order</t>
         </is>
       </c>
       <c r="K40" t="inlineStr">
@@ -2966,7 +2966,7 @@
       </c>
       <c r="J41" t="inlineStr">
         <is>
-          <t>To procure</t>
+          <t>On order</t>
         </is>
       </c>
       <c r="K41" t="inlineStr">
@@ -2996,7 +2996,7 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>M3 × 6 mm socket head screw</t>
+          <t>M3 × 0.5 × 6 mm socket head screw, 18-8 SS</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
@@ -3009,9 +3009,22 @@
           <t>McMaster</t>
         </is>
       </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>91292A111</t>
+        </is>
+      </c>
+      <c r="H42" t="n">
+        <v>100</v>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>pack</t>
+        </is>
+      </c>
       <c r="J42" t="inlineStr">
         <is>
-          <t>Specified</t>
+          <t>On order</t>
         </is>
       </c>
       <c r="K42" t="inlineStr">
@@ -3021,7 +3034,7 @@
       </c>
       <c r="L42" t="inlineStr">
         <is>
-          <t>Three per module. Provisional length (3 mm base + ~3 mm thread into the through-tapped cap; shorter than the cap thickness). SKU to be confirmed; check existing M3 stock.</t>
+          <t>Three per module. Provisional length (3 mm base + ~3 mm thread into the through-tapped cap; shorter than the cap thickness). Same series as the common 12 mm screw; no 6 mm screws in stock.</t>
         </is>
       </c>
     </row>
@@ -3563,7 +3576,7 @@
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>ABS printed flexure slit head</t>
+          <t>PLA printed flexure slit head</t>
         </is>
       </c>
       <c r="J52" t="inlineStr">
@@ -3598,7 +3611,7 @@
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>ABS printed slit-head spigot adapter</t>
+          <t>PLA printed slit-head spigot adapter</t>
         </is>
       </c>
       <c r="J53" t="inlineStr">
@@ -3628,7 +3641,7 @@
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>ABS printed slit-head blade clamp bars</t>
+          <t>PLA printed slit-head blade clamp bars</t>
         </is>
       </c>
       <c r="J54" t="inlineStr">
@@ -4048,7 +4061,7 @@
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>ABS printed carriage bodies</t>
+          <t>PLA printed carriage bodies</t>
         </is>
       </c>
       <c r="J62" t="inlineStr">
@@ -4121,7 +4134,7 @@
       </c>
       <c r="L63" t="inlineStr">
         <is>
-          <t>Nickel-plated rectangular magnets; one hard contact insert for the FAS100-driven ABS plunger of the cutoff carriage.</t>
+          <t>Nickel-plated rectangular magnets; one hard contact insert for the FAS100-driven PLA plunger of the cutoff carriage.</t>
         </is>
       </c>
     </row>
@@ -4141,7 +4154,7 @@
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>ABS printed open-center keeper frames</t>
+          <t>PLA printed open-center keeper frames</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
@@ -4219,7 +4232,7 @@
       </c>
       <c r="L65" t="inlineStr">
         <is>
-          <t>Reuse common M3 × 12 mm stock. Heads bear directly on ABS in ~0.5 mm recesses; tighten only to a light snug; verify printed fit.</t>
+          <t>Reuse common M3 × 12 mm stock. Heads bear directly on PLA in ~0.5 mm recesses; tighten only to a light snug; verify printed fit.</t>
         </is>
       </c>
     </row>
@@ -4277,7 +4290,7 @@
       </c>
       <c r="L66" t="inlineStr">
         <is>
-          <t>Full-height DIN 934 nut. ~2.5 mm captive hex pocket from carriage back, leaving ~1.5 mm ABS floor above pocket.</t>
+          <t>Full-height DIN 934 nut. ~2.5 mm captive hex pocket from carriage back, leaving ~1.5 mm PLA floor above pocket.</t>
         </is>
       </c>
     </row>
@@ -4297,7 +4310,7 @@
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>ABS printed cassettes</t>
+          <t>PLA printed cassettes</t>
         </is>
       </c>
       <c r="J67" t="inlineStr">
@@ -4428,7 +4441,7 @@
       </c>
       <c r="L69" t="inlineStr">
         <is>
-          <t>Provisional 14 mm length; fit-test with 4 mm bar.</t>
+          <t>Fit-tested on built cassettes with 4 mm bars: full nut engagement, head flush in countersink.</t>
         </is>
       </c>
     </row>
@@ -5203,7 +5216,7 @@
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>ABS printed phone rest</t>
+          <t>PLA printed phone rest</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">
@@ -5243,7 +5256,7 @@
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>ABS printed lens pointer shoe</t>
+          <t>PLA printed lens pointer shoe</t>
         </is>
       </c>
       <c r="E85" t="inlineStr">
@@ -5369,7 +5382,7 @@
       </c>
       <c r="J87" t="inlineStr">
         <is>
-          <t>To procure</t>
+          <t>On order</t>
         </is>
       </c>
       <c r="K87" t="inlineStr">
@@ -5399,7 +5412,7 @@
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>ABS printed lens collars</t>
+          <t>PLA printed lens collars</t>
         </is>
       </c>
       <c r="E88" t="inlineStr">
@@ -5583,7 +5596,7 @@
       </c>
       <c r="J91" t="inlineStr">
         <is>
-          <t>To procure</t>
+          <t>On order</t>
         </is>
       </c>
       <c r="K91" t="inlineStr">
@@ -5613,7 +5626,7 @@
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>ABS printed lens pointer yokes</t>
+          <t>PLA printed lens pointer yokes</t>
         </is>
       </c>
       <c r="E92" t="inlineStr">
@@ -5681,7 +5694,7 @@
       </c>
       <c r="J93" t="inlineStr">
         <is>
-          <t>To procure</t>
+          <t>On order</t>
         </is>
       </c>
       <c r="K93" t="inlineStr">
@@ -5739,7 +5752,7 @@
       </c>
       <c r="J94" t="inlineStr">
         <is>
-          <t>To procure</t>
+          <t>On order</t>
         </is>
       </c>
       <c r="K94" t="inlineStr">
@@ -6367,7 +6380,7 @@
       </c>
       <c r="L106" t="inlineStr">
         <is>
-          <t>Eight installed, four per bracket; existing stock was confirmed in hand for six, so confirm two more.</t>
+          <t>Eight installed, four per bracket. Two 5-packs in hand (10 nuts, two spare).</t>
         </is>
       </c>
     </row>
@@ -6884,7 +6897,7 @@
       </c>
       <c r="D116" t="inlineStr">
         <is>
-          <t>ABS printed front safety retainers</t>
+          <t>PLA printed front safety retainers</t>
         </is>
       </c>
       <c r="J116" t="inlineStr">
@@ -6997,7 +7010,7 @@
       </c>
       <c r="J118" t="inlineStr">
         <is>
-          <t>To procure</t>
+          <t>On order</t>
         </is>
       </c>
       <c r="K118" t="inlineStr">
@@ -7486,7 +7499,7 @@
       </c>
       <c r="L129" t="inlineStr">
         <is>
-          <t>Use sparingly: wick into Baltic-birch fibers for spherical-washer sockets; use needle-sized localized drops for ABS/metal calibration tacks and captive screw retention. No accelerator required.</t>
+          <t>Use sparingly: wick into Baltic-birch fibers for spherical-washer sockets; use needle-sized localized drops for PLA/metal calibration tacks and captive screw retention. No accelerator required.</t>
         </is>
       </c>
     </row>
@@ -7644,7 +7657,7 @@
       </c>
       <c r="E133" t="inlineStr">
         <is>
-          <t>ABS carriage sliding-interface lubricant</t>
+          <t>PLA carriage sliding-interface lubricant</t>
         </is>
       </c>
       <c r="F133" t="inlineStr">
@@ -7677,7 +7690,7 @@
       </c>
       <c r="L133" t="inlineStr">
         <is>
-          <t>Use only a trace film on dressed ABS-on-ABS sliding interfaces.</t>
+          <t>Use only a trace film on dressed PLA-on-PLA sliding interfaces.</t>
         </is>
       </c>
     </row>
@@ -8126,7 +8139,7 @@
       </c>
       <c r="J141" t="inlineStr">
         <is>
-          <t>To procure</t>
+          <t>On order</t>
         </is>
       </c>
       <c r="K141" t="inlineStr">
@@ -8184,7 +8197,7 @@
       </c>
       <c r="J142" t="inlineStr">
         <is>
-          <t>To procure</t>
+          <t>On order</t>
         </is>
       </c>
       <c r="K142" t="inlineStr">
@@ -8252,7 +8265,7 @@
       </c>
       <c r="L143" t="inlineStr">
         <is>
-          <t>Same series as the 1.6 mm drill SHP-006.</t>
+          <t>Same series as the 1.6 mm drill SHP-006. Deferred, not in the current order: lead hole size is provisional (§6.4), and the 2.5 mm drill SHP-025 may cut the lead holes instead. Decide after measuring the pigtail insulation.</t>
         </is>
       </c>
     </row>
@@ -8300,7 +8313,7 @@
       </c>
       <c r="J144" t="inlineStr">
         <is>
-          <t>To procure</t>
+          <t>On order</t>
         </is>
       </c>
       <c r="K144" t="inlineStr">
@@ -8310,7 +8323,7 @@
       </c>
       <c r="L144" t="inlineStr">
         <is>
-          <t>Listed for Hakko 900M. The M5 tip has a female threaded connection and mounts through the included adapter; how the adapter mates with the iron and with SHP-002 is unverified. Used with the Hakko iron SHP-028; set ABS installation near 250–265 °C, no higher than 280 °C.</t>
+          <t>Listed for Hakko 900M. The M5 tip has a female threaded connection and mounts through the included adapter; how the adapter mates with the iron and with SHP-002 is unverified. Used with the Hakko iron SHP-028; set PLA installation near 200–230 °C (typical for PLA; confirm on a scrap print), no higher than 250 °C.</t>
         </is>
       </c>
     </row>
@@ -8353,7 +8366,7 @@
       </c>
       <c r="J145" t="inlineStr">
         <is>
-          <t>To procure</t>
+          <t>On order</t>
         </is>
       </c>
       <c r="K145" t="inlineStr">

</xml_diff>

<commit_message>
rename 'lens pointer' to 'lens cradle'
</commit_message>
<xml_diff>
--- a/bom/schlieren-bom.xlsx
+++ b/bom/schlieren-bom.xlsx
@@ -5047,7 +5047,7 @@
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>Lens pointer adjusters</t>
+          <t>Lens cradle adjusters</t>
         </is>
       </c>
       <c r="F81" t="inlineStr">
@@ -5105,7 +5105,7 @@
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>Lens pointer adjusters and yoke joints</t>
+          <t>Lens cradle adjusters and yoke joints</t>
         </is>
       </c>
       <c r="F82" t="inlineStr">
@@ -5163,7 +5163,7 @@
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>Lens pointer adjuster handwheels</t>
+          <t>Lens cradle adjuster handwheels</t>
         </is>
       </c>
       <c r="F83" t="inlineStr">
@@ -5256,7 +5256,7 @@
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>PLA printed lens pointer shoe</t>
+          <t>PLA printed lens cradle shoe</t>
         </is>
       </c>
       <c r="E85" t="inlineStr">
@@ -5301,7 +5301,7 @@
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>Hard bearing pads under three lens-pointer screw tips</t>
+          <t>Hard bearing pads under three lens-cradle screw tips</t>
         </is>
       </c>
       <c r="F86" t="inlineStr">
@@ -5359,7 +5359,7 @@
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>Groove rods at the fourth lens-pointer screw</t>
+          <t>Groove rods at the fourth lens-cradle screw</t>
         </is>
       </c>
       <c r="F87" t="inlineStr">
@@ -5573,7 +5573,7 @@
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t>Lens pointer retaining bands</t>
+          <t>Lens cradle retaining bands</t>
         </is>
       </c>
       <c r="F91" t="inlineStr">
@@ -5626,7 +5626,7 @@
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>PLA printed lens pointer yokes</t>
+          <t>PLA printed lens cradle yokes</t>
         </is>
       </c>
       <c r="E92" t="inlineStr">
@@ -5646,7 +5646,7 @@
       </c>
       <c r="L92" t="inlineStr">
         <is>
-          <t>Printed on their side; each bolted to the pointer shoe with one countersunk M5 screw (CAM-016) into a heat-set insert (CAM-005).</t>
+          <t>Printed on their side; each bolted to the cradle shoe with one countersunk M5 screw (CAM-016) into a heat-set insert (CAM-005).</t>
         </is>
       </c>
     </row>
@@ -5704,7 +5704,7 @@
       </c>
       <c r="L93" t="inlineStr">
         <is>
-          <t>10 mm head, 3 mm hex drive. Each screws up through the pointer shoe deck into a heat-set insert in the yoke foot.</t>
+          <t>10 mm head, 3 mm hex drive. Each screws up through the cradle shoe deck into a heat-set insert in the yoke foot.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
BOM updates; add locating ridge for lens collar lateral stop pins
</commit_message>
<xml_diff>
--- a/bom/schlieren-bom.xlsx
+++ b/bom/schlieren-bom.xlsx
@@ -2904,6 +2904,9 @@
           <t>SM1CP2M</t>
         </is>
       </c>
+      <c r="H40" t="n">
+        <v>1</v>
+      </c>
       <c r="I40" t="inlineStr">
         <is>
           <t>each</t>
@@ -2911,7 +2914,7 @@
       </c>
       <c r="J40" t="inlineStr">
         <is>
-          <t>On order</t>
+          <t>In hand</t>
         </is>
       </c>
       <c r="K40" t="inlineStr">
@@ -3024,7 +3027,7 @@
       </c>
       <c r="J42" t="inlineStr">
         <is>
-          <t>On order</t>
+          <t>In hand</t>
         </is>
       </c>
       <c r="K42" t="inlineStr">
@@ -5382,7 +5385,7 @@
       </c>
       <c r="J87" t="inlineStr">
         <is>
-          <t>On order</t>
+          <t>In hand</t>
         </is>
       </c>
       <c r="K87" t="inlineStr">
@@ -5596,7 +5599,7 @@
       </c>
       <c r="J91" t="inlineStr">
         <is>
-          <t>On order</t>
+          <t>In hand</t>
         </is>
       </c>
       <c r="K91" t="inlineStr">
@@ -5694,7 +5697,7 @@
       </c>
       <c r="J93" t="inlineStr">
         <is>
-          <t>On order</t>
+          <t>In hand</t>
         </is>
       </c>
       <c r="K93" t="inlineStr">
@@ -5752,7 +5755,7 @@
       </c>
       <c r="J94" t="inlineStr">
         <is>
-          <t>On order</t>
+          <t>In hand</t>
         </is>
       </c>
       <c r="K94" t="inlineStr">
@@ -7010,7 +7013,7 @@
       </c>
       <c r="J118" t="inlineStr">
         <is>
-          <t>On order</t>
+          <t>In hand</t>
         </is>
       </c>
       <c r="K118" t="inlineStr">
@@ -8139,7 +8142,7 @@
       </c>
       <c r="J141" t="inlineStr">
         <is>
-          <t>On order</t>
+          <t>In hand</t>
         </is>
       </c>
       <c r="K141" t="inlineStr">
@@ -8197,7 +8200,7 @@
       </c>
       <c r="J142" t="inlineStr">
         <is>
-          <t>On order</t>
+          <t>In hand</t>
         </is>
       </c>
       <c r="K142" t="inlineStr">
@@ -8313,7 +8316,7 @@
       </c>
       <c r="J144" t="inlineStr">
         <is>
-          <t>On order</t>
+          <t>In hand</t>
         </is>
       </c>
       <c r="K144" t="inlineStr">
@@ -8323,7 +8326,7 @@
       </c>
       <c r="L144" t="inlineStr">
         <is>
-          <t>Listed for Hakko 900M. The M5 tip has a female threaded connection and mounts through the included adapter; how the adapter mates with the iron and with SHP-002 is unverified. Used with the Hakko iron SHP-028; set PLA installation near 200–230 °C (typical for PLA; confirm on a scrap print), no higher than 250 °C.</t>
+          <t>Listed for Hakko 900M. The M5 tip has a female threaded connection and mounts through the included adapter, which fits the Hakko iron (confirmed); how it mates with SHP-002 is unverified. Used with the Hakko iron SHP-028; set PLA installation near 200–230 °C (typical for PLA; confirm on a scrap print), no higher than 250 °C.</t>
         </is>
       </c>
     </row>
@@ -8366,7 +8369,7 @@
       </c>
       <c r="J145" t="inlineStr">
         <is>
-          <t>On order</t>
+          <t>In hand</t>
         </is>
       </c>
       <c r="K145" t="inlineStr">
@@ -8376,7 +8379,7 @@
       </c>
       <c r="L145" t="inlineStr">
         <is>
-          <t>Ordered 2026-10-08; vendor not recorded here. Takes Hakko T18 (900M-style) tips. Drives the SHP-027 tip set; adapter fit to SHP-002 unverified.</t>
+          <t>Ordered 2026-10-08; vendor not recorded here. Takes Hakko T18 (900M-style) tips. Drives the SHP-027 tip set; the SHP-027 adapter fits the iron (confirmed); fit of SHP-002 unverified.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add hardware models for LED module model, correct BOM lint
</commit_message>
<xml_diff>
--- a/bom/schlieren-bom.xlsx
+++ b/bom/schlieren-bom.xlsx
@@ -2838,7 +2838,7 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>DP11 connection</t>
+          <t>DP100 connection</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
@@ -2924,7 +2924,7 @@
       </c>
       <c r="L40" t="inlineStr">
         <is>
-          <t>One per LED module. Drill/tap: M2 board holes (front), M3 heatsink holes (rear, ~2.5 mm deep), lead pass-through holes at r ≈ 11 mm.</t>
+          <t>One per LED module. Drill/tap, all through holes (§6.4): M2 board holes, M3 heatsink holes, lead pass-through holes at r = 11.0 mm.</t>
         </is>
       </c>
     </row>
@@ -3037,7 +3037,7 @@
       </c>
       <c r="L42" t="inlineStr">
         <is>
-          <t>Three per module. Provisional length (3 mm base + ~3 mm thread into the through-tapped cap; shorter than the cap thickness). Same series as the common 12 mm screw; no 6 mm screws in stock.</t>
+          <t>Three per module. Provisional length (3 mm base + ~3 mm thread into the through-tapped cap; shorter than the cap thickness). Same series as the common 12 mm screw.</t>
         </is>
       </c>
     </row>
@@ -3322,7 +3322,7 @@
       </c>
       <c r="K47" t="inlineStr">
         <is>
-          <t>§§7.3–7.4</t>
+          <t>§7.7</t>
         </is>
       </c>
       <c r="L47" t="inlineStr">
@@ -4235,7 +4235,7 @@
       </c>
       <c r="L65" t="inlineStr">
         <is>
-          <t>Reuse common M3 × 12 mm stock. Heads bear directly on PLA in ~0.5 mm recesses; tighten only to a light snug; verify printed fit.</t>
+          <t>Reuse common M3 × 12 mm stock. Heads bear directly on PLA in ~0.5 mm recesses; tighten only to a light snug.</t>
         </is>
       </c>
     </row>
@@ -5604,7 +5604,7 @@
       </c>
       <c r="K91" t="inlineStr">
         <is>
-          <t>§9.5</t>
+          <t>§9.8</t>
         </is>
       </c>
       <c r="L91" t="inlineStr">
@@ -6658,7 +6658,7 @@
       </c>
       <c r="L111" t="inlineStr">
         <is>
-          <t>Order one pack. Four screws are the provisional installed quantity if this length matches the measured CAMVATE plate thickness; otherwise use MIR-024.</t>
+          <t>Four screws are the provisional installed quantity if this length matches the measured CAMVATE plate thickness; otherwise use MIR-024.</t>
         </is>
       </c>
     </row>
@@ -6716,7 +6716,7 @@
       </c>
       <c r="L112" t="inlineStr">
         <is>
-          <t>Order one pack. Four screws are the provisional installed quantity if this length matches the measured CAMVATE plate thickness; otherwise use MIR-023.</t>
+          <t>Four screws are the provisional installed quantity if this length matches the measured CAMVATE plate thickness; otherwise use MIR-023.</t>
         </is>
       </c>
     </row>
@@ -6774,7 +6774,7 @@
       </c>
       <c r="L113" t="inlineStr">
         <is>
-          <t>Complete 577/501/504-compatible quick-release assembly with removable sliding plate and receiver. Exact removable-plate hole pattern and final M4 screw length to be verified on arrival.</t>
+          <t>Complete 577/501/504-compatible quick-release assembly with removable sliding plate and receiver. The removable plate is drilled and tapped M4 to the §10.9 layout.</t>
         </is>
       </c>
     </row>
@@ -7023,7 +7023,7 @@
       </c>
       <c r="L118" t="inlineStr">
         <is>
-          <t>Four per bracket, two through the plate and two through the base; eight installed, so order two 5-packs (two spare). 3/16 in hex drive; head Ø0.547 in × 0.166 in. Pushed through from the bracket side, with MIR-013 washers and MIR-012 locknuts behind the plywood. Thread projects about 0.12 in past the locknut.</t>
+          <t>Four per bracket, two through the plate and two through the base; eight installed. 3/16 in hex drive; head Ø0.547 in × 0.166 in. Pushed through from the bracket side, with MIR-013 washers and MIR-012 locknuts behind the plywood. Thread projects about 0.12 in past the locknut.</t>
         </is>
       </c>
     </row>
@@ -7071,7 +7071,7 @@
       </c>
       <c r="K119" t="inlineStr">
         <is>
-          <t>§9.5</t>
+          <t>§9.7</t>
         </is>
       </c>
     </row>
@@ -7119,7 +7119,7 @@
       </c>
       <c r="K120" t="inlineStr">
         <is>
-          <t>§9.5</t>
+          <t>§9.7</t>
         </is>
       </c>
     </row>
@@ -7497,7 +7497,7 @@
       </c>
       <c r="K129" t="inlineStr">
         <is>
-          <t>§§6.2, 7, 8.4, 10.4</t>
+          <t>§§8.3, 8.4, 8.7, 10.4</t>
         </is>
       </c>
       <c r="L129" t="inlineStr">
@@ -7920,7 +7920,7 @@
       </c>
       <c r="L137" t="inlineStr">
         <is>
-          <t>Use with 3.3 mm tap drill; exact hole locations await measurement of the delivered plate.</t>
+          <t>Use with the 3.3 mm tap drill (SHP-020); hole locations in §10.9.</t>
         </is>
       </c>
     </row>
@@ -8089,7 +8089,7 @@
       </c>
       <c r="K140" t="inlineStr">
         <is>
-          <t>§§8, 8.7</t>
+          <t>§§8.6, 8.7</t>
         </is>
       </c>
       <c r="L140" t="inlineStr">
@@ -8152,7 +8152,7 @@
       </c>
       <c r="L141" t="inlineStr">
         <is>
-          <t>All holes are through holes, so a plug chamfer is enough; no bottoming tap needed. Use with the 2.5 mm tap drill (SHP-025). Confirm no M3 tap already in shop stock.</t>
+          <t>All holes are through holes, so a plug chamfer is enough; no bottoming tap needed. Use with the 2.5 mm tap drill (SHP-025).</t>
         </is>
       </c>
     </row>
@@ -8379,7 +8379,7 @@
       </c>
       <c r="L145" t="inlineStr">
         <is>
-          <t>Ordered 2026-10-08; vendor not recorded here. Takes Hakko T18 (900M-style) tips. Drives the SHP-027 tip set; the SHP-027 adapter fits the iron (confirmed); fit of SHP-002 unverified.</t>
+          <t>Vendor not recorded here. Takes Hakko T18 (900M-style) tips. Drives the SHP-027 tip set; the SHP-027 adapter fits the iron (confirmed); fit of SHP-002 unverified.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Rail mount hardware clarification
</commit_message>
<xml_diff>
--- a/bom/schlieren-bom.xlsx
+++ b/bom/schlieren-bom.xlsx
@@ -1286,6 +1286,11 @@
           <t>§4.3</t>
         </is>
       </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>Shared stock with FRM-011: two 10-packs in hand, 12 allocated (4 here, 8 on the yaw clamps); 8 spare.</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1496,6 +1501,11 @@
       <c r="K12" t="inlineStr">
         <is>
           <t>§4.3</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>Shared stock with FRM-007: two 10-packs in hand, 12 allocated (8 here, 4 on the rail pivots); 8 spare.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add spot drill bits to bom; re-render figures and doc
</commit_message>
<xml_diff>
--- a/bom/schlieren-bom.xlsx
+++ b/bom/schlieren-bom.xlsx
@@ -11,7 +11,7 @@
     <sheet name="BOM" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'BOM'!$A$1:$L$145</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'BOM'!$A$1:$L$147</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -837,7 +837,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L145"/>
+  <dimension ref="A1:L147"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -8391,9 +8391,125 @@
         </is>
       </c>
     </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>SHP-029</t>
+        </is>
+      </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>Shop supplies</t>
+        </is>
+      </c>
+      <c r="C146" t="n">
+        <v>1</v>
+      </c>
+      <c r="D146" t="inlineStr">
+        <is>
+          <t>Hole-starting cobalt-steel drill bit, uncoated, 90° point, 1/8" size</t>
+        </is>
+      </c>
+      <c r="E146" t="inlineStr">
+        <is>
+          <t>Spot hole locations in the SM1CP2M cap and heatsink base before drilling</t>
+        </is>
+      </c>
+      <c r="F146" t="inlineStr">
+        <is>
+          <t>McMaster</t>
+        </is>
+      </c>
+      <c r="G146" t="inlineStr">
+        <is>
+          <t>27445A201</t>
+        </is>
+      </c>
+      <c r="H146" t="n">
+        <v>1</v>
+      </c>
+      <c r="I146" t="inlineStr">
+        <is>
+          <t>each</t>
+        </is>
+      </c>
+      <c r="J146" t="inlineStr">
+        <is>
+          <t>On order</t>
+        </is>
+      </c>
+      <c r="K146" t="inlineStr">
+        <is>
+          <t>§6.4</t>
+        </is>
+      </c>
+      <c r="L146" t="inlineStr">
+        <is>
+          <t>1/8" shank fits the Dremel 4486 chuck (1/8" maximum). Use before the 1.6, 2.0, 2.5, and 3.3 mm drills.</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>SHP-030</t>
+        </is>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>Shop supplies</t>
+        </is>
+      </c>
+      <c r="C147" t="n">
+        <v>1</v>
+      </c>
+      <c r="D147" t="inlineStr">
+        <is>
+          <t>Center drill, high-speed steel, 60° countersink, trade size 1, 1-1/4" overall length</t>
+        </is>
+      </c>
+      <c r="E147" t="inlineStr">
+        <is>
+          <t>Backup hole spotter; spots the cap and heatsink holes</t>
+        </is>
+      </c>
+      <c r="F147" t="inlineStr">
+        <is>
+          <t>McMaster</t>
+        </is>
+      </c>
+      <c r="G147" t="inlineStr">
+        <is>
+          <t>2915A11</t>
+        </is>
+      </c>
+      <c r="H147" t="n">
+        <v>1</v>
+      </c>
+      <c r="I147" t="inlineStr">
+        <is>
+          <t>each</t>
+        </is>
+      </c>
+      <c r="J147" t="inlineStr">
+        <is>
+          <t>On order</t>
+        </is>
+      </c>
+      <c r="K147" t="inlineStr">
+        <is>
+          <t>§6.4</t>
+        </is>
+      </c>
+      <c r="L147" t="inlineStr">
+        <is>
+          <t>3/64" pilot, 1/8" body; fits the Dremel 4486 chuck. Spare for SHP-029.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L145"/>
-  <conditionalFormatting sqref="J2:J145">
+  <autoFilter ref="A1:L147"/>
+  <conditionalFormatting sqref="J2:J147">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"In hand"</formula>
     </cfRule>
@@ -8411,7 +8527,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="J2:J145" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
+    <dataValidation sqref="J2:J147" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
       <formula1>"In hand,On order,To procure,Specified,CAD ready,CAD open"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
render rail hardware in camera support
</commit_message>
<xml_diff>
--- a/bom/schlieren-bom.xlsx
+++ b/bom/schlieren-bom.xlsx
@@ -8435,7 +8435,7 @@
       </c>
       <c r="J146" t="inlineStr">
         <is>
-          <t>On order</t>
+          <t>In hand</t>
         </is>
       </c>
       <c r="K146" t="inlineStr">
@@ -8493,7 +8493,7 @@
       </c>
       <c r="J147" t="inlineStr">
         <is>
-          <t>On order</t>
+          <t>In hand</t>
         </is>
       </c>
       <c r="K147" t="inlineStr">

</xml_diff>

<commit_message>
Update white lithium grease selection
</commit_message>
<xml_diff>
--- a/bom/schlieren-bom.xlsx
+++ b/bom/schlieren-bom.xlsx
@@ -7089,7 +7089,7 @@
       </c>
       <c r="D119" t="inlineStr">
         <is>
-          <t>White lithium grease, NLGI #2</t>
+          <t>Dynatex 159375 White Lithium Grease NLGI 2</t>
         </is>
       </c>
       <c r="E119" t="inlineStr">
@@ -7099,7 +7099,12 @@
       </c>
       <c r="F119" t="inlineStr">
         <is>
-          <t>Lucas Oil Products</t>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="G119" t="inlineStr">
+        <is>
+          <t>B009XE8M3G</t>
         </is>
       </c>
       <c r="H119" t="n">
@@ -7112,7 +7117,7 @@
       </c>
       <c r="J119" t="inlineStr">
         <is>
-          <t>In hand</t>
+          <t>On order</t>
         </is>
       </c>
       <c r="K119" t="inlineStr">
@@ -7122,7 +7127,7 @@
       </c>
       <c r="L119" t="inlineStr">
         <is>
-          <t>Existing shop stock inspected 2026-09-16 and appears usable.</t>
+          <t>Small tube to transport with the apparatus.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update notes on heat set installation tooling
</commit_message>
<xml_diff>
--- a/bom/schlieren-bom.xlsx
+++ b/bom/schlieren-bom.xlsx
@@ -7,11 +7,11 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Summary" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="BOM" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="BOM" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Summary" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'BOM'!$A$1:$L$141</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'BOM'!$A$1:$L$141</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -30,10 +30,10 @@
     </font>
     <font>
       <b val="1"/>
-      <sz val="14"/>
     </font>
     <font>
       <b val="1"/>
+      <sz val="14"/>
     </font>
   </fonts>
   <fills count="2">
@@ -474,387 +474,6 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E29"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="22" customWidth="1" min="1" max="1"/>
-    <col width="60" customWidth="1" min="2" max="2"/>
-    <col width="18" customWidth="1" min="4" max="4"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>iPhone Schlieren BOM / Procurement Tracker</t>
-        </is>
-      </c>
-    </row>
-    <row r="2"/>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Canonical workbook</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Generated from bom/bom.csv in Git. Edits made here count only once reconciled into the CSV (reconcile-bom).</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Design baseline</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>docs/design/ fragments in Git (consolidated: schlieren-design).</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Quantity model</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Qty is the numeric required/allocated amount for that BOM line; package counts do not belong in Qty.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Blank Qty</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>Quantity is not yet frozen or the item is an as-required consumable/working-stock line.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Package fields</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>Package Size is units per Purchase Unit where known. Unknown vendor package sizes are intentionally blank.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>Entry count</t>
-        </is>
-      </c>
-      <c r="B8">
-        <f>COUNTA(BOM!A:A)-1</f>
-        <v/>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="2" t="inlineStr">
-        <is>
-          <t>Procurement state</t>
-        </is>
-      </c>
-      <c r="B10" s="2" t="inlineStr">
-        <is>
-          <t>Entries</t>
-        </is>
-      </c>
-      <c r="D10" s="2" t="inlineStr">
-        <is>
-          <t>Subsystem</t>
-        </is>
-      </c>
-      <c r="E10" s="2" t="inlineStr">
-        <is>
-          <t>Entries</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>In hand</t>
-        </is>
-      </c>
-      <c r="B11">
-        <f>COUNTIF(BOM!J:J,"In hand")</f>
-        <v/>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>Tabletop frame</t>
-        </is>
-      </c>
-      <c r="E11">
-        <f>COUNTIF(BOM!B:B,D11)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>On order</t>
-        </is>
-      </c>
-      <c r="B12">
-        <f>COUNTIF(BOM!J:J,"On order")</f>
-        <v/>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>Optical supports</t>
-        </is>
-      </c>
-      <c r="E12">
-        <f>COUNTIF(BOM!B:B,D12)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>To procure</t>
-        </is>
-      </c>
-      <c r="B13">
-        <f>COUNTIF(BOM!J:J,"To procure")</f>
-        <v/>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>Light source</t>
-        </is>
-      </c>
-      <c r="E13">
-        <f>COUNTIF(BOM!B:B,D13)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>Specified</t>
-        </is>
-      </c>
-      <c r="B14">
-        <f>COUNTIF(BOM!J:J,"Specified")</f>
-        <v/>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>Source slit</t>
-        </is>
-      </c>
-      <c r="E14">
-        <f>COUNTIF(BOM!B:B,D14)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>CAD ready</t>
-        </is>
-      </c>
-      <c r="B15">
-        <f>COUNTIF(BOM!J:J,"CAD ready")</f>
-        <v/>
-      </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>Carriages</t>
-        </is>
-      </c>
-      <c r="E15">
-        <f>COUNTIF(BOM!B:B,D15)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>CAD open</t>
-        </is>
-      </c>
-      <c r="B16">
-        <f>COUNTIF(BOM!J:J,"CAD open")</f>
-        <v/>
-      </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>Cassettes</t>
-        </is>
-      </c>
-      <c r="E16">
-        <f>COUNTIF(BOM!B:B,D16)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="17">
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>Imager</t>
-        </is>
-      </c>
-      <c r="E17">
-        <f>COUNTIF(BOM!B:B,D17)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="18">
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>Mirror cell</t>
-        </is>
-      </c>
-      <c r="E18">
-        <f>COUNTIF(BOM!B:B,D18)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="19">
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>Shop supplies</t>
-        </is>
-      </c>
-      <c r="E19">
-        <f>COUNTIF(BOM!B:B,D19)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="20">
-      <c r="D20" t="inlineStr">
-        <is>
-          <t>Unused</t>
-        </is>
-      </c>
-      <c r="E20">
-        <f>COUNTIF(BOM!B:B,D20)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>Rollup key</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>Use Vendor + SKU for procurement rollups.</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>Shared parts</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>Keep separate BOM rows for separate subsystem allocations; roll them up by Vendor+SKU.</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>Package math</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>Vendor/SKU rollups may sum Qty and divide by Package Size where Package Size is known.</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>Spare/surplus</t>
-        </is>
-      </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>Unavoidable package surplus is not added to required Qty; track it in procurement/inventory rollups or notes.</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>Data rule</t>
-        </is>
-      </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>Do not insert subsystem header or separator rows inside the BOM table.</t>
-        </is>
-      </c>
-    </row>
-    <row r="26"/>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>Specified</t>
-        </is>
-      </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>Part defined by the design; vendor, SKU, or quantity still to be confirmed.</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>CAD ready</t>
-        </is>
-      </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>Printed part with a build123d model in src/schlieren/parts/; ready to print and fit-test.</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>CAD open</t>
-        </is>
-      </c>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>Printed part whose custom geometry is still to be designed.</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
   <dimension ref="A1:L141"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -873,62 +492,62 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="2" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>ID</t>
         </is>
       </c>
-      <c r="B1" s="2" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Subsystem</t>
         </is>
       </c>
-      <c r="C1" s="2" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Qty</t>
         </is>
       </c>
-      <c r="D1" s="2" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Item</t>
         </is>
       </c>
-      <c r="E1" s="2" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Purpose</t>
         </is>
       </c>
-      <c r="F1" s="2" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Vendor</t>
         </is>
       </c>
-      <c r="G1" s="2" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>SKU</t>
         </is>
       </c>
-      <c r="H1" s="2" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Pkg Size</t>
         </is>
       </c>
-      <c r="I1" s="2" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Purchase Unit</t>
         </is>
       </c>
-      <c r="J1" s="2" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Procurement state</t>
         </is>
       </c>
-      <c r="K1" s="2" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Source section</t>
         </is>
       </c>
-      <c r="L1" s="2" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
@@ -6599,7 +6218,7 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>SHP-002</t>
+          <t>SHP-003</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
@@ -6612,17 +6231,17 @@
       </c>
       <c r="D110" t="inlineStr">
         <is>
-          <t>Heat-set installation tip</t>
+          <t>Optical spanner wrench</t>
         </is>
       </c>
       <c r="F110" t="inlineStr">
         <is>
-          <t>McMaster</t>
+          <t>Amazon</t>
         </is>
       </c>
       <c r="G110" t="inlineStr">
         <is>
-          <t>92160A327</t>
+          <t>B0CKSL364Q</t>
         </is>
       </c>
       <c r="H110" t="n">
@@ -6636,18 +6255,13 @@
       <c r="J110" t="inlineStr">
         <is>
           <t>In hand</t>
-        </is>
-      </c>
-      <c r="K110" t="inlineStr">
-        <is>
-          <t>§9.7</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>SHP-003</t>
+          <t>SHP-004</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
@@ -6660,7 +6274,12 @@
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>Optical spanner wrench</t>
+          <t>Metric feeler gauge set</t>
+        </is>
+      </c>
+      <c r="E111" t="inlineStr">
+        <is>
+          <t>Source-slit blade spacing</t>
         </is>
       </c>
       <c r="F111" t="inlineStr">
@@ -6670,7 +6289,7 @@
       </c>
       <c r="G111" t="inlineStr">
         <is>
-          <t>B0CKSL364Q</t>
+          <t>B07XPD9L1C</t>
         </is>
       </c>
       <c r="H111" t="n">
@@ -6684,13 +6303,18 @@
       <c r="J111" t="inlineStr">
         <is>
           <t>In hand</t>
+        </is>
+      </c>
+      <c r="K111" t="inlineStr">
+        <is>
+          <t>§7.4</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>SHP-004</t>
+          <t>SHP-005</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
@@ -6703,22 +6327,22 @@
       </c>
       <c r="D112" t="inlineStr">
         <is>
-          <t>Metric feeler gauge set</t>
+          <t>M2 tap</t>
         </is>
       </c>
       <c r="E112" t="inlineStr">
         <is>
-          <t>Source-slit blade spacing</t>
+          <t>LED board mounting into SM1CP2M cap</t>
         </is>
       </c>
       <c r="F112" t="inlineStr">
         <is>
-          <t>Amazon</t>
+          <t>McMaster</t>
         </is>
       </c>
       <c r="G112" t="inlineStr">
         <is>
-          <t>B07XPD9L1C</t>
+          <t>8305A78</t>
         </is>
       </c>
       <c r="H112" t="n">
@@ -6736,14 +6360,19 @@
       </c>
       <c r="K112" t="inlineStr">
         <is>
-          <t>§7.4</t>
+          <t>§6.4</t>
+        </is>
+      </c>
+      <c r="L112" t="inlineStr">
+        <is>
+          <t>Plug chamfer; sufficient for the through M2 holes.</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>SHP-005</t>
+          <t>SHP-006</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
@@ -6756,12 +6385,12 @@
       </c>
       <c r="D113" t="inlineStr">
         <is>
-          <t>M2 tap</t>
+          <t>M2 tap drill, 1.6mm</t>
         </is>
       </c>
       <c r="E113" t="inlineStr">
         <is>
-          <t>LED board mounting into SM1CP2M cap</t>
+          <t>LED mounting</t>
         </is>
       </c>
       <c r="F113" t="inlineStr">
@@ -6771,7 +6400,7 @@
       </c>
       <c r="G113" t="inlineStr">
         <is>
-          <t>8305A78</t>
+          <t>2979N13</t>
         </is>
       </c>
       <c r="H113" t="n">
@@ -6790,18 +6419,13 @@
       <c r="K113" t="inlineStr">
         <is>
           <t>§6.4</t>
-        </is>
-      </c>
-      <c r="L113" t="inlineStr">
-        <is>
-          <t>Plug chamfer; sufficient for the through M2 holes.</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>SHP-006</t>
+          <t>SHP-011</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
@@ -6814,12 +6438,12 @@
       </c>
       <c r="D114" t="inlineStr">
         <is>
-          <t>M2 tap drill, 1.6mm</t>
+          <t>Loctite 4061 cyanoacrylate adhesive, 0.7 fl. oz., low viscosity (~20 cP)</t>
         </is>
       </c>
       <c r="E114" t="inlineStr">
         <is>
-          <t>LED mounting</t>
+          <t>Plywood fiber conditioning and localized tack bonds</t>
         </is>
       </c>
       <c r="F114" t="inlineStr">
@@ -6829,7 +6453,7 @@
       </c>
       <c r="G114" t="inlineStr">
         <is>
-          <t>2979N13</t>
+          <t>1818A45</t>
         </is>
       </c>
       <c r="H114" t="n">
@@ -6847,14 +6471,19 @@
       </c>
       <c r="K114" t="inlineStr">
         <is>
-          <t>§6.4</t>
+          <t>§§8.3, 8.4, 8.7, 10.4</t>
+        </is>
+      </c>
+      <c r="L114" t="inlineStr">
+        <is>
+          <t>Use sparingly: wick into Baltic-birch fibers for the spherical-washer sockets (§10.4); needle-sized drops retain the carriage magnet pad and datum pins (§§8.3, 8.4) and keep the cassette clamp-bar screws captive (§8.7). No accelerator required.</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>SHP-011</t>
+          <t>SHP-012</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
@@ -6867,22 +6496,22 @@
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t>Loctite 4061 cyanoacrylate adhesive, 0.7 fl. oz., low viscosity (~20 cP)</t>
+          <t>UHMW Sheet 1/8" x 12" x 12"</t>
         </is>
       </c>
       <c r="E115" t="inlineStr">
         <is>
-          <t>Plywood fiber conditioning and localized tack bonds</t>
+          <t>Mirror mount releasing assembly surface</t>
         </is>
       </c>
       <c r="F115" t="inlineStr">
         <is>
-          <t>McMaster</t>
+          <t>US Plastics</t>
         </is>
       </c>
       <c r="G115" t="inlineStr">
         <is>
-          <t>1818A45</t>
+          <t>46489</t>
         </is>
       </c>
       <c r="H115" t="n">
@@ -6900,19 +6529,14 @@
       </c>
       <c r="K115" t="inlineStr">
         <is>
-          <t>§§8.3, 8.4, 8.7, 10.4</t>
-        </is>
-      </c>
-      <c r="L115" t="inlineStr">
-        <is>
-          <t>Use sparingly: wick into Baltic-birch fibers for the spherical-washer sockets (§10.4); needle-sized drops retain the carriage magnet pad and datum pins (§§8.3, 8.4) and keep the cassette clamp-bar screws captive (§8.7). No accelerator required.</t>
+          <t>§10.6</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>SHP-012</t>
+          <t>SHP-014</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
@@ -6925,22 +6549,22 @@
       </c>
       <c r="D116" t="inlineStr">
         <is>
-          <t>UHMW Sheet 1/8" x 12" x 12"</t>
+          <t>West System G/Flex 650 Epoxy Adhesive, 2 x 4 oz</t>
         </is>
       </c>
       <c r="E116" t="inlineStr">
         <is>
-          <t>Mirror mount releasing assembly surface</t>
+          <t>Mirror cell adjuster sleeves, spring seat washer tack</t>
         </is>
       </c>
       <c r="F116" t="inlineStr">
         <is>
-          <t>US Plastics</t>
+          <t>Amazon</t>
         </is>
       </c>
       <c r="G116" t="inlineStr">
         <is>
-          <t>46489</t>
+          <t>B002IZFPQE</t>
         </is>
       </c>
       <c r="H116" t="n">
@@ -6958,14 +6582,14 @@
       </c>
       <c r="K116" t="inlineStr">
         <is>
-          <t>§10.6</t>
+          <t>§10.2</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>SHP-014</t>
+          <t>SHP-015</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
@@ -6978,22 +6602,22 @@
       </c>
       <c r="D117" t="inlineStr">
         <is>
-          <t>West System G/Flex 650 Epoxy Adhesive, 2 x 4 oz</t>
+          <t>Silicone grease, clear, NLGI 1</t>
         </is>
       </c>
       <c r="E117" t="inlineStr">
         <is>
-          <t>Mirror cell adjuster sleeves, spring seat washer tack</t>
+          <t>PLA carriage sliding-interface lubricant</t>
         </is>
       </c>
       <c r="F117" t="inlineStr">
         <is>
-          <t>Amazon</t>
+          <t>McMaster</t>
         </is>
       </c>
       <c r="G117" t="inlineStr">
         <is>
-          <t>B002IZFPQE</t>
+          <t>1418K51</t>
         </is>
       </c>
       <c r="H117" t="n">
@@ -7011,14 +6635,19 @@
       </c>
       <c r="K117" t="inlineStr">
         <is>
-          <t>§10.2</t>
+          <t>§8.4</t>
+        </is>
+      </c>
+      <c r="L117" t="inlineStr">
+        <is>
+          <t>Use only a trace film on dressed PLA-on-PLA sliding interfaces.</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>SHP-015</t>
+          <t>SHP-016</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
@@ -7031,22 +6660,22 @@
       </c>
       <c r="D118" t="inlineStr">
         <is>
-          <t>Silicone grease, clear, NLGI 1</t>
+          <t>Dynatex 159375 White Lithium Grease NLGI 2</t>
         </is>
       </c>
       <c r="E118" t="inlineStr">
         <is>
-          <t>PLA carriage sliding-interface lubricant</t>
+          <t>Light grease for mirror-cell spherical washer interfaces</t>
         </is>
       </c>
       <c r="F118" t="inlineStr">
         <is>
-          <t>McMaster</t>
+          <t>Amazon</t>
         </is>
       </c>
       <c r="G118" t="inlineStr">
         <is>
-          <t>1418K51</t>
+          <t>B009XE8M3G</t>
         </is>
       </c>
       <c r="H118" t="n">
@@ -7059,24 +6688,24 @@
       </c>
       <c r="J118" t="inlineStr">
         <is>
-          <t>In hand</t>
+          <t>On order</t>
         </is>
       </c>
       <c r="K118" t="inlineStr">
         <is>
-          <t>§8.4</t>
+          <t>§10.4</t>
         </is>
       </c>
       <c r="L118" t="inlineStr">
         <is>
-          <t>Use only a trace film on dressed PLA-on-PLA sliding interfaces.</t>
+          <t>Small tube to transport with the apparatus.</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>SHP-016</t>
+          <t>SHP-017</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
@@ -7089,22 +6718,22 @@
       </c>
       <c r="D119" t="inlineStr">
         <is>
-          <t>Dynatex 159375 White Lithium Grease NLGI 2</t>
+          <t>1/2" Forstner bit, standard-point smooth-finish</t>
         </is>
       </c>
       <c r="E119" t="inlineStr">
         <is>
-          <t>Light grease for mirror-cell spherical washer interfaces</t>
+          <t>Spherical-washer counterbores</t>
         </is>
       </c>
       <c r="F119" t="inlineStr">
         <is>
-          <t>Amazon</t>
+          <t>McMaster</t>
         </is>
       </c>
       <c r="G119" t="inlineStr">
         <is>
-          <t>B009XE8M3G</t>
+          <t>2890A56</t>
         </is>
       </c>
       <c r="H119" t="n">
@@ -7117,7 +6746,7 @@
       </c>
       <c r="J119" t="inlineStr">
         <is>
-          <t>On order</t>
+          <t>In hand</t>
         </is>
       </c>
       <c r="K119" t="inlineStr">
@@ -7127,14 +6756,14 @@
       </c>
       <c r="L119" t="inlineStr">
         <is>
-          <t>Small tube to transport with the apparatus.</t>
+          <t>Use in drill press for shallow close-fit spherical-washer sockets; test in scrap Baltic birch before cutting final plate.</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>SHP-017</t>
+          <t>SHP-018</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
@@ -7147,12 +6776,12 @@
       </c>
       <c r="D120" t="inlineStr">
         <is>
-          <t>1/2" Forstner bit, standard-point smooth-finish</t>
+          <t>5/8" Forstner bit, standard-point smooth-finish</t>
         </is>
       </c>
       <c r="E120" t="inlineStr">
         <is>
-          <t>Spherical-washer counterbores</t>
+          <t>Spring-seat washer counterbores</t>
         </is>
       </c>
       <c r="F120" t="inlineStr">
@@ -7162,7 +6791,7 @@
       </c>
       <c r="G120" t="inlineStr">
         <is>
-          <t>2890A56</t>
+          <t>2890A58</t>
         </is>
       </c>
       <c r="H120" t="n">
@@ -7180,19 +6809,19 @@
       </c>
       <c r="K120" t="inlineStr">
         <is>
-          <t>§10.4</t>
+          <t>§10.3</t>
         </is>
       </c>
       <c r="L120" t="inlineStr">
         <is>
-          <t>Use in drill press for shallow close-fit spherical-washer sockets; test in scrap Baltic birch before cutting final plate.</t>
+          <t>Use in drill press for shallow spring-seat-washer registration counterbores; test depth/fit in scrap first.</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>SHP-018</t>
+          <t>SHP-019</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
@@ -7205,12 +6834,12 @@
       </c>
       <c r="D121" t="inlineStr">
         <is>
-          <t>5/8" Forstner bit, standard-point smooth-finish</t>
+          <t>M4 × 0.7 high-speed-steel plug-chamfer hex-bit tap</t>
         </is>
       </c>
       <c r="E121" t="inlineStr">
         <is>
-          <t>Spring-seat washer counterbores</t>
+          <t>Tap CAMVATE quick-release plate mounting holes</t>
         </is>
       </c>
       <c r="F121" t="inlineStr">
@@ -7220,7 +6849,7 @@
       </c>
       <c r="G121" t="inlineStr">
         <is>
-          <t>2890A58</t>
+          <t>1021N23</t>
         </is>
       </c>
       <c r="H121" t="n">
@@ -7238,19 +6867,19 @@
       </c>
       <c r="K121" t="inlineStr">
         <is>
-          <t>§10.3</t>
+          <t>§10.9</t>
         </is>
       </c>
       <c r="L121" t="inlineStr">
         <is>
-          <t>Use in drill press for shallow spring-seat-washer registration counterbores; test depth/fit in scrap first.</t>
+          <t>Use with the 3.3 mm tap drill (SHP-020); hole locations in §10.9.</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>SHP-019</t>
+          <t>SHP-020</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
@@ -7263,12 +6892,12 @@
       </c>
       <c r="D122" t="inlineStr">
         <is>
-          <t>M4 × 0.7 high-speed-steel plug-chamfer hex-bit tap</t>
+          <t>3.3 mm black-oxide HSS jobber-length drill bit</t>
         </is>
       </c>
       <c r="E122" t="inlineStr">
         <is>
-          <t>Tap CAMVATE quick-release plate mounting holes</t>
+          <t>M4 × 0.7 tap drill for CAMVATE quick-release plate; M3 heatsink clearance holes</t>
         </is>
       </c>
       <c r="F122" t="inlineStr">
@@ -7278,7 +6907,7 @@
       </c>
       <c r="G122" t="inlineStr">
         <is>
-          <t>1021N23</t>
+          <t>2958A64</t>
         </is>
       </c>
       <c r="H122" t="n">
@@ -7296,19 +6925,19 @@
       </c>
       <c r="K122" t="inlineStr">
         <is>
-          <t>§10.9</t>
+          <t>§§6.4, 10.9</t>
         </is>
       </c>
       <c r="L122" t="inlineStr">
         <is>
-          <t>Use with the 3.3 mm tap drill (SHP-020); hole locations in §10.9.</t>
+          <t>Standard 3.3 mm tap-drill size for M4 × 0.7. Also drills the Ø3.3 M3 clearance holes in the heatsink base (§6.4).</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>SHP-020</t>
+          <t>SHP-021</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
@@ -7321,12 +6950,12 @@
       </c>
       <c r="D123" t="inlineStr">
         <is>
-          <t>3.3 mm black-oxide HSS jobber-length drill bit</t>
+          <t>Loctite 243 medium-strength removable threadlocker, 0.34 fl. oz.</t>
         </is>
       </c>
       <c r="E123" t="inlineStr">
         <is>
-          <t>M4 × 0.7 tap drill for CAMVATE quick-release plate; M3 heatsink clearance holes</t>
+          <t>Removable thread retention for quick-release plate mounting screws</t>
         </is>
       </c>
       <c r="F123" t="inlineStr">
@@ -7336,7 +6965,7 @@
       </c>
       <c r="G123" t="inlineStr">
         <is>
-          <t>2958A64</t>
+          <t>91458A115</t>
         </is>
       </c>
       <c r="H123" t="n">
@@ -7354,19 +6983,19 @@
       </c>
       <c r="K123" t="inlineStr">
         <is>
-          <t>§§6.4, 10.9</t>
+          <t>§10.9</t>
         </is>
       </c>
       <c r="L123" t="inlineStr">
         <is>
-          <t>Standard 3.3 mm tap-drill size for M4 × 0.7. Also drills the Ø3.3 M3 clearance holes in the heatsink base (§6.4).</t>
+          <t>Apply only after the screw fit is confirmed (the hole sizes are provisional, §10.9); preferred over high-strength Loctite 271 for this serviceable joint.</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>SHP-021</t>
+          <t>SHP-022</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
@@ -7379,22 +7008,22 @@
       </c>
       <c r="D124" t="inlineStr">
         <is>
-          <t>Loctite 243 medium-strength removable threadlocker, 0.34 fl. oz.</t>
+          <t>Rosco Photofoil matte black aluminum wrap, 12"x10'</t>
         </is>
       </c>
       <c r="E124" t="inlineStr">
         <is>
-          <t>Removable thread retention for quick-release plate mounting screws</t>
+          <t>Opaque masking / thin-sheet cutoff experiments</t>
         </is>
       </c>
       <c r="F124" t="inlineStr">
         <is>
-          <t>McMaster</t>
+          <t>Fullcompass</t>
         </is>
       </c>
       <c r="G124" t="inlineStr">
         <is>
-          <t>91458A115</t>
+          <t>01001-1210</t>
         </is>
       </c>
       <c r="H124" t="n">
@@ -7402,7 +7031,7 @@
       </c>
       <c r="I124" t="inlineStr">
         <is>
-          <t>each</t>
+          <t>pack</t>
         </is>
       </c>
       <c r="J124" t="inlineStr">
@@ -7412,19 +7041,19 @@
       </c>
       <c r="K124" t="inlineStr">
         <is>
-          <t>§10.9</t>
+          <t>§§8.6, 8.7</t>
         </is>
       </c>
       <c r="L124" t="inlineStr">
         <is>
-          <t>Apply only after the screw fit is confirmed (the hole sizes are provisional, §10.9); preferred over high-strength Loctite 271 for this serviceable joint.</t>
+          <t>Retained as general shop stock for opaque masking and thin-sheet cutoff experiments.</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>SHP-022</t>
+          <t>SHP-023</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
@@ -7437,22 +7066,22 @@
       </c>
       <c r="D125" t="inlineStr">
         <is>
-          <t>Rosco Photofoil matte black aluminum wrap, 12"x10'</t>
+          <t>M3 × 0.5 high-speed-steel plug-chamfer tap, 5/8" thread length</t>
         </is>
       </c>
       <c r="E125" t="inlineStr">
         <is>
-          <t>Opaque masking / thin-sheet cutoff experiments</t>
+          <t>Tap through M3 heatsink-screw holes in SM1CP2M cap</t>
         </is>
       </c>
       <c r="F125" t="inlineStr">
         <is>
-          <t>Fullcompass</t>
+          <t>McMaster</t>
         </is>
       </c>
       <c r="G125" t="inlineStr">
         <is>
-          <t>01001-1210</t>
+          <t>8305A32</t>
         </is>
       </c>
       <c r="H125" t="n">
@@ -7460,7 +7089,7 @@
       </c>
       <c r="I125" t="inlineStr">
         <is>
-          <t>pack</t>
+          <t>each</t>
         </is>
       </c>
       <c r="J125" t="inlineStr">
@@ -7470,19 +7099,19 @@
       </c>
       <c r="K125" t="inlineStr">
         <is>
-          <t>§§8.6, 8.7</t>
+          <t>§6.4</t>
         </is>
       </c>
       <c r="L125" t="inlineStr">
         <is>
-          <t>Retained as general shop stock for opaque masking and thin-sheet cutoff experiments.</t>
+          <t>All holes are through holes, so a plug chamfer is enough; no bottoming tap needed. Use with the 2.5 mm tap drill (SHP-025).</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>SHP-023</t>
+          <t>SHP-025</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
@@ -7495,12 +7124,12 @@
       </c>
       <c r="D126" t="inlineStr">
         <is>
-          <t>M3 × 0.5 high-speed-steel plug-chamfer tap, 5/8" thread length</t>
+          <t>2.5 mm TiN-coated HSS short-length drill bit, 43 mm overall</t>
         </is>
       </c>
       <c r="E126" t="inlineStr">
         <is>
-          <t>Tap through M3 heatsink-screw holes in SM1CP2M cap</t>
+          <t>M3 tap drill for through holes in SM1CP2M cap</t>
         </is>
       </c>
       <c r="F126" t="inlineStr">
@@ -7510,7 +7139,7 @@
       </c>
       <c r="G126" t="inlineStr">
         <is>
-          <t>8305A32</t>
+          <t>2979N15</t>
         </is>
       </c>
       <c r="H126" t="n">
@@ -7533,14 +7162,14 @@
       </c>
       <c r="L126" t="inlineStr">
         <is>
-          <t>All holes are through holes, so a plug chamfer is enough; no bottoming tap needed. Use with the 2.5 mm tap drill (SHP-025).</t>
+          <t>Short-length stub drill for rigid drilling in the thin cap; same series as the 1.6 mm drill SHP-006.</t>
         </is>
       </c>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>SHP-025</t>
+          <t>SHP-026</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
@@ -7553,12 +7182,12 @@
       </c>
       <c r="D127" t="inlineStr">
         <is>
-          <t>2.5 mm TiN-coated HSS short-length drill bit, 43 mm overall</t>
+          <t>2.0 mm uncoated HSS short-length drill bit, 38 mm overall</t>
         </is>
       </c>
       <c r="E127" t="inlineStr">
         <is>
-          <t>M3 tap drill for through holes in SM1CP2M cap</t>
+          <t>Lead holes through SM1CP2M cap and heatsink base</t>
         </is>
       </c>
       <c r="F127" t="inlineStr">
@@ -7568,7 +7197,7 @@
       </c>
       <c r="G127" t="inlineStr">
         <is>
-          <t>2979N15</t>
+          <t>2979N14</t>
         </is>
       </c>
       <c r="H127" t="n">
@@ -7581,7 +7210,7 @@
       </c>
       <c r="J127" t="inlineStr">
         <is>
-          <t>In hand</t>
+          <t>To procure</t>
         </is>
       </c>
       <c r="K127" t="inlineStr">
@@ -7591,14 +7220,14 @@
       </c>
       <c r="L127" t="inlineStr">
         <is>
-          <t>Short-length stub drill for rigid drilling in the thin cap; same series as the 1.6 mm drill SHP-006.</t>
+          <t>Same series as the 1.6 mm drill SHP-006. Deferred, not in the current order: lead hole size is provisional (§6.4), and the 2.5 mm drill SHP-025 may cut the lead holes instead. Decide after measuring the pigtail insulation.</t>
         </is>
       </c>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>SHP-026</t>
+          <t>SHP-027</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
@@ -7611,12 +7240,12 @@
       </c>
       <c r="D128" t="inlineStr">
         <is>
-          <t>2.0 mm uncoated HSS short-length drill bit, 38 mm overall</t>
+          <t>Heat-set insert installation tip set, 8 pieces (M2 to M8) with 1/4 in shank adapter</t>
         </is>
       </c>
       <c r="E128" t="inlineStr">
         <is>
-          <t>Lead holes through SM1CP2M cap and heatsink base</t>
+          <t>Fits a Hakko 900M-style iron; M5 tip sets the CAM-005 inserts</t>
         </is>
       </c>
       <c r="F128" t="inlineStr">
@@ -7626,7 +7255,7 @@
       </c>
       <c r="G128" t="inlineStr">
         <is>
-          <t>2979N14</t>
+          <t>8915N111</t>
         </is>
       </c>
       <c r="H128" t="n">
@@ -7639,24 +7268,24 @@
       </c>
       <c r="J128" t="inlineStr">
         <is>
-          <t>To procure</t>
+          <t>In hand</t>
         </is>
       </c>
       <c r="K128" t="inlineStr">
         <is>
-          <t>§6.4</t>
+          <t>§9.7</t>
         </is>
       </c>
       <c r="L128" t="inlineStr">
         <is>
-          <t>Same series as the 1.6 mm drill SHP-006. Deferred, not in the current order: lead hole size is provisional (§6.4), and the 2.5 mm drill SHP-025 may cut the lead holes instead. Decide after measuring the pigtail insulation.</t>
+          <t>Listed for Hakko 900M. The M5 tip has a female threaded connection and mounts through the included adapter, which fits the Hakko iron (confirmed). Replaces the 1/4 in plug tip UNU-011. Used with the Hakko iron SHP-028; set PLA installation near 200–230 °C (typical for PLA; confirm on a scrap print), no higher than 250 °C.</t>
         </is>
       </c>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>SHP-027</t>
+          <t>SHP-028</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
@@ -7669,22 +7298,17 @@
       </c>
       <c r="D129" t="inlineStr">
         <is>
-          <t>Heat-set insert installation tip set, 8 pieces (M2 to M8) with 1/4 in shank adapter</t>
+          <t>Hakko FX888DX-10 soldering station</t>
         </is>
       </c>
       <c r="E129" t="inlineStr">
         <is>
-          <t>Fits a Hakko 900M-style iron; M5 tip sets the CAM-005 inserts</t>
-        </is>
-      </c>
-      <c r="F129" t="inlineStr">
-        <is>
-          <t>McMaster</t>
+          <t>Heat-set insert installation (CAM-005)</t>
         </is>
       </c>
       <c r="G129" t="inlineStr">
         <is>
-          <t>8915N111</t>
+          <t>FX888DX-10</t>
         </is>
       </c>
       <c r="H129" t="n">
@@ -7707,14 +7331,14 @@
       </c>
       <c r="L129" t="inlineStr">
         <is>
-          <t>Listed for Hakko 900M. The M5 tip has a female threaded connection and mounts through the included adapter, which fits the Hakko iron (confirmed); how it mates with SHP-002 is unverified. Used with the Hakko iron SHP-028; set PLA installation near 200–230 °C (typical for PLA; confirm on a scrap print), no higher than 250 °C.</t>
+          <t>Vendor not recorded here. Takes Hakko T18 (900M-style) tips. Drives the SHP-027 tip set; the SHP-027 adapter fits the iron (confirmed).</t>
         </is>
       </c>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>SHP-028</t>
+          <t>SHP-029</t>
         </is>
       </c>
       <c r="B130" t="inlineStr">
@@ -7727,17 +7351,22 @@
       </c>
       <c r="D130" t="inlineStr">
         <is>
-          <t>Hakko FX888DX-10 soldering station</t>
+          <t>Hole-starting cobalt-steel drill bit, uncoated, 90° point, 1/8" size</t>
         </is>
       </c>
       <c r="E130" t="inlineStr">
         <is>
-          <t>Heat-set insert installation (CAM-005)</t>
+          <t>Spot hole locations in the SM1CP2M cap and heatsink base before drilling</t>
+        </is>
+      </c>
+      <c r="F130" t="inlineStr">
+        <is>
+          <t>McMaster</t>
         </is>
       </c>
       <c r="G130" t="inlineStr">
         <is>
-          <t>FX888DX-10</t>
+          <t>27445A201</t>
         </is>
       </c>
       <c r="H130" t="n">
@@ -7755,19 +7384,19 @@
       </c>
       <c r="K130" t="inlineStr">
         <is>
-          <t>§9.7</t>
+          <t>§6.4</t>
         </is>
       </c>
       <c r="L130" t="inlineStr">
         <is>
-          <t>Vendor not recorded here. Takes Hakko T18 (900M-style) tips. Drives the SHP-027 tip set; the SHP-027 adapter fits the iron (confirmed); fit of SHP-002 unverified.</t>
+          <t>1/8" shank fits the Dremel 4486 chuck (1/8" maximum). Use before the 1.6, 2.0, 2.5, and 3.3 mm drills.</t>
         </is>
       </c>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>SHP-029</t>
+          <t>SHP-030</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
@@ -7780,12 +7409,12 @@
       </c>
       <c r="D131" t="inlineStr">
         <is>
-          <t>Hole-starting cobalt-steel drill bit, uncoated, 90° point, 1/8" size</t>
+          <t>Center drill, high-speed steel, 60° countersink, trade size 1, 1-1/4" overall length</t>
         </is>
       </c>
       <c r="E131" t="inlineStr">
         <is>
-          <t>Spot hole locations in the SM1CP2M cap and heatsink base before drilling</t>
+          <t>Backup hole spotter; spots the cap and heatsink holes</t>
         </is>
       </c>
       <c r="F131" t="inlineStr">
@@ -7795,7 +7424,7 @@
       </c>
       <c r="G131" t="inlineStr">
         <is>
-          <t>27445A201</t>
+          <t>2915A11</t>
         </is>
       </c>
       <c r="H131" t="n">
@@ -7818,46 +7447,43 @@
       </c>
       <c r="L131" t="inlineStr">
         <is>
-          <t>1/8" shank fits the Dremel 4486 chuck (1/8" maximum). Use before the 1.6, 2.0, 2.5, and 3.3 mm drills.</t>
+          <t>3/64" pilot, 1/8" body; fits the Dremel 4486 chuck. Spare for SHP-029.</t>
         </is>
       </c>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>SHP-030</t>
+          <t>UNU-001</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>Shop supplies</t>
-        </is>
-      </c>
-      <c r="C132" t="n">
-        <v>1</v>
+          <t>Unused</t>
+        </is>
       </c>
       <c r="D132" t="inlineStr">
         <is>
-          <t>Center drill, high-speed steel, 60° countersink, trade size 1, 1-1/4" overall length</t>
+          <t>Heatsink, 6063-T5 non-anodized aluminum, Ø55 mm x 20 mm.</t>
         </is>
       </c>
       <c r="E132" t="inlineStr">
         <is>
-          <t>Backup hole spotter; spots the cap and heatsink holes</t>
+          <t>Existing spare stock; former LED heatsink</t>
         </is>
       </c>
       <c r="F132" t="inlineStr">
         <is>
-          <t>McMaster</t>
+          <t>HeatsinkOnline</t>
         </is>
       </c>
       <c r="G132" t="inlineStr">
         <is>
-          <t>2915A11</t>
+          <t>64ASL-8-55</t>
         </is>
       </c>
       <c r="H132" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="I132" t="inlineStr">
         <is>
@@ -7869,21 +7495,16 @@
           <t>In hand</t>
         </is>
       </c>
-      <c r="K132" t="inlineStr">
-        <is>
-          <t>§6.4</t>
-        </is>
-      </c>
       <c r="L132" t="inlineStr">
         <is>
-          <t>3/64" pilot, 1/8" body; fits the Dremel 4486 chuck. Spare for SHP-029.</t>
+          <t>No longer allocated after the threaded SM1 LED module decision; replaced by LGT-018 (Alpha CN40-40B). Four in hand retained as spares.</t>
         </is>
       </c>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>UNU-001</t>
+          <t>UNU-002</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
@@ -7893,26 +7514,26 @@
       </c>
       <c r="D133" t="inlineStr">
         <is>
-          <t>Heatsink, 6063-T5 non-anodized aluminum, Ø55 mm x 20 mm.</t>
+          <t>SM1 lens tube, 1.50" Thread Depth</t>
         </is>
       </c>
       <c r="E133" t="inlineStr">
         <is>
-          <t>Existing spare stock; former LED heatsink</t>
+          <t>Existing stock; former carriage-tube allocation</t>
         </is>
       </c>
       <c r="F133" t="inlineStr">
         <is>
-          <t>HeatsinkOnline</t>
+          <t>Thorlabs</t>
         </is>
       </c>
       <c r="G133" t="inlineStr">
         <is>
-          <t>64ASL-8-55</t>
+          <t>SM1L15</t>
         </is>
       </c>
       <c r="H133" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="I133" t="inlineStr">
         <is>
@@ -7926,14 +7547,14 @@
       </c>
       <c r="L133" t="inlineStr">
         <is>
-          <t>No longer allocated after the threaded SM1 LED module decision; replaced by LGT-018 (Alpha CN40-40B). Four in hand retained as spares.</t>
+          <t>No longer allocated: the cutoff carriage mounts in the SM1RC/M on an integral printed spigot (§8.1); both tubes in hand are spare.</t>
         </is>
       </c>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>UNU-002</t>
+          <t>UNU-003</t>
         </is>
       </c>
       <c r="B134" t="inlineStr">
@@ -7943,22 +7564,22 @@
       </c>
       <c r="D134" t="inlineStr">
         <is>
-          <t>SM1 lens tube, 1.50" Thread Depth</t>
+          <t>4 mm × 45 mm shoulder screw, 18-8 SS</t>
         </is>
       </c>
       <c r="E134" t="inlineStr">
         <is>
-          <t>Existing stock; former carriage-tube allocation</t>
+          <t>Existing stock; former spring guide / retract handle</t>
         </is>
       </c>
       <c r="F134" t="inlineStr">
         <is>
-          <t>Thorlabs</t>
+          <t>McMaster</t>
         </is>
       </c>
       <c r="G134" t="inlineStr">
         <is>
-          <t>SM1L15</t>
+          <t>91273A377</t>
         </is>
       </c>
       <c r="H134" t="n">
@@ -7976,14 +7597,14 @@
       </c>
       <c r="L134" t="inlineStr">
         <is>
-          <t>No longer allocated: the cutoff carriage mounts in the SM1RC/M on an integral printed spigot (§8.1); both tubes in hand are spare.</t>
+          <t>No longer allocated: the spring seats in printed cups and the plunger retracts by a thumb tab (§8.5); both screws in hand are spare.</t>
         </is>
       </c>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>UNU-003</t>
+          <t>UNU-005</t>
         </is>
       </c>
       <c r="B135" t="inlineStr">
@@ -7993,12 +7614,12 @@
       </c>
       <c r="D135" t="inlineStr">
         <is>
-          <t>4 mm × 45 mm shoulder screw, 18-8 SS</t>
+          <t>5/16" × 1-1/2" hex-drive flat-head screw, 316 SS</t>
         </is>
       </c>
       <c r="E135" t="inlineStr">
         <is>
-          <t>Existing stock; former spring guide / retract handle</t>
+          <t>Existing alternate/fallback bracket screw stock</t>
         </is>
       </c>
       <c r="F135" t="inlineStr">
@@ -8008,15 +7629,15 @@
       </c>
       <c r="G135" t="inlineStr">
         <is>
-          <t>91273A377</t>
+          <t>90585A587</t>
         </is>
       </c>
       <c r="H135" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="I135" t="inlineStr">
         <is>
-          <t>each</t>
+          <t>pack</t>
         </is>
       </c>
       <c r="J135" t="inlineStr">
@@ -8026,14 +7647,14 @@
       </c>
       <c r="L135" t="inlineStr">
         <is>
-          <t>No longer allocated: the spring seats in printed cups and the plunger retracts by a thumb tab (§8.5); both screws in hand are spare.</t>
+          <t>Previously baseline bracket screw; retained as in-hand alternate stock after corner-clearance review.</t>
         </is>
       </c>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>UNU-005</t>
+          <t>UNU-006</t>
         </is>
       </c>
       <c r="B136" t="inlineStr">
@@ -8043,12 +7664,12 @@
       </c>
       <c r="D136" t="inlineStr">
         <is>
-          <t>5/16" × 1-1/2" hex-drive flat-head screw, 316 SS</t>
+          <t>1/4"-20 × 1-1/2" flat-head screws</t>
         </is>
       </c>
       <c r="E136" t="inlineStr">
         <is>
-          <t>Existing alternate/fallback bracket screw stock</t>
+          <t>Existing spare stock; former C2564 tripod-interface hardware</t>
         </is>
       </c>
       <c r="F136" t="inlineStr">
@@ -8058,15 +7679,15 @@
       </c>
       <c r="G136" t="inlineStr">
         <is>
-          <t>90585A587</t>
+          <t>94518A525</t>
         </is>
       </c>
       <c r="H136" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="I136" t="inlineStr">
         <is>
-          <t>pack</t>
+          <t>each</t>
         </is>
       </c>
       <c r="J136" t="inlineStr">
@@ -8076,14 +7697,14 @@
       </c>
       <c r="L136" t="inlineStr">
         <is>
-          <t>Previously baseline bracket screw; retained as in-hand alternate stock after corner-clearance review.</t>
+          <t>No longer allocated to the active tripod interface after transition to the CAMVATE 577/501/504 quick-release system; retain as in-hand spare hardware.</t>
         </is>
       </c>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>UNU-006</t>
+          <t>UNU-007</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
@@ -8093,7 +7714,7 @@
       </c>
       <c r="D137" t="inlineStr">
         <is>
-          <t>1/4"-20 × 1-1/2" flat-head screws</t>
+          <t>1/4"-20 flex-top locknuts</t>
         </is>
       </c>
       <c r="E137" t="inlineStr">
@@ -8108,15 +7729,15 @@
       </c>
       <c r="G137" t="inlineStr">
         <is>
-          <t>94518A525</t>
+          <t>91839A123</t>
         </is>
       </c>
       <c r="H137" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="I137" t="inlineStr">
         <is>
-          <t>each</t>
+          <t>pack</t>
         </is>
       </c>
       <c r="J137" t="inlineStr">
@@ -8133,7 +7754,7 @@
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>UNU-007</t>
+          <t>UNU-008</t>
         </is>
       </c>
       <c r="B138" t="inlineStr">
@@ -8143,7 +7764,7 @@
       </c>
       <c r="D138" t="inlineStr">
         <is>
-          <t>1/4"-20 flex-top locknuts</t>
+          <t>1/4" thin washers</t>
         </is>
       </c>
       <c r="E138" t="inlineStr">
@@ -8158,11 +7779,11 @@
       </c>
       <c r="G138" t="inlineStr">
         <is>
-          <t>91839A123</t>
+          <t>98019A255</t>
         </is>
       </c>
       <c r="H138" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="I138" t="inlineStr">
         <is>
@@ -8183,7 +7804,7 @@
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>UNU-008</t>
+          <t>UNU-009</t>
         </is>
       </c>
       <c r="B139" t="inlineStr">
@@ -8193,12 +7814,12 @@
       </c>
       <c r="D139" t="inlineStr">
         <is>
-          <t>1/4" thin washers</t>
+          <t>5/16"-18 × 1-3/8" hex-drive flat-head screw, 316 SS</t>
         </is>
       </c>
       <c r="E139" t="inlineStr">
         <is>
-          <t>Existing spare stock; former C2564 tripod-interface hardware</t>
+          <t>Existing alternate bracket screw stock</t>
         </is>
       </c>
       <c r="F139" t="inlineStr">
@@ -8208,11 +7829,11 @@
       </c>
       <c r="G139" t="inlineStr">
         <is>
-          <t>98019A255</t>
+          <t>90585A997</t>
         </is>
       </c>
       <c r="H139" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="I139" t="inlineStr">
         <is>
@@ -8226,14 +7847,14 @@
       </c>
       <c r="L139" t="inlineStr">
         <is>
-          <t>No longer allocated to the active tripod interface after transition to the CAMVATE 577/501/504 quick-release system; retain as in-hand spare hardware.</t>
+          <t>Former baseline bracket screw; retained as in-hand alternate stock after the change to button-head screws (MIR-026).</t>
         </is>
       </c>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>UNU-009</t>
+          <t>UNU-010</t>
         </is>
       </c>
       <c r="B140" t="inlineStr">
@@ -8243,12 +7864,12 @@
       </c>
       <c r="D140" t="inlineStr">
         <is>
-          <t>5/16"-18 × 1-3/8" hex-drive flat-head screw, 316 SS</t>
+          <t>M4 × 0.7 × 16 mm 90° flat-head hex-drive screw, 18-8 stainless</t>
         </is>
       </c>
       <c r="E140" t="inlineStr">
         <is>
-          <t>Existing alternate bracket screw stock</t>
+          <t>Existing spare stock; short-length alternative quick-release plate screw</t>
         </is>
       </c>
       <c r="F140" t="inlineStr">
@@ -8258,11 +7879,11 @@
       </c>
       <c r="G140" t="inlineStr">
         <is>
-          <t>90585A997</t>
+          <t>92125A194</t>
         </is>
       </c>
       <c r="H140" t="n">
-        <v>5</v>
+        <v>100</v>
       </c>
       <c r="I140" t="inlineStr">
         <is>
@@ -8276,14 +7897,14 @@
       </c>
       <c r="L140" t="inlineStr">
         <is>
-          <t>Former baseline bracket screw; retained as in-hand alternate stock after the change to button-head screws (MIR-026).</t>
+          <t>Not allocated: the quick-release plate takes the 18 mm screw (MIR-024); this pack is spare.</t>
         </is>
       </c>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>UNU-010</t>
+          <t>UNU-011</t>
         </is>
       </c>
       <c r="B141" t="inlineStr">
@@ -8293,12 +7914,7 @@
       </c>
       <c r="D141" t="inlineStr">
         <is>
-          <t>M4 × 0.7 × 16 mm 90° flat-head hex-drive screw, 18-8 stainless</t>
-        </is>
-      </c>
-      <c r="E141" t="inlineStr">
-        <is>
-          <t>Existing spare stock; short-length alternative quick-release plate screw</t>
+          <t>Heat-set installation tip</t>
         </is>
       </c>
       <c r="F141" t="inlineStr">
@@ -8308,15 +7924,15 @@
       </c>
       <c r="G141" t="inlineStr">
         <is>
-          <t>92125A194</t>
+          <t>92160A327</t>
         </is>
       </c>
       <c r="H141" t="n">
-        <v>100</v>
+        <v>1</v>
       </c>
       <c r="I141" t="inlineStr">
         <is>
-          <t>pack</t>
+          <t>each</t>
         </is>
       </c>
       <c r="J141" t="inlineStr">
@@ -8326,7 +7942,7 @@
       </c>
       <c r="L141" t="inlineStr">
         <is>
-          <t>Not allocated: the quick-release plate takes the 18 mm screw (MIR-024); this pack is spare.</t>
+          <t>No longer allocated; replaced by the SHP-027 tip set (8915N111), whose adapter is verified on the Hakko iron.</t>
         </is>
       </c>
     </row>
@@ -8361,4 +7977,385 @@
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E29"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="60" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>iPhone Schlieren BOM / Procurement Tracker</t>
+        </is>
+      </c>
+    </row>
+    <row r="2"/>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Canonical workbook</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Generated from bom/bom.csv in Git. Edits made here count only once reconciled into the CSV (reconcile-bom).</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Design baseline</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>docs/design/ fragments in Git (consolidated: schlieren-design).</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Quantity model</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Qty is the numeric required/allocated amount for that BOM line; package counts do not belong in Qty.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Blank Qty</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Quantity is not yet frozen or the item is an as-required consumable/working-stock line.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Package fields</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Package Size is units per Purchase Unit where known. Unknown vendor package sizes are intentionally blank.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Entry count</t>
+        </is>
+      </c>
+      <c r="B8">
+        <f>COUNTA(BOM!A:A)-1</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="1" t="inlineStr">
+        <is>
+          <t>Procurement state</t>
+        </is>
+      </c>
+      <c r="B10" s="1" t="inlineStr">
+        <is>
+          <t>Entries</t>
+        </is>
+      </c>
+      <c r="D10" s="1" t="inlineStr">
+        <is>
+          <t>Subsystem</t>
+        </is>
+      </c>
+      <c r="E10" s="1" t="inlineStr">
+        <is>
+          <t>Entries</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>In hand</t>
+        </is>
+      </c>
+      <c r="B11">
+        <f>COUNTIF(BOM!J:J,"In hand")</f>
+        <v/>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Tabletop frame</t>
+        </is>
+      </c>
+      <c r="E11">
+        <f>COUNTIF(BOM!B:B,D11)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>On order</t>
+        </is>
+      </c>
+      <c r="B12">
+        <f>COUNTIF(BOM!J:J,"On order")</f>
+        <v/>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Optical supports</t>
+        </is>
+      </c>
+      <c r="E12">
+        <f>COUNTIF(BOM!B:B,D12)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>To procure</t>
+        </is>
+      </c>
+      <c r="B13">
+        <f>COUNTIF(BOM!J:J,"To procure")</f>
+        <v/>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Light source</t>
+        </is>
+      </c>
+      <c r="E13">
+        <f>COUNTIF(BOM!B:B,D13)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Specified</t>
+        </is>
+      </c>
+      <c r="B14">
+        <f>COUNTIF(BOM!J:J,"Specified")</f>
+        <v/>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Source slit</t>
+        </is>
+      </c>
+      <c r="E14">
+        <f>COUNTIF(BOM!B:B,D14)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>CAD ready</t>
+        </is>
+      </c>
+      <c r="B15">
+        <f>COUNTIF(BOM!J:J,"CAD ready")</f>
+        <v/>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Carriages</t>
+        </is>
+      </c>
+      <c r="E15">
+        <f>COUNTIF(BOM!B:B,D15)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>CAD open</t>
+        </is>
+      </c>
+      <c r="B16">
+        <f>COUNTIF(BOM!J:J,"CAD open")</f>
+        <v/>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Cassettes</t>
+        </is>
+      </c>
+      <c r="E16">
+        <f>COUNTIF(BOM!B:B,D16)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Imager</t>
+        </is>
+      </c>
+      <c r="E17">
+        <f>COUNTIF(BOM!B:B,D17)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Mirror cell</t>
+        </is>
+      </c>
+      <c r="E18">
+        <f>COUNTIF(BOM!B:B,D18)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Shop supplies</t>
+        </is>
+      </c>
+      <c r="E19">
+        <f>COUNTIF(BOM!B:B,D19)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Unused</t>
+        </is>
+      </c>
+      <c r="E20">
+        <f>COUNTIF(BOM!B:B,D20)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Rollup key</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Use Vendor + SKU for procurement rollups.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Shared parts</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Keep separate BOM rows for separate subsystem allocations; roll them up by Vendor+SKU.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Package math</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Vendor/SKU rollups may sum Qty and divide by Package Size where Package Size is known.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Spare/surplus</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Unavoidable package surplus is not added to required Qty; track it in procurement/inventory rollups or notes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Data rule</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Do not insert subsystem header or separator rows inside the BOM table.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26"/>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Specified</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Part defined by the design; vendor, SKU, or quantity still to be confirmed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>CAD ready</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Printed part with a build123d model in src/schlieren/parts/; ready to print and fit-test.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>CAD open</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Printed part whose custom geometry is still to be designed.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Light source drilling plan updates
</commit_message>
<xml_diff>
--- a/bom/schlieren-bom.xlsx
+++ b/bom/schlieren-bom.xlsx
@@ -7182,7 +7182,7 @@
       </c>
       <c r="D127" t="inlineStr">
         <is>
-          <t>2.0 mm uncoated HSS short-length drill bit, 38 mm overall</t>
+          <t>2mm Premium High Speed Steel Jobber Length Drill, 10 pack</t>
         </is>
       </c>
       <c r="E127" t="inlineStr">
@@ -7192,25 +7192,25 @@
       </c>
       <c r="F127" t="inlineStr">
         <is>
-          <t>McMaster</t>
+          <t>Amazon</t>
         </is>
       </c>
       <c r="G127" t="inlineStr">
         <is>
-          <t>2979N14</t>
+          <t>B07211L28S</t>
         </is>
       </c>
       <c r="H127" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="I127" t="inlineStr">
         <is>
-          <t>each</t>
+          <t>pack</t>
         </is>
       </c>
       <c r="J127" t="inlineStr">
         <is>
-          <t>To procure</t>
+          <t>On order</t>
         </is>
       </c>
       <c r="K127" t="inlineStr">
@@ -7220,7 +7220,7 @@
       </c>
       <c r="L127" t="inlineStr">
         <is>
-          <t>Same series as the 1.6 mm drill SHP-006. Deferred, not in the current order: lead hole size is provisional (§6.4), and the 2.5 mm drill SHP-025 may cut the lead holes instead. Decide after measuring the pigtail insulation.</t>
+          <t>Lead holes (§6.4): the pigtail wire measures about 1.7 mm over its insulation. McMaster alternative if wanted later: 2979N14, 2.0 mm uncoated HSS short-length drill bit, 38 mm overall (same series as the 1.6 mm drill SHP-006).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Doc and terminology/naming revisions
</commit_message>
<xml_diff>
--- a/bom/schlieren-bom.xlsx
+++ b/bom/schlieren-bom.xlsx
@@ -3025,7 +3025,7 @@
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Hard bearing pads under the FAS100 ball tips</t>
+          <t>Flat bearing inserts under the FAS100 ball tips</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
@@ -3730,7 +3730,7 @@
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>Hard bearing pads for FAS100-driven plungers</t>
+          <t>Flat bearing inserts for FAS100-driven plungers</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
@@ -3763,7 +3763,7 @@
       </c>
       <c r="L62" t="inlineStr">
         <is>
-          <t>Nickel-plated rectangular magnets; one hard contact insert for the FAS100-driven PLA plunger of the cutoff carriage.</t>
+          <t>Nickel-plated rectangular magnets; one flat bearing insert for the FAS100-driven PLA plunger of the cutoff carriage.</t>
         </is>
       </c>
     </row>
@@ -4860,7 +4860,7 @@
       </c>
       <c r="L83" t="inlineStr">
         <is>
-          <t>Lens-specific. Two locating walls and a countersunk M5 hole per yoke; two M5 side-slot clamp holes.</t>
+          <t>Lens-specific. Two locating walls and a countersunk M5 hole per yoke; two M5 side-channel clamp holes.</t>
         </is>
       </c>
     </row>
@@ -4885,7 +4885,7 @@
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>Hard bearing pads under three lens-cradle screw tips</t>
+          <t>Flat bearing inserts under three lens-cradle screw tips</t>
         </is>
       </c>
       <c r="F84" t="inlineStr">
@@ -5016,7 +5016,7 @@
       </c>
       <c r="L86" t="inlineStr">
         <is>
-          <t>Two collars for the 37 mm barrel, identical except that the aft collar's left pad pocket seats the groove rods (CAM-010) in place of a magnet.</t>
+          <t>Two collars for the 37 mm barrel, identical except that the aft collar's left pad pocket seats the groove rods (CAM-010) in place of a flat bearing insert.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add LED hole drilling fixture
</commit_message>
<xml_diff>
--- a/bom/schlieren-bom.xlsx
+++ b/bom/schlieren-bom.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Summary" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'BOM'!$A$1:$L$143</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'BOM'!$A$1:$L$151</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -474,7 +474,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L143"/>
+  <dimension ref="A1:L151"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -2705,7 +2705,7 @@
       </c>
       <c r="J42" t="inlineStr">
         <is>
-          <t>On order</t>
+          <t>In hand</t>
         </is>
       </c>
       <c r="K42" t="inlineStr">
@@ -3959,7 +3959,7 @@
       </c>
       <c r="L66" t="inlineStr">
         <is>
-          <t>Also faces the two slit-head blade clamp bars (§7.5).</t>
+          <t>Also faces the two slit-head blade clamp bars (§7.5), and supplies the Ø10 mm hold-down disc under the drilling-fixture plate (§6.8).</t>
         </is>
       </c>
     </row>
@@ -5914,7 +5914,7 @@
       </c>
       <c r="L103" t="inlineStr">
         <is>
-          <t>Eight installed, one under each bracket locknut.</t>
+          <t>Eight installed, one under each bracket locknut. Two more from the pack in SHP-038.</t>
         </is>
       </c>
     </row>
@@ -7276,7 +7276,7 @@
       </c>
       <c r="J128" t="inlineStr">
         <is>
-          <t>On order</t>
+          <t>In hand</t>
         </is>
       </c>
       <c r="K128" t="inlineStr">
@@ -7520,36 +7520,39 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>UNU-001</t>
+          <t>SHP-031</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>Unused</t>
-        </is>
+          <t>Shop supplies</t>
+        </is>
+      </c>
+      <c r="C133" t="n">
+        <v>2</v>
       </c>
       <c r="D133" t="inlineStr">
         <is>
-          <t>Heatsink, 6063-T5 non-anodized aluminum, Ø55 mm x 20 mm.</t>
+          <t>Metric press-fit drill bushing, 1.6 mm ID, 4 mm OD, 6 mm long, chamfer on one end</t>
         </is>
       </c>
       <c r="E133" t="inlineStr">
         <is>
-          <t>Existing spare stock; former LED heatsink</t>
+          <t>M2 tap-drill positions in the drilling fixture plate</t>
         </is>
       </c>
       <c r="F133" t="inlineStr">
         <is>
-          <t>HeatsinkOnline</t>
+          <t>McMaster</t>
         </is>
       </c>
       <c r="G133" t="inlineStr">
         <is>
-          <t>64ASL-8-55</t>
+          <t>96990A132</t>
         </is>
       </c>
       <c r="H133" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="I133" t="inlineStr">
         <is>
@@ -7558,48 +7561,56 @@
       </c>
       <c r="J133" t="inlineStr">
         <is>
-          <t>In hand</t>
+          <t>To procure</t>
+        </is>
+      </c>
+      <c r="K133" t="inlineStr">
+        <is>
+          <t>§6.8</t>
         </is>
       </c>
       <c r="L133" t="inlineStr">
         <is>
-          <t>No longer allocated after the threaded SM1 LED module decision; replaced by LGT-018 (Alpha CN40-40B). Four in hand retained as spares.</t>
+          <t>Hardened steel, headless. Pressed into the printed bushing plate (SHP-034). No spare in the quantity.</t>
         </is>
       </c>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>UNU-002</t>
+          <t>SHP-032</t>
         </is>
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>Unused</t>
-        </is>
+          <t>Shop supplies</t>
+        </is>
+      </c>
+      <c r="C134" t="n">
+        <v>3</v>
       </c>
       <c r="D134" t="inlineStr">
         <is>
-          <t>SM1 lens tube, 1.50" Thread Depth</t>
+          <t>Metric press-fit drill bushing, 2.5 mm ID, 5 mm OD, 6 mm long, chamfer on one end</t>
         </is>
       </c>
       <c r="E134" t="inlineStr">
         <is>
-          <t>Existing stock; former carriage-tube allocation</t>
+          <t>M3 tap-drill positions in the cap, M3 pilot positions in the heatsink</t>
         </is>
       </c>
       <c r="F134" t="inlineStr">
         <is>
-          <t>Thorlabs</t>
+          <t>McMaster</t>
         </is>
       </c>
       <c r="G134" t="inlineStr">
         <is>
-          <t>SM1L15</t>
+          <t>96990A147</t>
         </is>
       </c>
       <c r="H134" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I134" t="inlineStr">
         <is>
@@ -7608,34 +7619,42 @@
       </c>
       <c r="J134" t="inlineStr">
         <is>
-          <t>In hand</t>
+          <t>To procure</t>
+        </is>
+      </c>
+      <c r="K134" t="inlineStr">
+        <is>
+          <t>§6.8</t>
         </is>
       </c>
       <c r="L134" t="inlineStr">
         <is>
-          <t>No longer allocated: the cutoff carriage mounts in the SM1RC/M on an integral printed spigot (§8.1); both tubes in hand are spare.</t>
+          <t>Hardened steel, headless. Pressed into the printed bushing plate (SHP-034). No spare in the quantity.</t>
         </is>
       </c>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>UNU-003</t>
+          <t>SHP-033</t>
         </is>
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>Unused</t>
-        </is>
+          <t>Shop supplies</t>
+        </is>
+      </c>
+      <c r="C135" t="n">
+        <v>2</v>
       </c>
       <c r="D135" t="inlineStr">
         <is>
-          <t>4 mm × 45 mm shoulder screw, 18-8 SS</t>
+          <t>Metric press-fit drill bushing, 2 mm ID, 5 mm OD, 6 mm long, chamfer on one end</t>
         </is>
       </c>
       <c r="E135" t="inlineStr">
         <is>
-          <t>Existing stock; former spring guide / retract handle</t>
+          <t>Lead-hole positions in the cap and the heatsink base</t>
         </is>
       </c>
       <c r="F135" t="inlineStr">
@@ -7645,11 +7664,11 @@
       </c>
       <c r="G135" t="inlineStr">
         <is>
-          <t>91273A377</t>
+          <t>96990A139</t>
         </is>
       </c>
       <c r="H135" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I135" t="inlineStr">
         <is>
@@ -7658,84 +7677,82 @@
       </c>
       <c r="J135" t="inlineStr">
         <is>
-          <t>In hand</t>
+          <t>To procure</t>
+        </is>
+      </c>
+      <c r="K135" t="inlineStr">
+        <is>
+          <t>§6.8</t>
         </is>
       </c>
       <c r="L135" t="inlineStr">
         <is>
-          <t>No longer allocated: the spring seats in printed cups and the plunger retracts by a thumb tab (§8.5); both screws in hand are spare.</t>
+          <t>Hardened steel, headless. Pressed into the printed bushing plate (SHP-034). No spare in the quantity.</t>
         </is>
       </c>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>UNU-005</t>
+          <t>SHP-034</t>
         </is>
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>Unused</t>
-        </is>
+          <t>Shop supplies</t>
+        </is>
+      </c>
+      <c r="C136" t="n">
+        <v>1</v>
       </c>
       <c r="D136" t="inlineStr">
         <is>
-          <t>5/16" × 1-1/2" hex-drive flat-head screw, 316 SS</t>
+          <t>PLA printed LED-module drilling fixture</t>
         </is>
       </c>
       <c r="E136" t="inlineStr">
         <is>
-          <t>Existing alternate/fallback bracket screw stock</t>
-        </is>
-      </c>
-      <c r="F136" t="inlineStr">
-        <is>
-          <t>McMaster</t>
-        </is>
-      </c>
-      <c r="G136" t="inlineStr">
-        <is>
-          <t>90585A587</t>
-        </is>
-      </c>
-      <c r="H136" t="n">
-        <v>5</v>
-      </c>
-      <c r="I136" t="inlineStr">
-        <is>
-          <t>pack</t>
+          <t>Bushing plate, cap nest, and heatsink nest for drilling the SM1CP2M cap and CN40-40B heatsink</t>
         </is>
       </c>
       <c r="J136" t="inlineStr">
         <is>
-          <t>In hand</t>
+          <t>CAD ready</t>
+        </is>
+      </c>
+      <c r="K136" t="inlineStr">
+        <is>
+          <t>§6.8</t>
         </is>
       </c>
       <c r="L136" t="inlineStr">
         <is>
-          <t>Previously baseline bracket screw; retained as in-hand alternate stock after corner-clearance review.</t>
+          <t>Set of three prints, plus a bore coupon to print first (sets the bushing bore size). Fastened with five M3 × 12 mm screws (four plate corners, one cap clamp) from the common 100-pack (SLT-007), into five M3 heat-set inserts (SHP-035) set in the nests.</t>
         </is>
       </c>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>UNU-006</t>
+          <t>SHP-035</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>Unused</t>
-        </is>
+          <t>Shop supplies</t>
+        </is>
+      </c>
+      <c r="C137" t="n">
+        <v>5</v>
       </c>
       <c r="D137" t="inlineStr">
         <is>
-          <t>1/4"-20 × 1-1/2" flat-head screws</t>
+          <t>Brass flanged heat-set threaded inserts for plastic, M3 × 0.5 mm, 5.7 mm installed length</t>
         </is>
       </c>
       <c r="E137" t="inlineStr">
         <is>
-          <t>Existing spare stock; former C2564 tripod-interface hardware</t>
+          <t>Plate screws (4) and cap clamp screw (1) in the drilling fixture nests</t>
         </is>
       </c>
       <c r="F137" t="inlineStr">
@@ -7745,47 +7762,55 @@
       </c>
       <c r="G137" t="inlineStr">
         <is>
-          <t>94518A525</t>
+          <t>97171A310</t>
         </is>
       </c>
       <c r="H137" t="n">
-        <v>4</v>
+        <v>50</v>
       </c>
       <c r="I137" t="inlineStr">
         <is>
-          <t>each</t>
+          <t>pack</t>
         </is>
       </c>
       <c r="J137" t="inlineStr">
         <is>
-          <t>In hand</t>
+          <t>To procure</t>
+        </is>
+      </c>
+      <c r="K137" t="inlineStr">
+        <is>
+          <t>§6.8</t>
         </is>
       </c>
       <c r="L137" t="inlineStr">
         <is>
-          <t>No longer allocated to the active tripod interface after transition to the CAMVATE 577/501/504 quick-release system; retain as in-hand spare hardware.</t>
+          <t>Ø4 mm hole, Ø5.5 mm flange recessed. Set with the M3 tip of the SHP-027 tip set on the Hakko iron (SHP-028); the M3 tip is not yet confirmed to be in the set. Forty-five spare.</t>
         </is>
       </c>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>UNU-007</t>
+          <t>SHP-036</t>
         </is>
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>Unused</t>
-        </is>
+          <t>Shop supplies</t>
+        </is>
+      </c>
+      <c r="C138" t="n">
+        <v>2</v>
       </c>
       <c r="D138" t="inlineStr">
         <is>
-          <t>1/4"-20 flex-top locknuts</t>
+          <t>5/16"-18 × 1-1/4" 18-8 stainless square-neck carriage bolt</t>
         </is>
       </c>
       <c r="E138" t="inlineStr">
         <is>
-          <t>Existing spare stock; former C2564 tripod-interface hardware</t>
+          <t>Drilling fixture mounting: bolts in the drill-press base slots</t>
         </is>
       </c>
       <c r="F138" t="inlineStr">
@@ -7795,11 +7820,11 @@
       </c>
       <c r="G138" t="inlineStr">
         <is>
-          <t>91839A123</t>
+          <t>92356A589</t>
         </is>
       </c>
       <c r="H138" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="I138" t="inlineStr">
         <is>
@@ -7808,34 +7833,42 @@
       </c>
       <c r="J138" t="inlineStr">
         <is>
-          <t>In hand</t>
+          <t>To procure</t>
+        </is>
+      </c>
+      <c r="K138" t="inlineStr">
+        <is>
+          <t>§6.8</t>
         </is>
       </c>
       <c r="L138" t="inlineStr">
         <is>
-          <t>No longer allocated to the active tripod interface after transition to the CAMVATE 577/501/504 quick-release system; retain as in-hand spare hardware.</t>
+          <t>Head under the base, 0.32" square neck in the 3/8" base slot; one per nest ear, two used at a time.</t>
         </is>
       </c>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>UNU-008</t>
+          <t>SHP-037</t>
         </is>
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>Unused</t>
-        </is>
+          <t>Shop supplies</t>
+        </is>
+      </c>
+      <c r="C139" t="n">
+        <v>2</v>
       </c>
       <c r="D139" t="inlineStr">
         <is>
-          <t>1/4" thin washers</t>
+          <t>5/16"-18 18-8 stainless flanged knurled-head thumb nut</t>
         </is>
       </c>
       <c r="E139" t="inlineStr">
         <is>
-          <t>Existing spare stock; former C2564 tripod-interface hardware</t>
+          <t>Drilling fixture mounting: clamp the nest ears from the top</t>
         </is>
       </c>
       <c r="F139" t="inlineStr">
@@ -7845,47 +7878,55 @@
       </c>
       <c r="G139" t="inlineStr">
         <is>
-          <t>98019A255</t>
+          <t>95150A180</t>
         </is>
       </c>
       <c r="H139" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="I139" t="inlineStr">
         <is>
-          <t>pack</t>
+          <t>each</t>
         </is>
       </c>
       <c r="J139" t="inlineStr">
         <is>
-          <t>In hand</t>
+          <t>To procure</t>
+        </is>
+      </c>
+      <c r="K139" t="inlineStr">
+        <is>
+          <t>§6.8</t>
         </is>
       </c>
       <c r="L139" t="inlineStr">
         <is>
-          <t>No longer allocated to the active tripod interface after transition to the CAMVATE 577/501/504 quick-release system; retain as in-hand spare hardware.</t>
+          <t>5/8" knurled head, 17/32" collar on the washer.</t>
         </is>
       </c>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>UNU-009</t>
+          <t>SHP-038</t>
         </is>
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>Unused</t>
-        </is>
+          <t>Shop supplies</t>
+        </is>
+      </c>
+      <c r="C140" t="n">
+        <v>2</v>
       </c>
       <c r="D140" t="inlineStr">
         <is>
-          <t>5/16"-18 × 1-3/8" hex-drive flat-head screw, 316 SS</t>
+          <t>5/16" SAE washer, 0.344" ID × 0.688" OD, 18-8 SS black oxide</t>
         </is>
       </c>
       <c r="E140" t="inlineStr">
         <is>
-          <t>Existing alternate bracket screw stock</t>
+          <t>Drilling fixture mounting: under the thumb nuts on the nest ears</t>
         </is>
       </c>
       <c r="F140" t="inlineStr">
@@ -7895,11 +7936,11 @@
       </c>
       <c r="G140" t="inlineStr">
         <is>
-          <t>90585A997</t>
+          <t>96659A134</t>
         </is>
       </c>
       <c r="H140" t="n">
-        <v>5</v>
+        <v>25</v>
       </c>
       <c r="I140" t="inlineStr">
         <is>
@@ -7911,16 +7952,21 @@
           <t>In hand</t>
         </is>
       </c>
+      <c r="K140" t="inlineStr">
+        <is>
+          <t>§6.8</t>
+        </is>
+      </c>
       <c r="L140" t="inlineStr">
         <is>
-          <t>Former baseline bracket screw; retained as in-hand alternate stock after the change to button-head screws (MIR-026).</t>
+          <t>Shared 25-pack with MIR-013 (eight used there).</t>
         </is>
       </c>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>UNU-010</t>
+          <t>UNU-001</t>
         </is>
       </c>
       <c r="B141" t="inlineStr">
@@ -7930,30 +7976,30 @@
       </c>
       <c r="D141" t="inlineStr">
         <is>
-          <t>M4 × 0.7 × 16 mm 90° flat-head hex-drive screw, 18-8 stainless</t>
+          <t>Heatsink, 6063-T5 non-anodized aluminum, Ø55 mm x 20 mm.</t>
         </is>
       </c>
       <c r="E141" t="inlineStr">
         <is>
-          <t>Existing spare stock; short-length alternative quick-release plate screw</t>
+          <t>Existing spare stock; former LED heatsink</t>
         </is>
       </c>
       <c r="F141" t="inlineStr">
         <is>
-          <t>McMaster</t>
+          <t>HeatsinkOnline</t>
         </is>
       </c>
       <c r="G141" t="inlineStr">
         <is>
-          <t>92125A194</t>
+          <t>64ASL-8-55</t>
         </is>
       </c>
       <c r="H141" t="n">
-        <v>100</v>
+        <v>4</v>
       </c>
       <c r="I141" t="inlineStr">
         <is>
-          <t>pack</t>
+          <t>each</t>
         </is>
       </c>
       <c r="J141" t="inlineStr">
@@ -7963,14 +8009,14 @@
       </c>
       <c r="L141" t="inlineStr">
         <is>
-          <t>Not allocated: the quick-release plate takes the 18 mm screw (MIR-024); this pack is spare.</t>
+          <t>No longer allocated after the threaded SM1 LED module decision; replaced by LGT-018 (Alpha CN40-40B). Four in hand retained as spares.</t>
         </is>
       </c>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>UNU-011</t>
+          <t>UNU-002</t>
         </is>
       </c>
       <c r="B142" t="inlineStr">
@@ -7980,21 +8026,26 @@
       </c>
       <c r="D142" t="inlineStr">
         <is>
-          <t>Heat-set installation tip</t>
+          <t>SM1 lens tube, 1.50" Thread Depth</t>
+        </is>
+      </c>
+      <c r="E142" t="inlineStr">
+        <is>
+          <t>Existing stock; former carriage-tube allocation</t>
         </is>
       </c>
       <c r="F142" t="inlineStr">
         <is>
-          <t>McMaster</t>
+          <t>Thorlabs</t>
         </is>
       </c>
       <c r="G142" t="inlineStr">
         <is>
-          <t>92160A327</t>
+          <t>SM1L15</t>
         </is>
       </c>
       <c r="H142" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I142" t="inlineStr">
         <is>
@@ -8008,63 +8059,458 @@
       </c>
       <c r="L142" t="inlineStr">
         <is>
-          <t>No longer allocated; replaced by the SHP-027 tip set (8915N111), whose adapter is verified on the Hakko iron.</t>
+          <t>No longer allocated: the cutoff carriage mounts in the SM1RC/M on an integral printed spigot (§8.1); both tubes in hand are spare.</t>
         </is>
       </c>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
+          <t>UNU-003</t>
+        </is>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>Unused</t>
+        </is>
+      </c>
+      <c r="D143" t="inlineStr">
+        <is>
+          <t>4 mm × 45 mm shoulder screw, 18-8 SS</t>
+        </is>
+      </c>
+      <c r="E143" t="inlineStr">
+        <is>
+          <t>Existing stock; former spring guide / retract handle</t>
+        </is>
+      </c>
+      <c r="F143" t="inlineStr">
+        <is>
+          <t>McMaster</t>
+        </is>
+      </c>
+      <c r="G143" t="inlineStr">
+        <is>
+          <t>91273A377</t>
+        </is>
+      </c>
+      <c r="H143" t="n">
+        <v>2</v>
+      </c>
+      <c r="I143" t="inlineStr">
+        <is>
+          <t>each</t>
+        </is>
+      </c>
+      <c r="J143" t="inlineStr">
+        <is>
+          <t>In hand</t>
+        </is>
+      </c>
+      <c r="L143" t="inlineStr">
+        <is>
+          <t>No longer allocated: the spring seats in printed cups and the plunger retracts by a thumb tab (§8.5); both screws in hand are spare.</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>UNU-005</t>
+        </is>
+      </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>Unused</t>
+        </is>
+      </c>
+      <c r="D144" t="inlineStr">
+        <is>
+          <t>5/16" × 1-1/2" hex-drive flat-head screw, 316 SS</t>
+        </is>
+      </c>
+      <c r="E144" t="inlineStr">
+        <is>
+          <t>Existing alternate/fallback bracket screw stock</t>
+        </is>
+      </c>
+      <c r="F144" t="inlineStr">
+        <is>
+          <t>McMaster</t>
+        </is>
+      </c>
+      <c r="G144" t="inlineStr">
+        <is>
+          <t>90585A587</t>
+        </is>
+      </c>
+      <c r="H144" t="n">
+        <v>5</v>
+      </c>
+      <c r="I144" t="inlineStr">
+        <is>
+          <t>pack</t>
+        </is>
+      </c>
+      <c r="J144" t="inlineStr">
+        <is>
+          <t>In hand</t>
+        </is>
+      </c>
+      <c r="L144" t="inlineStr">
+        <is>
+          <t>Previously baseline bracket screw; retained as in-hand alternate stock after corner-clearance review.</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>UNU-006</t>
+        </is>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>Unused</t>
+        </is>
+      </c>
+      <c r="D145" t="inlineStr">
+        <is>
+          <t>1/4"-20 × 1-1/2" flat-head screws</t>
+        </is>
+      </c>
+      <c r="E145" t="inlineStr">
+        <is>
+          <t>Existing spare stock; former C2564 tripod-interface hardware</t>
+        </is>
+      </c>
+      <c r="F145" t="inlineStr">
+        <is>
+          <t>McMaster</t>
+        </is>
+      </c>
+      <c r="G145" t="inlineStr">
+        <is>
+          <t>94518A525</t>
+        </is>
+      </c>
+      <c r="H145" t="n">
+        <v>4</v>
+      </c>
+      <c r="I145" t="inlineStr">
+        <is>
+          <t>each</t>
+        </is>
+      </c>
+      <c r="J145" t="inlineStr">
+        <is>
+          <t>In hand</t>
+        </is>
+      </c>
+      <c r="L145" t="inlineStr">
+        <is>
+          <t>No longer allocated to the active tripod interface after transition to the CAMVATE 577/501/504 quick-release system; retain as in-hand spare hardware.</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>UNU-007</t>
+        </is>
+      </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>Unused</t>
+        </is>
+      </c>
+      <c r="D146" t="inlineStr">
+        <is>
+          <t>1/4"-20 flex-top locknuts</t>
+        </is>
+      </c>
+      <c r="E146" t="inlineStr">
+        <is>
+          <t>Existing spare stock; former C2564 tripod-interface hardware</t>
+        </is>
+      </c>
+      <c r="F146" t="inlineStr">
+        <is>
+          <t>McMaster</t>
+        </is>
+      </c>
+      <c r="G146" t="inlineStr">
+        <is>
+          <t>91839A123</t>
+        </is>
+      </c>
+      <c r="H146" t="n">
+        <v>5</v>
+      </c>
+      <c r="I146" t="inlineStr">
+        <is>
+          <t>pack</t>
+        </is>
+      </c>
+      <c r="J146" t="inlineStr">
+        <is>
+          <t>In hand</t>
+        </is>
+      </c>
+      <c r="L146" t="inlineStr">
+        <is>
+          <t>No longer allocated to the active tripod interface after transition to the CAMVATE 577/501/504 quick-release system; retain as in-hand spare hardware.</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>UNU-008</t>
+        </is>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>Unused</t>
+        </is>
+      </c>
+      <c r="D147" t="inlineStr">
+        <is>
+          <t>1/4" thin washers</t>
+        </is>
+      </c>
+      <c r="E147" t="inlineStr">
+        <is>
+          <t>Existing spare stock; former C2564 tripod-interface hardware</t>
+        </is>
+      </c>
+      <c r="F147" t="inlineStr">
+        <is>
+          <t>McMaster</t>
+        </is>
+      </c>
+      <c r="G147" t="inlineStr">
+        <is>
+          <t>98019A255</t>
+        </is>
+      </c>
+      <c r="H147" t="n">
+        <v>10</v>
+      </c>
+      <c r="I147" t="inlineStr">
+        <is>
+          <t>pack</t>
+        </is>
+      </c>
+      <c r="J147" t="inlineStr">
+        <is>
+          <t>In hand</t>
+        </is>
+      </c>
+      <c r="L147" t="inlineStr">
+        <is>
+          <t>No longer allocated to the active tripod interface after transition to the CAMVATE 577/501/504 quick-release system; retain as in-hand spare hardware.</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>UNU-009</t>
+        </is>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>Unused</t>
+        </is>
+      </c>
+      <c r="D148" t="inlineStr">
+        <is>
+          <t>5/16"-18 × 1-3/8" hex-drive flat-head screw, 316 SS</t>
+        </is>
+      </c>
+      <c r="E148" t="inlineStr">
+        <is>
+          <t>Existing alternate bracket screw stock</t>
+        </is>
+      </c>
+      <c r="F148" t="inlineStr">
+        <is>
+          <t>McMaster</t>
+        </is>
+      </c>
+      <c r="G148" t="inlineStr">
+        <is>
+          <t>90585A997</t>
+        </is>
+      </c>
+      <c r="H148" t="n">
+        <v>5</v>
+      </c>
+      <c r="I148" t="inlineStr">
+        <is>
+          <t>pack</t>
+        </is>
+      </c>
+      <c r="J148" t="inlineStr">
+        <is>
+          <t>In hand</t>
+        </is>
+      </c>
+      <c r="L148" t="inlineStr">
+        <is>
+          <t>Former baseline bracket screw; retained as in-hand alternate stock after the change to button-head screws (MIR-026).</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>UNU-010</t>
+        </is>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>Unused</t>
+        </is>
+      </c>
+      <c r="D149" t="inlineStr">
+        <is>
+          <t>M4 × 0.7 × 16 mm 90° flat-head hex-drive screw, 18-8 stainless</t>
+        </is>
+      </c>
+      <c r="E149" t="inlineStr">
+        <is>
+          <t>Existing spare stock; short-length alternative quick-release plate screw</t>
+        </is>
+      </c>
+      <c r="F149" t="inlineStr">
+        <is>
+          <t>McMaster</t>
+        </is>
+      </c>
+      <c r="G149" t="inlineStr">
+        <is>
+          <t>92125A194</t>
+        </is>
+      </c>
+      <c r="H149" t="n">
+        <v>100</v>
+      </c>
+      <c r="I149" t="inlineStr">
+        <is>
+          <t>pack</t>
+        </is>
+      </c>
+      <c r="J149" t="inlineStr">
+        <is>
+          <t>In hand</t>
+        </is>
+      </c>
+      <c r="L149" t="inlineStr">
+        <is>
+          <t>Not allocated: the quick-release plate takes the 18 mm screw (MIR-024); this pack is spare.</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>UNU-011</t>
+        </is>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>Unused</t>
+        </is>
+      </c>
+      <c r="D150" t="inlineStr">
+        <is>
+          <t>Heat-set installation tip</t>
+        </is>
+      </c>
+      <c r="F150" t="inlineStr">
+        <is>
+          <t>McMaster</t>
+        </is>
+      </c>
+      <c r="G150" t="inlineStr">
+        <is>
+          <t>92160A327</t>
+        </is>
+      </c>
+      <c r="H150" t="n">
+        <v>1</v>
+      </c>
+      <c r="I150" t="inlineStr">
+        <is>
+          <t>each</t>
+        </is>
+      </c>
+      <c r="J150" t="inlineStr">
+        <is>
+          <t>In hand</t>
+        </is>
+      </c>
+      <c r="L150" t="inlineStr">
+        <is>
+          <t>No longer allocated; replaced by the SHP-027 tip set (8915N111), whose adapter is verified on the Hakko iron.</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
           <t>UNU-012</t>
         </is>
       </c>
-      <c r="B143" t="inlineStr">
+      <c r="B151" t="inlineStr">
         <is>
           <t>Unused</t>
         </is>
       </c>
-      <c r="D143" t="inlineStr">
+      <c r="D151" t="inlineStr">
         <is>
           <t>M2 × 5 mm button head hex-drive screw 18-8 SS</t>
         </is>
       </c>
-      <c r="E143" t="inlineStr">
+      <c r="E151" t="inlineStr">
         <is>
           <t>Existing spare stock; former LED board mounting screws, tapped into SM1CP2M cap</t>
         </is>
       </c>
-      <c r="F143" t="inlineStr">
+      <c r="F151" t="inlineStr">
         <is>
           <t>McMaster</t>
         </is>
       </c>
-      <c r="G143" t="inlineStr">
+      <c r="G151" t="inlineStr">
         <is>
           <t>92095A452</t>
         </is>
       </c>
-      <c r="H143" t="n">
+      <c r="H151" t="n">
         <v>25</v>
       </c>
-      <c r="I143" t="inlineStr">
+      <c r="I151" t="inlineStr">
         <is>
           <t>pack</t>
         </is>
       </c>
-      <c r="J143" t="inlineStr">
-        <is>
-          <t>In hand</t>
-        </is>
-      </c>
-      <c r="L143" t="inlineStr">
+      <c r="J151" t="inlineStr">
+        <is>
+          <t>In hand</t>
+        </is>
+      </c>
+      <c r="L151" t="inlineStr">
         <is>
           <t>No longer allocated: 5 mm was a bit short; replaced by LGT-020 (92095A453 M2 × 6 mm).</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L143"/>
-  <conditionalFormatting sqref="J2:J143">
+  <autoFilter ref="A1:L151"/>
+  <conditionalFormatting sqref="J2:J151">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"In hand"</formula>
     </cfRule>
@@ -8081,13 +8527,13 @@
       <formula>"CAD open"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A2:L143">
+  <conditionalFormatting sqref="A2:L151">
     <cfRule type="expression" priority="6" dxfId="5">
       <formula>$B2&lt;&gt;$B1</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="J2:J143" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
+    <dataValidation sqref="J2:J151" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
       <formula1>"In hand,On order,To procure,Specified,CAD ready,CAD open"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Adjust heatsink drill cage
</commit_message>
<xml_diff>
--- a/bom/schlieren-bom.xlsx
+++ b/bom/schlieren-bom.xlsx
@@ -7404,7 +7404,7 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>SHP-029</t>
+          <t>SHP-031</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
@@ -7413,16 +7413,16 @@
         </is>
       </c>
       <c r="C131" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D131" t="inlineStr">
         <is>
-          <t>Hole-starting cobalt-steel drill bit, uncoated, 90° point, 1/8" size</t>
+          <t>Metric press-fit drill bushing, 1.6 mm ID, 4 mm OD, 6 mm long, chamfer on one end</t>
         </is>
       </c>
       <c r="E131" t="inlineStr">
         <is>
-          <t>Spot hole locations in the SM1CP2M cap and heatsink base before drilling</t>
+          <t>M2 tap-drill positions in the drilling fixture plate</t>
         </is>
       </c>
       <c r="F131" t="inlineStr">
@@ -7432,7 +7432,7 @@
       </c>
       <c r="G131" t="inlineStr">
         <is>
-          <t>27445A201</t>
+          <t>96990A132</t>
         </is>
       </c>
       <c r="H131" t="n">
@@ -7445,24 +7445,24 @@
       </c>
       <c r="J131" t="inlineStr">
         <is>
-          <t>In hand</t>
+          <t>To procure</t>
         </is>
       </c>
       <c r="K131" t="inlineStr">
         <is>
-          <t>§6.4</t>
+          <t>§6.8</t>
         </is>
       </c>
       <c r="L131" t="inlineStr">
         <is>
-          <t>1/8" shank fits the Dremel 4486 chuck (1/8" maximum). Use before the 1.6, 2.0, 2.5, and 3.3 mm drills.</t>
+          <t>Hardened steel, headless. Pressed into the printed bushing plate (SHP-034). No spare in the quantity.</t>
         </is>
       </c>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>SHP-030</t>
+          <t>SHP-032</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
@@ -7471,16 +7471,16 @@
         </is>
       </c>
       <c r="C132" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D132" t="inlineStr">
         <is>
-          <t>Center drill, high-speed steel, 60° countersink, trade size 1, 1-1/4" overall length</t>
+          <t>Metric press-fit drill bushing, 2.5 mm ID, 5 mm OD, 6 mm long, chamfer on one end</t>
         </is>
       </c>
       <c r="E132" t="inlineStr">
         <is>
-          <t>Backup hole spotter; spots the cap and heatsink holes</t>
+          <t>M3 tap-drill positions in the cap, M3 pilot positions in the heatsink</t>
         </is>
       </c>
       <c r="F132" t="inlineStr">
@@ -7490,7 +7490,7 @@
       </c>
       <c r="G132" t="inlineStr">
         <is>
-          <t>2915A11</t>
+          <t>96990A147</t>
         </is>
       </c>
       <c r="H132" t="n">
@@ -7503,24 +7503,24 @@
       </c>
       <c r="J132" t="inlineStr">
         <is>
-          <t>In hand</t>
+          <t>To procure</t>
         </is>
       </c>
       <c r="K132" t="inlineStr">
         <is>
-          <t>§6.4</t>
+          <t>§6.8</t>
         </is>
       </c>
       <c r="L132" t="inlineStr">
         <is>
-          <t>3/64" pilot, 1/8" body; fits the Dremel 4486 chuck. Spare for SHP-029.</t>
+          <t>Hardened steel, headless. Pressed into the printed bushing plate (SHP-034). No spare in the quantity.</t>
         </is>
       </c>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>SHP-031</t>
+          <t>SHP-033</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
@@ -7533,12 +7533,12 @@
       </c>
       <c r="D133" t="inlineStr">
         <is>
-          <t>Metric press-fit drill bushing, 1.6 mm ID, 4 mm OD, 6 mm long, chamfer on one end</t>
+          <t>Metric press-fit drill bushing, 2 mm ID, 5 mm OD, 6 mm long, chamfer on one end</t>
         </is>
       </c>
       <c r="E133" t="inlineStr">
         <is>
-          <t>M2 tap-drill positions in the drilling fixture plate</t>
+          <t>Lead-hole positions in the cap and the heatsink base</t>
         </is>
       </c>
       <c r="F133" t="inlineStr">
@@ -7548,7 +7548,7 @@
       </c>
       <c r="G133" t="inlineStr">
         <is>
-          <t>96990A132</t>
+          <t>96990A139</t>
         </is>
       </c>
       <c r="H133" t="n">
@@ -7578,7 +7578,7 @@
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>SHP-032</t>
+          <t>SHP-034</t>
         </is>
       </c>
       <c r="B134" t="inlineStr">
@@ -7587,39 +7587,21 @@
         </is>
       </c>
       <c r="C134" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D134" t="inlineStr">
         <is>
-          <t>Metric press-fit drill bushing, 2.5 mm ID, 5 mm OD, 6 mm long, chamfer on one end</t>
+          <t>PLA printed LED-module drilling fixture</t>
         </is>
       </c>
       <c r="E134" t="inlineStr">
         <is>
-          <t>M3 tap-drill positions in the cap, M3 pilot positions in the heatsink</t>
-        </is>
-      </c>
-      <c r="F134" t="inlineStr">
-        <is>
-          <t>McMaster</t>
-        </is>
-      </c>
-      <c r="G134" t="inlineStr">
-        <is>
-          <t>96990A147</t>
-        </is>
-      </c>
-      <c r="H134" t="n">
-        <v>1</v>
-      </c>
-      <c r="I134" t="inlineStr">
-        <is>
-          <t>each</t>
+          <t>Bushing plate, cap nest, and heatsink nest for drilling the SM1CP2M cap and CN40-40B heatsink</t>
         </is>
       </c>
       <c r="J134" t="inlineStr">
         <is>
-          <t>To procure</t>
+          <t>CAD ready</t>
         </is>
       </c>
       <c r="K134" t="inlineStr">
@@ -7629,14 +7611,14 @@
       </c>
       <c r="L134" t="inlineStr">
         <is>
-          <t>Hardened steel, headless. Pressed into the printed bushing plate (SHP-034). No spare in the quantity.</t>
+          <t>Set of three prints, plus a bore coupon to print first (sets the bushing bore size). Fastened with five M3 × 12 mm screws (four plate corners, one cap clamp) from the common 100-pack (SLT-007), into five M3 heat-set inserts (SHP-035) set in the nests.</t>
         </is>
       </c>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>SHP-033</t>
+          <t>SHP-035</t>
         </is>
       </c>
       <c r="B135" t="inlineStr">
@@ -7645,16 +7627,16 @@
         </is>
       </c>
       <c r="C135" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="D135" t="inlineStr">
         <is>
-          <t>Metric press-fit drill bushing, 2 mm ID, 5 mm OD, 6 mm long, chamfer on one end</t>
+          <t>Brass flanged heat-set threaded inserts for plastic, M3 × 0.5 mm, 5.7 mm installed length</t>
         </is>
       </c>
       <c r="E135" t="inlineStr">
         <is>
-          <t>Lead-hole positions in the cap and the heatsink base</t>
+          <t>Plate screws (4) and cap clamp screw (1) in the drilling fixture nests</t>
         </is>
       </c>
       <c r="F135" t="inlineStr">
@@ -7664,15 +7646,15 @@
       </c>
       <c r="G135" t="inlineStr">
         <is>
-          <t>96990A139</t>
+          <t>97171A310</t>
         </is>
       </c>
       <c r="H135" t="n">
-        <v>1</v>
+        <v>50</v>
       </c>
       <c r="I135" t="inlineStr">
         <is>
-          <t>each</t>
+          <t>pack</t>
         </is>
       </c>
       <c r="J135" t="inlineStr">
@@ -7687,14 +7669,14 @@
       </c>
       <c r="L135" t="inlineStr">
         <is>
-          <t>Hardened steel, headless. Pressed into the printed bushing plate (SHP-034). No spare in the quantity.</t>
+          <t>Ø4 mm hole, Ø5.5 mm flange recessed. Set with the M3 tip of the SHP-027 tip set on the Hakko iron (SHP-028); the M3 tip is not yet confirmed to be in the set. Forty-five spare.</t>
         </is>
       </c>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>SHP-034</t>
+          <t>SHP-036</t>
         </is>
       </c>
       <c r="B136" t="inlineStr">
@@ -7703,21 +7685,39 @@
         </is>
       </c>
       <c r="C136" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D136" t="inlineStr">
         <is>
-          <t>PLA printed LED-module drilling fixture</t>
+          <t>5/16"-18 × 1-1/4" 18-8 stainless square-neck carriage bolt</t>
         </is>
       </c>
       <c r="E136" t="inlineStr">
         <is>
-          <t>Bushing plate, cap nest, and heatsink nest for drilling the SM1CP2M cap and CN40-40B heatsink</t>
+          <t>Drilling fixture mounting: bolts in the drill-press base slots</t>
+        </is>
+      </c>
+      <c r="F136" t="inlineStr">
+        <is>
+          <t>McMaster</t>
+        </is>
+      </c>
+      <c r="G136" t="inlineStr">
+        <is>
+          <t>92356A589</t>
+        </is>
+      </c>
+      <c r="H136" t="n">
+        <v>10</v>
+      </c>
+      <c r="I136" t="inlineStr">
+        <is>
+          <t>pack</t>
         </is>
       </c>
       <c r="J136" t="inlineStr">
         <is>
-          <t>CAD ready</t>
+          <t>To procure</t>
         </is>
       </c>
       <c r="K136" t="inlineStr">
@@ -7727,14 +7727,14 @@
       </c>
       <c r="L136" t="inlineStr">
         <is>
-          <t>Set of three prints, plus a bore coupon to print first (sets the bushing bore size). Fastened with five M3 × 12 mm screws (four plate corners, one cap clamp) from the common 100-pack (SLT-007), into five M3 heat-set inserts (SHP-035) set in the nests.</t>
+          <t>Head under the base, 0.32" square neck in the 3/8" base slot; one per nest ear, two used at a time.</t>
         </is>
       </c>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>SHP-035</t>
+          <t>SHP-037</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
@@ -7743,16 +7743,16 @@
         </is>
       </c>
       <c r="C137" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D137" t="inlineStr">
         <is>
-          <t>Brass flanged heat-set threaded inserts for plastic, M3 × 0.5 mm, 5.7 mm installed length</t>
+          <t>5/16"-18 18-8 stainless flanged knurled-head thumb nut</t>
         </is>
       </c>
       <c r="E137" t="inlineStr">
         <is>
-          <t>Plate screws (4) and cap clamp screw (1) in the drilling fixture nests</t>
+          <t>Drilling fixture mounting: clamp the nest ears from the top</t>
         </is>
       </c>
       <c r="F137" t="inlineStr">
@@ -7762,15 +7762,15 @@
       </c>
       <c r="G137" t="inlineStr">
         <is>
-          <t>97171A310</t>
+          <t>95150A180</t>
         </is>
       </c>
       <c r="H137" t="n">
-        <v>50</v>
+        <v>1</v>
       </c>
       <c r="I137" t="inlineStr">
         <is>
-          <t>pack</t>
+          <t>each</t>
         </is>
       </c>
       <c r="J137" t="inlineStr">
@@ -7785,14 +7785,14 @@
       </c>
       <c r="L137" t="inlineStr">
         <is>
-          <t>Ø4 mm hole, Ø5.5 mm flange recessed. Set with the M3 tip of the SHP-027 tip set on the Hakko iron (SHP-028); the M3 tip is not yet confirmed to be in the set. Forty-five spare.</t>
+          <t>5/8" knurled head, 17/32" collar on the washer.</t>
         </is>
       </c>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>SHP-036</t>
+          <t>SHP-038</t>
         </is>
       </c>
       <c r="B138" t="inlineStr">
@@ -7805,12 +7805,12 @@
       </c>
       <c r="D138" t="inlineStr">
         <is>
-          <t>5/16"-18 × 1-1/4" 18-8 stainless square-neck carriage bolt</t>
+          <t>5/16" SAE washer, 0.344" ID × 0.688" OD, 18-8 SS black oxide</t>
         </is>
       </c>
       <c r="E138" t="inlineStr">
         <is>
-          <t>Drilling fixture mounting: bolts in the drill-press base slots</t>
+          <t>Drilling fixture mounting: under the thumb nuts on the nest ears</t>
         </is>
       </c>
       <c r="F138" t="inlineStr">
@@ -7820,11 +7820,11 @@
       </c>
       <c r="G138" t="inlineStr">
         <is>
-          <t>92356A589</t>
+          <t>96659A134</t>
         </is>
       </c>
       <c r="H138" t="n">
-        <v>10</v>
+        <v>25</v>
       </c>
       <c r="I138" t="inlineStr">
         <is>
@@ -7833,7 +7833,7 @@
       </c>
       <c r="J138" t="inlineStr">
         <is>
-          <t>To procure</t>
+          <t>In hand</t>
         </is>
       </c>
       <c r="K138" t="inlineStr">
@@ -7843,46 +7843,43 @@
       </c>
       <c r="L138" t="inlineStr">
         <is>
-          <t>Head under the base, 0.32" square neck in the 3/8" base slot; one per nest ear, two used at a time.</t>
+          <t>Shared 25-pack with MIR-013 (eight used there).</t>
         </is>
       </c>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>SHP-037</t>
+          <t>UNU-001</t>
         </is>
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>Shop supplies</t>
-        </is>
-      </c>
-      <c r="C139" t="n">
-        <v>2</v>
+          <t>Unused</t>
+        </is>
       </c>
       <c r="D139" t="inlineStr">
         <is>
-          <t>5/16"-18 18-8 stainless flanged knurled-head thumb nut</t>
+          <t>Heatsink, 6063-T5 non-anodized aluminum, Ø55 mm x 20 mm.</t>
         </is>
       </c>
       <c r="E139" t="inlineStr">
         <is>
-          <t>Drilling fixture mounting: clamp the nest ears from the top</t>
+          <t>Existing spare stock; former LED heatsink</t>
         </is>
       </c>
       <c r="F139" t="inlineStr">
         <is>
-          <t>McMaster</t>
+          <t>HeatsinkOnline</t>
         </is>
       </c>
       <c r="G139" t="inlineStr">
         <is>
-          <t>95150A180</t>
+          <t>64ASL-8-55</t>
         </is>
       </c>
       <c r="H139" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="I139" t="inlineStr">
         <is>
@@ -7891,60 +7888,52 @@
       </c>
       <c r="J139" t="inlineStr">
         <is>
-          <t>To procure</t>
-        </is>
-      </c>
-      <c r="K139" t="inlineStr">
-        <is>
-          <t>§6.8</t>
+          <t>In hand</t>
         </is>
       </c>
       <c r="L139" t="inlineStr">
         <is>
-          <t>5/8" knurled head, 17/32" collar on the washer.</t>
+          <t>No longer allocated after the threaded SM1 LED module decision; replaced by LGT-018 (Alpha CN40-40B). Four in hand retained as spares.</t>
         </is>
       </c>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>SHP-038</t>
+          <t>UNU-002</t>
         </is>
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>Shop supplies</t>
-        </is>
-      </c>
-      <c r="C140" t="n">
+          <t>Unused</t>
+        </is>
+      </c>
+      <c r="D140" t="inlineStr">
+        <is>
+          <t>SM1 lens tube, 1.50" Thread Depth</t>
+        </is>
+      </c>
+      <c r="E140" t="inlineStr">
+        <is>
+          <t>Existing stock; former carriage-tube allocation</t>
+        </is>
+      </c>
+      <c r="F140" t="inlineStr">
+        <is>
+          <t>Thorlabs</t>
+        </is>
+      </c>
+      <c r="G140" t="inlineStr">
+        <is>
+          <t>SM1L15</t>
+        </is>
+      </c>
+      <c r="H140" t="n">
         <v>2</v>
       </c>
-      <c r="D140" t="inlineStr">
-        <is>
-          <t>5/16" SAE washer, 0.344" ID × 0.688" OD, 18-8 SS black oxide</t>
-        </is>
-      </c>
-      <c r="E140" t="inlineStr">
-        <is>
-          <t>Drilling fixture mounting: under the thumb nuts on the nest ears</t>
-        </is>
-      </c>
-      <c r="F140" t="inlineStr">
-        <is>
-          <t>McMaster</t>
-        </is>
-      </c>
-      <c r="G140" t="inlineStr">
-        <is>
-          <t>96659A134</t>
-        </is>
-      </c>
-      <c r="H140" t="n">
-        <v>25</v>
-      </c>
       <c r="I140" t="inlineStr">
         <is>
-          <t>pack</t>
+          <t>each</t>
         </is>
       </c>
       <c r="J140" t="inlineStr">
@@ -7952,21 +7941,16 @@
           <t>In hand</t>
         </is>
       </c>
-      <c r="K140" t="inlineStr">
-        <is>
-          <t>§6.8</t>
-        </is>
-      </c>
       <c r="L140" t="inlineStr">
         <is>
-          <t>Shared 25-pack with MIR-013 (eight used there).</t>
+          <t>No longer allocated: the cutoff carriage mounts in the SM1RC/M on an integral printed spigot (§8.1); both tubes in hand are spare.</t>
         </is>
       </c>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>UNU-001</t>
+          <t>UNU-003</t>
         </is>
       </c>
       <c r="B141" t="inlineStr">
@@ -7976,26 +7960,26 @@
       </c>
       <c r="D141" t="inlineStr">
         <is>
-          <t>Heatsink, 6063-T5 non-anodized aluminum, Ø55 mm x 20 mm.</t>
+          <t>4 mm × 45 mm shoulder screw, 18-8 SS</t>
         </is>
       </c>
       <c r="E141" t="inlineStr">
         <is>
-          <t>Existing spare stock; former LED heatsink</t>
+          <t>Existing stock; former spring guide / retract handle</t>
         </is>
       </c>
       <c r="F141" t="inlineStr">
         <is>
-          <t>HeatsinkOnline</t>
+          <t>McMaster</t>
         </is>
       </c>
       <c r="G141" t="inlineStr">
         <is>
-          <t>64ASL-8-55</t>
+          <t>91273A377</t>
         </is>
       </c>
       <c r="H141" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="I141" t="inlineStr">
         <is>
@@ -8009,14 +7993,14 @@
       </c>
       <c r="L141" t="inlineStr">
         <is>
-          <t>No longer allocated after the threaded SM1 LED module decision; replaced by LGT-018 (Alpha CN40-40B). Four in hand retained as spares.</t>
+          <t>No longer allocated: the spring seats in printed cups and the plunger retracts by a thumb tab (§8.5); both screws in hand are spare.</t>
         </is>
       </c>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>UNU-002</t>
+          <t>UNU-005</t>
         </is>
       </c>
       <c r="B142" t="inlineStr">
@@ -8026,30 +8010,30 @@
       </c>
       <c r="D142" t="inlineStr">
         <is>
-          <t>SM1 lens tube, 1.50" Thread Depth</t>
+          <t>5/16" × 1-1/2" hex-drive flat-head screw, 316 SS</t>
         </is>
       </c>
       <c r="E142" t="inlineStr">
         <is>
-          <t>Existing stock; former carriage-tube allocation</t>
+          <t>Existing alternate/fallback bracket screw stock</t>
         </is>
       </c>
       <c r="F142" t="inlineStr">
         <is>
-          <t>Thorlabs</t>
+          <t>McMaster</t>
         </is>
       </c>
       <c r="G142" t="inlineStr">
         <is>
-          <t>SM1L15</t>
+          <t>90585A587</t>
         </is>
       </c>
       <c r="H142" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="I142" t="inlineStr">
         <is>
-          <t>each</t>
+          <t>pack</t>
         </is>
       </c>
       <c r="J142" t="inlineStr">
@@ -8059,14 +8043,14 @@
       </c>
       <c r="L142" t="inlineStr">
         <is>
-          <t>No longer allocated: the cutoff carriage mounts in the SM1RC/M on an integral printed spigot (§8.1); both tubes in hand are spare.</t>
+          <t>Previously baseline bracket screw; retained as in-hand alternate stock after corner-clearance review.</t>
         </is>
       </c>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>UNU-003</t>
+          <t>UNU-006</t>
         </is>
       </c>
       <c r="B143" t="inlineStr">
@@ -8076,12 +8060,12 @@
       </c>
       <c r="D143" t="inlineStr">
         <is>
-          <t>4 mm × 45 mm shoulder screw, 18-8 SS</t>
+          <t>1/4"-20 × 1-1/2" flat-head screws</t>
         </is>
       </c>
       <c r="E143" t="inlineStr">
         <is>
-          <t>Existing stock; former spring guide / retract handle</t>
+          <t>Existing spare stock; former C2564 tripod-interface hardware</t>
         </is>
       </c>
       <c r="F143" t="inlineStr">
@@ -8091,11 +8075,11 @@
       </c>
       <c r="G143" t="inlineStr">
         <is>
-          <t>91273A377</t>
+          <t>94518A525</t>
         </is>
       </c>
       <c r="H143" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="I143" t="inlineStr">
         <is>
@@ -8109,14 +8093,14 @@
       </c>
       <c r="L143" t="inlineStr">
         <is>
-          <t>No longer allocated: the spring seats in printed cups and the plunger retracts by a thumb tab (§8.5); both screws in hand are spare.</t>
+          <t>No longer allocated to the active tripod interface after transition to the CAMVATE 577/501/504 quick-release system; retain as in-hand spare hardware.</t>
         </is>
       </c>
     </row>
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>UNU-005</t>
+          <t>UNU-007</t>
         </is>
       </c>
       <c r="B144" t="inlineStr">
@@ -8126,12 +8110,12 @@
       </c>
       <c r="D144" t="inlineStr">
         <is>
-          <t>5/16" × 1-1/2" hex-drive flat-head screw, 316 SS</t>
+          <t>1/4"-20 flex-top locknuts</t>
         </is>
       </c>
       <c r="E144" t="inlineStr">
         <is>
-          <t>Existing alternate/fallback bracket screw stock</t>
+          <t>Existing spare stock; former C2564 tripod-interface hardware</t>
         </is>
       </c>
       <c r="F144" t="inlineStr">
@@ -8141,7 +8125,7 @@
       </c>
       <c r="G144" t="inlineStr">
         <is>
-          <t>90585A587</t>
+          <t>91839A123</t>
         </is>
       </c>
       <c r="H144" t="n">
@@ -8159,14 +8143,14 @@
       </c>
       <c r="L144" t="inlineStr">
         <is>
-          <t>Previously baseline bracket screw; retained as in-hand alternate stock after corner-clearance review.</t>
+          <t>No longer allocated to the active tripod interface after transition to the CAMVATE 577/501/504 quick-release system; retain as in-hand spare hardware.</t>
         </is>
       </c>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>UNU-006</t>
+          <t>UNU-008</t>
         </is>
       </c>
       <c r="B145" t="inlineStr">
@@ -8176,7 +8160,7 @@
       </c>
       <c r="D145" t="inlineStr">
         <is>
-          <t>1/4"-20 × 1-1/2" flat-head screws</t>
+          <t>1/4" thin washers</t>
         </is>
       </c>
       <c r="E145" t="inlineStr">
@@ -8191,15 +8175,15 @@
       </c>
       <c r="G145" t="inlineStr">
         <is>
-          <t>94518A525</t>
+          <t>98019A255</t>
         </is>
       </c>
       <c r="H145" t="n">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="I145" t="inlineStr">
         <is>
-          <t>each</t>
+          <t>pack</t>
         </is>
       </c>
       <c r="J145" t="inlineStr">
@@ -8216,7 +8200,7 @@
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>UNU-007</t>
+          <t>UNU-009</t>
         </is>
       </c>
       <c r="B146" t="inlineStr">
@@ -8226,12 +8210,12 @@
       </c>
       <c r="D146" t="inlineStr">
         <is>
-          <t>1/4"-20 flex-top locknuts</t>
+          <t>5/16"-18 × 1-3/8" hex-drive flat-head screw, 316 SS</t>
         </is>
       </c>
       <c r="E146" t="inlineStr">
         <is>
-          <t>Existing spare stock; former C2564 tripod-interface hardware</t>
+          <t>Existing alternate bracket screw stock</t>
         </is>
       </c>
       <c r="F146" t="inlineStr">
@@ -8241,7 +8225,7 @@
       </c>
       <c r="G146" t="inlineStr">
         <is>
-          <t>91839A123</t>
+          <t>90585A997</t>
         </is>
       </c>
       <c r="H146" t="n">
@@ -8259,14 +8243,14 @@
       </c>
       <c r="L146" t="inlineStr">
         <is>
-          <t>No longer allocated to the active tripod interface after transition to the CAMVATE 577/501/504 quick-release system; retain as in-hand spare hardware.</t>
+          <t>Former baseline bracket screw; retained as in-hand alternate stock after the change to button-head screws (MIR-026).</t>
         </is>
       </c>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>UNU-008</t>
+          <t>UNU-010</t>
         </is>
       </c>
       <c r="B147" t="inlineStr">
@@ -8276,12 +8260,12 @@
       </c>
       <c r="D147" t="inlineStr">
         <is>
-          <t>1/4" thin washers</t>
+          <t>M4 × 0.7 × 16 mm 90° flat-head hex-drive screw, 18-8 stainless</t>
         </is>
       </c>
       <c r="E147" t="inlineStr">
         <is>
-          <t>Existing spare stock; former C2564 tripod-interface hardware</t>
+          <t>Existing spare stock; short-length alternative quick-release plate screw</t>
         </is>
       </c>
       <c r="F147" t="inlineStr">
@@ -8291,11 +8275,11 @@
       </c>
       <c r="G147" t="inlineStr">
         <is>
-          <t>98019A255</t>
+          <t>92125A194</t>
         </is>
       </c>
       <c r="H147" t="n">
-        <v>10</v>
+        <v>100</v>
       </c>
       <c r="I147" t="inlineStr">
         <is>
@@ -8309,14 +8293,14 @@
       </c>
       <c r="L147" t="inlineStr">
         <is>
-          <t>No longer allocated to the active tripod interface after transition to the CAMVATE 577/501/504 quick-release system; retain as in-hand spare hardware.</t>
+          <t>Not allocated: the quick-release plate takes the 18 mm screw (MIR-024); this pack is spare.</t>
         </is>
       </c>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>UNU-009</t>
+          <t>UNU-011</t>
         </is>
       </c>
       <c r="B148" t="inlineStr">
@@ -8326,12 +8310,7 @@
       </c>
       <c r="D148" t="inlineStr">
         <is>
-          <t>5/16"-18 × 1-3/8" hex-drive flat-head screw, 316 SS</t>
-        </is>
-      </c>
-      <c r="E148" t="inlineStr">
-        <is>
-          <t>Existing alternate bracket screw stock</t>
+          <t>Heat-set installation tip</t>
         </is>
       </c>
       <c r="F148" t="inlineStr">
@@ -8341,15 +8320,15 @@
       </c>
       <c r="G148" t="inlineStr">
         <is>
-          <t>90585A997</t>
+          <t>92160A327</t>
         </is>
       </c>
       <c r="H148" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="I148" t="inlineStr">
         <is>
-          <t>pack</t>
+          <t>each</t>
         </is>
       </c>
       <c r="J148" t="inlineStr">
@@ -8359,14 +8338,14 @@
       </c>
       <c r="L148" t="inlineStr">
         <is>
-          <t>Former baseline bracket screw; retained as in-hand alternate stock after the change to button-head screws (MIR-026).</t>
+          <t>No longer allocated; replaced by the SHP-027 tip set (8915N111), whose adapter is verified on the Hakko iron.</t>
         </is>
       </c>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>UNU-010</t>
+          <t>UNU-012</t>
         </is>
       </c>
       <c r="B149" t="inlineStr">
@@ -8376,12 +8355,12 @@
       </c>
       <c r="D149" t="inlineStr">
         <is>
-          <t>M4 × 0.7 × 16 mm 90° flat-head hex-drive screw, 18-8 stainless</t>
+          <t>M2 × 5 mm button head hex-drive screw 18-8 SS</t>
         </is>
       </c>
       <c r="E149" t="inlineStr">
         <is>
-          <t>Existing spare stock; short-length alternative quick-release plate screw</t>
+          <t>Existing spare stock; former LED board mounting screws, tapped into SM1CP2M cap</t>
         </is>
       </c>
       <c r="F149" t="inlineStr">
@@ -8391,11 +8370,11 @@
       </c>
       <c r="G149" t="inlineStr">
         <is>
-          <t>92125A194</t>
+          <t>92095A452</t>
         </is>
       </c>
       <c r="H149" t="n">
-        <v>100</v>
+        <v>25</v>
       </c>
       <c r="I149" t="inlineStr">
         <is>
@@ -8409,14 +8388,14 @@
       </c>
       <c r="L149" t="inlineStr">
         <is>
-          <t>Not allocated: the quick-release plate takes the 18 mm screw (MIR-024); this pack is spare.</t>
+          <t>No longer allocated: 5 mm was a bit short; replaced by LGT-020 (92095A453 M2 × 6 mm).</t>
         </is>
       </c>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>UNU-011</t>
+          <t>UNU-013</t>
         </is>
       </c>
       <c r="B150" t="inlineStr">
@@ -8426,7 +8405,12 @@
       </c>
       <c r="D150" t="inlineStr">
         <is>
-          <t>Heat-set installation tip</t>
+          <t>Hole-starting cobalt-steel drill bit, uncoated, 90° point, 1/8" size</t>
+        </is>
+      </c>
+      <c r="E150" t="inlineStr">
+        <is>
+          <t>Existing spare stock; former hole spotter</t>
         </is>
       </c>
       <c r="F150" t="inlineStr">
@@ -8436,7 +8420,7 @@
       </c>
       <c r="G150" t="inlineStr">
         <is>
-          <t>92160A327</t>
+          <t>27445A201</t>
         </is>
       </c>
       <c r="H150" t="n">
@@ -8450,18 +8434,13 @@
       <c r="J150" t="inlineStr">
         <is>
           <t>In hand</t>
-        </is>
-      </c>
-      <c r="L150" t="inlineStr">
-        <is>
-          <t>No longer allocated; replaced by the SHP-027 tip set (8915N111), whose adapter is verified on the Hakko iron.</t>
         </is>
       </c>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>UNU-012</t>
+          <t>UNU-014</t>
         </is>
       </c>
       <c r="B151" t="inlineStr">
@@ -8471,12 +8450,12 @@
       </c>
       <c r="D151" t="inlineStr">
         <is>
-          <t>M2 × 5 mm button head hex-drive screw 18-8 SS</t>
+          <t>Center drill, high-speed steel, 60° countersink, trade size 1, 1-1/4" overall length</t>
         </is>
       </c>
       <c r="E151" t="inlineStr">
         <is>
-          <t>Existing spare stock; former LED board mounting screws, tapped into SM1CP2M cap</t>
+          <t>Existing spare stock; former hole spotter</t>
         </is>
       </c>
       <c r="F151" t="inlineStr">
@@ -8486,25 +8465,20 @@
       </c>
       <c r="G151" t="inlineStr">
         <is>
-          <t>92095A452</t>
+          <t>2915A11</t>
         </is>
       </c>
       <c r="H151" t="n">
-        <v>25</v>
+        <v>1</v>
       </c>
       <c r="I151" t="inlineStr">
         <is>
-          <t>pack</t>
+          <t>each</t>
         </is>
       </c>
       <c r="J151" t="inlineStr">
         <is>
           <t>In hand</t>
-        </is>
-      </c>
-      <c r="L151" t="inlineStr">
-        <is>
-          <t>No longer allocated: 5 mm was a bit short; replaced by LGT-020 (92095A453 M2 × 6 mm).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Adjust drill fixture bores after test fits with coupon
</commit_message>
<xml_diff>
--- a/bom/schlieren-bom.xlsx
+++ b/bom/schlieren-bom.xlsx
@@ -7445,7 +7445,7 @@
       </c>
       <c r="J131" t="inlineStr">
         <is>
-          <t>To procure</t>
+          <t>In hand</t>
         </is>
       </c>
       <c r="K131" t="inlineStr">
@@ -7503,7 +7503,7 @@
       </c>
       <c r="J132" t="inlineStr">
         <is>
-          <t>To procure</t>
+          <t>In hand</t>
         </is>
       </c>
       <c r="K132" t="inlineStr">
@@ -7561,7 +7561,7 @@
       </c>
       <c r="J133" t="inlineStr">
         <is>
-          <t>To procure</t>
+          <t>In hand</t>
         </is>
       </c>
       <c r="K133" t="inlineStr">
@@ -7659,7 +7659,7 @@
       </c>
       <c r="J135" t="inlineStr">
         <is>
-          <t>To procure</t>
+          <t>In hand</t>
         </is>
       </c>
       <c r="K135" t="inlineStr">
@@ -7669,7 +7669,7 @@
       </c>
       <c r="L135" t="inlineStr">
         <is>
-          <t>Ø4 mm hole, Ø5.5 mm flange recessed. Set with the M3 tip of the SHP-027 tip set on the Hakko iron (SHP-028); the M3 tip is not yet confirmed to be in the set. Forty-five spare.</t>
+          <t>Ø4 mm hole, Ø5.5 mm flange recessed. Set with the M3 tip of the SHP-027 tip set on the Hakko iron (SHP-028). Forty-five spare.</t>
         </is>
       </c>
     </row>
@@ -7717,7 +7717,7 @@
       </c>
       <c r="J136" t="inlineStr">
         <is>
-          <t>To procure</t>
+          <t>In hand</t>
         </is>
       </c>
       <c r="K136" t="inlineStr">
@@ -7775,7 +7775,7 @@
       </c>
       <c r="J137" t="inlineStr">
         <is>
-          <t>To procure</t>
+          <t>On order</t>
         </is>
       </c>
       <c r="K137" t="inlineStr">

</xml_diff>